<commit_message>
Muestra de tarjeta semanal completa (S26) y % ≥12 °Brix calculado de la distribución
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016MoDN2MbHCPujrwTZ2bJdV
</commit_message>
<xml_diff>
--- a/Datos de azucar y firmeza por melon en general.xlsx
+++ b/Datos de azucar y firmeza por melon en general.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>% &gt; 12 °Brix</t>
+          <t>% ≥ 12 °Brix</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -619,7 +619,7 @@
         <v>7407</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>0.6985</v>
+        <v>0.8304</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>3509</v>
@@ -663,7 +663,7 @@
         <v>95</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.6947</v>
+        <v>0.6943</v>
       </c>
       <c r="K3" s="5" t="n">
         <v>45</v>
@@ -711,7 +711,7 @@
         <v>95</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>0.6947</v>
+        <v>0.6943</v>
       </c>
       <c r="K4" s="8" t="n">
         <v>45</v>
@@ -755,7 +755,7 @@
         <v>165</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.3999</v>
+        <v>0.6906</v>
       </c>
       <c r="K5" s="5" t="n">
         <v>80</v>
@@ -851,7 +851,7 @@
         <v>35</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.3714</v>
+        <v>0.3999</v>
       </c>
       <c r="K7" s="8" t="n">
         <v>15</v>
@@ -899,7 +899,7 @@
         <v>10</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="K8" s="8" t="n">
         <v>5</v>
@@ -947,7 +947,7 @@
         <v>110</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>0.4181</v>
+        <v>0.8087</v>
       </c>
       <c r="K9" s="8" t="n">
         <v>55</v>
@@ -991,7 +991,7 @@
         <v>664</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>0.8488</v>
+        <v>0.8431</v>
       </c>
       <c r="K10" s="5" t="n">
         <v>319</v>
@@ -1183,7 +1183,7 @@
         <v>99</v>
       </c>
       <c r="J14" s="11" t="n">
-        <v>0.9272</v>
+        <v>0.8989</v>
       </c>
       <c r="K14" s="8" t="n">
         <v>54</v>
@@ -1327,7 +1327,7 @@
         <v>142</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>0.7586000000000001</v>
+        <v>0.753</v>
       </c>
       <c r="K17" s="8" t="n">
         <v>65</v>
@@ -1423,7 +1423,7 @@
         <v>70</v>
       </c>
       <c r="J19" s="11" t="n">
-        <v>0.9428</v>
+        <v>0.9425</v>
       </c>
       <c r="K19" s="8" t="n">
         <v>35</v>
@@ -1471,7 +1471,7 @@
         <v>118</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9486</v>
       </c>
       <c r="K20" s="8" t="n">
         <v>60</v>
@@ -1519,7 +1519,7 @@
         <v>70</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>0.9571</v>
+        <v>0.9567</v>
       </c>
       <c r="K21" s="8" t="n">
         <v>35</v>
@@ -1563,7 +1563,7 @@
         <v>1290</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>0.5151</v>
+        <v>0.7485000000000001</v>
       </c>
       <c r="K22" s="5" t="n">
         <v>580</v>
@@ -1611,7 +1611,7 @@
         <v>140</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>0.7357</v>
+        <v>0.7138</v>
       </c>
       <c r="K23" s="8" t="n">
         <v>65</v>
@@ -1659,7 +1659,7 @@
         <v>10</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K24" s="8" t="n">
         <v>5</v>
@@ -1707,7 +1707,7 @@
         <v>100</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>0.8</v>
+        <v>0.96</v>
       </c>
       <c r="K25" s="8" t="n">
         <v>45</v>
@@ -1755,7 +1755,7 @@
         <v>90</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>0.7111</v>
+        <v>0.7108</v>
       </c>
       <c r="K26" s="8" t="n">
         <v>40</v>
@@ -1803,7 +1803,7 @@
         <v>150</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>0.9066</v>
+        <v>0.9462</v>
       </c>
       <c r="K27" s="8" t="n">
         <v>75</v>
@@ -1851,7 +1851,7 @@
         <v>10</v>
       </c>
       <c r="J28" s="11" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K28" s="8" t="n">
         <v>5</v>
@@ -1899,7 +1899,7 @@
         <v>20</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29" s="8" t="n">
         <v>10</v>
@@ -1995,7 +1995,7 @@
         <v>140</v>
       </c>
       <c r="J31" s="11" t="n">
-        <v>0.9</v>
+        <v>0.8995</v>
       </c>
       <c r="K31" s="8" t="n">
         <v>70</v>
@@ -2091,7 +2091,7 @@
         <v>101</v>
       </c>
       <c r="J33" s="11" t="n">
-        <v>0.29</v>
+        <v>0.9207</v>
       </c>
       <c r="K33" s="8" t="n">
         <v>50</v>
@@ -2139,7 +2139,7 @@
         <v>10</v>
       </c>
       <c r="J34" s="11" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K34" s="8" t="n">
         <v>5</v>
@@ -2187,7 +2187,7 @@
         <v>292</v>
       </c>
       <c r="J35" s="11" t="n">
-        <v>0.3071</v>
+        <v>0.6261</v>
       </c>
       <c r="K35" s="8" t="n">
         <v>115</v>
@@ -2235,7 +2235,7 @@
         <v>50</v>
       </c>
       <c r="J36" s="11" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="K36" s="8" t="n">
         <v>15</v>
@@ -2283,7 +2283,7 @@
         <v>157</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>0.1375</v>
+        <v>0.643</v>
       </c>
       <c r="K37" s="8" t="n">
         <v>70</v>
@@ -2327,7 +2327,7 @@
         <v>401</v>
       </c>
       <c r="J38" s="7" t="n">
-        <v>0.9002</v>
+        <v>0.8997000000000001</v>
       </c>
       <c r="K38" s="5" t="n">
         <v>194</v>
@@ -2375,7 +2375,7 @@
         <v>180</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>0.9888</v>
+        <v>0.9826</v>
       </c>
       <c r="K39" s="8" t="n">
         <v>90</v>
@@ -2471,7 +2471,7 @@
         <v>211</v>
       </c>
       <c r="J41" s="11" t="n">
-        <v>0.8199</v>
+        <v>0.8242</v>
       </c>
       <c r="K41" s="8" t="n">
         <v>100</v>
@@ -2515,7 +2515,7 @@
         <v>543</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>0.9391</v>
+        <v>0.9371</v>
       </c>
       <c r="K42" s="5" t="n">
         <v>264</v>
@@ -2563,7 +2563,7 @@
         <v>112</v>
       </c>
       <c r="J43" s="11" t="n">
-        <v>1</v>
+        <v>0.9997</v>
       </c>
       <c r="K43" s="8" t="n">
         <v>55</v>
@@ -2611,7 +2611,7 @@
         <v>30</v>
       </c>
       <c r="J44" s="11" t="n">
-        <v>0.9</v>
+        <v>0.8999</v>
       </c>
       <c r="K44" s="8" t="n">
         <v>15</v>
@@ -2659,7 +2659,7 @@
         <v>60</v>
       </c>
       <c r="J45" s="11" t="n">
-        <v>0.8833</v>
+        <v>0.8831</v>
       </c>
       <c r="K45" s="8" t="n">
         <v>30</v>
@@ -2707,7 +2707,7 @@
         <v>141</v>
       </c>
       <c r="J46" s="11" t="n">
-        <v>0.9214</v>
+        <v>0.9142</v>
       </c>
       <c r="K46" s="8" t="n">
         <v>69</v>
@@ -2803,7 +2803,7 @@
         <v>30</v>
       </c>
       <c r="J48" s="11" t="n">
-        <v>1</v>
+        <v>0.9998</v>
       </c>
       <c r="K48" s="8" t="n">
         <v>15</v>
@@ -2851,7 +2851,7 @@
         <v>30</v>
       </c>
       <c r="J49" s="11" t="n">
-        <v>0.8333</v>
+        <v>0.8331</v>
       </c>
       <c r="K49" s="8" t="n">
         <v>10</v>
@@ -2991,7 +2991,7 @@
         <v>452</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>0.6704</v>
+        <v>0.6788</v>
       </c>
       <c r="K52" s="5" t="n">
         <v>214</v>
@@ -3039,7 +3039,7 @@
         <v>40</v>
       </c>
       <c r="J53" s="11" t="n">
-        <v>0.5</v>
+        <v>0.475</v>
       </c>
       <c r="K53" s="8" t="n">
         <v>20</v>
@@ -3087,7 +3087,7 @@
         <v>101</v>
       </c>
       <c r="J54" s="11" t="n">
-        <v>0.6</v>
+        <v>0.6039</v>
       </c>
       <c r="K54" s="8" t="n">
         <v>45</v>
@@ -3231,7 +3231,7 @@
         <v>130</v>
       </c>
       <c r="J57" s="11" t="n">
-        <v>0.6846</v>
+        <v>0.6993</v>
       </c>
       <c r="K57" s="8" t="n">
         <v>59</v>
@@ -3279,7 +3279,7 @@
         <v>161</v>
       </c>
       <c r="J58" s="11" t="n">
-        <v>0.7046</v>
+        <v>0.7201</v>
       </c>
       <c r="K58" s="8" t="n">
         <v>80</v>
@@ -3323,7 +3323,7 @@
         <v>866</v>
       </c>
       <c r="J59" s="7" t="n">
-        <v>0.8578</v>
+        <v>0.8793</v>
       </c>
       <c r="K59" s="5" t="n">
         <v>400</v>
@@ -3419,7 +3419,7 @@
         <v>30</v>
       </c>
       <c r="J61" s="11" t="n">
-        <v>0.7665999999999999</v>
+        <v>0.7664</v>
       </c>
       <c r="K61" s="8" t="n">
         <v>15</v>
@@ -3611,7 +3611,7 @@
         <v>137</v>
       </c>
       <c r="J65" s="11" t="n">
-        <v>0.6115</v>
+        <v>0.5976</v>
       </c>
       <c r="K65" s="8" t="n">
         <v>35</v>
@@ -3707,7 +3707,7 @@
         <v>70</v>
       </c>
       <c r="J67" s="11" t="n">
-        <v>0.9428</v>
+        <v>0.9424</v>
       </c>
       <c r="K67" s="8" t="n">
         <v>35</v>
@@ -3755,7 +3755,7 @@
         <v>139</v>
       </c>
       <c r="J68" s="11" t="n">
-        <v>0.9</v>
+        <v>0.9272</v>
       </c>
       <c r="K68" s="8" t="n">
         <v>65</v>
@@ -3803,7 +3803,7 @@
         <v>390</v>
       </c>
       <c r="J69" s="11" t="n">
-        <v>0.9102</v>
+        <v>0.9532</v>
       </c>
       <c r="K69" s="8" t="n">
         <v>195</v>
@@ -3847,7 +3847,7 @@
         <v>1000</v>
       </c>
       <c r="J70" s="7" t="n">
-        <v>0.475</v>
+        <v>0.7796999999999999</v>
       </c>
       <c r="K70" s="5" t="n">
         <v>460</v>
@@ -3943,7 +3943,7 @@
         <v>189</v>
       </c>
       <c r="J72" s="11" t="n">
-        <v>0.19</v>
+        <v>0.9201</v>
       </c>
       <c r="K72" s="8" t="n">
         <v>95</v>
@@ -3991,7 +3991,7 @@
         <v>30</v>
       </c>
       <c r="J73" s="11" t="n">
-        <v>0.6333</v>
+        <v>0.6331</v>
       </c>
       <c r="K73" s="8" t="n">
         <v>15</v>
@@ -4039,7 +4039,7 @@
         <v>130</v>
       </c>
       <c r="J74" s="11" t="n">
-        <v>0.8307</v>
+        <v>0.8223</v>
       </c>
       <c r="K74" s="8" t="n">
         <v>65</v>
@@ -4327,7 +4327,7 @@
         <v>60</v>
       </c>
       <c r="J80" s="11" t="n">
-        <v>0.3166</v>
+        <v>0.9829</v>
       </c>
       <c r="K80" s="8" t="n">
         <v>25</v>
@@ -4423,7 +4423,7 @@
         <v>10</v>
       </c>
       <c r="J82" s="11" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K82" s="8" t="n">
         <v>5</v>
@@ -4519,7 +4519,7 @@
         <v>40</v>
       </c>
       <c r="J84" s="11" t="n">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="K84" s="8" t="n">
         <v>20</v>
@@ -4567,7 +4567,7 @@
         <v>71</v>
       </c>
       <c r="J85" s="11" t="n">
-        <v>0.1142</v>
+        <v>0.7461</v>
       </c>
       <c r="K85" s="8" t="n">
         <v>35</v>
@@ -4615,7 +4615,7 @@
         <v>130</v>
       </c>
       <c r="J86" s="11" t="n">
-        <v>0.0387</v>
+        <v>0.1842</v>
       </c>
       <c r="K86" s="8" t="n">
         <v>30</v>
@@ -4663,7 +4663,7 @@
         <v>50</v>
       </c>
       <c r="J87" s="11" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.96</v>
       </c>
       <c r="K87" s="8" t="n">
         <v>25</v>
@@ -4755,7 +4755,7 @@
         <v>1000</v>
       </c>
       <c r="J89" s="7" t="n">
-        <v>0.6364</v>
+        <v>0.9386</v>
       </c>
       <c r="K89" s="5" t="n">
         <v>509</v>
@@ -4803,7 +4803,7 @@
         <v>109</v>
       </c>
       <c r="J90" s="11" t="n">
-        <v>0.8909</v>
+        <v>0.8894</v>
       </c>
       <c r="K90" s="8" t="n">
         <v>54</v>
@@ -4851,7 +4851,7 @@
         <v>150</v>
       </c>
       <c r="J91" s="11" t="n">
-        <v>0.3687</v>
+        <v>0.9796</v>
       </c>
       <c r="K91" s="8" t="n">
         <v>75</v>
@@ -4947,7 +4947,7 @@
         <v>299</v>
       </c>
       <c r="J93" s="11" t="n">
-        <v>0.8714</v>
+        <v>0.9425</v>
       </c>
       <c r="K93" s="8" t="n">
         <v>155</v>
@@ -4995,7 +4995,7 @@
         <v>261</v>
       </c>
       <c r="J94" s="11" t="n">
-        <v>0.45</v>
+        <v>0.9804</v>
       </c>
       <c r="K94" s="8" t="n">
         <v>130</v>
@@ -5139,7 +5139,7 @@
         <v>21</v>
       </c>
       <c r="J97" s="11" t="n">
-        <v>0</v>
+        <v>0.8092</v>
       </c>
       <c r="K97" s="8" t="n">
         <v>10</v>
@@ -5187,7 +5187,7 @@
         <v>100</v>
       </c>
       <c r="J98" s="11" t="n">
-        <v>0.57</v>
+        <v>0.91</v>
       </c>
       <c r="K98" s="8" t="n">
         <v>55</v>
@@ -5231,7 +5231,7 @@
         <v>155</v>
       </c>
       <c r="J99" s="7" t="n">
-        <v>0.8129</v>
+        <v>0.8127</v>
       </c>
       <c r="K99" s="5" t="n">
         <v>75</v>
@@ -5279,7 +5279,7 @@
         <v>95</v>
       </c>
       <c r="J100" s="11" t="n">
-        <v>0.7052</v>
+        <v>0.7049</v>
       </c>
       <c r="K100" s="8" t="n">
         <v>45</v>
@@ -5419,7 +5419,7 @@
         <v>281</v>
       </c>
       <c r="J103" s="7" t="n">
-        <v>0.8925</v>
+        <v>0.8929</v>
       </c>
       <c r="K103" s="5" t="n">
         <v>135</v>
@@ -5467,7 +5467,7 @@
         <v>140</v>
       </c>
       <c r="J104" s="11" t="n">
-        <v>0.9357</v>
+        <v>0.9353</v>
       </c>
       <c r="K104" s="8" t="n">
         <v>65</v>
@@ -5515,7 +5515,7 @@
         <v>71</v>
       </c>
       <c r="J105" s="11" t="n">
-        <v>0.8</v>
+        <v>0.8023</v>
       </c>
       <c r="K105" s="8" t="n">
         <v>35</v>
@@ -5611,7 +5611,7 @@
         <v>30</v>
       </c>
       <c r="J107" s="11" t="n">
-        <v>0.9</v>
+        <v>0.8997000000000001</v>
       </c>
       <c r="K107" s="8" t="n">
         <v>15</v>
@@ -5655,7 +5655,7 @@
         <v>314</v>
       </c>
       <c r="J108" s="7" t="n">
-        <v>0.8328</v>
+        <v>0.834</v>
       </c>
       <c r="K108" s="5" t="n">
         <v>150</v>
@@ -5703,7 +5703,7 @@
         <v>29</v>
       </c>
       <c r="J109" s="11" t="n">
-        <v>0.5</v>
+        <v>0.5171</v>
       </c>
       <c r="K109" s="8" t="n">
         <v>10</v>
@@ -5751,7 +5751,7 @@
         <v>120</v>
       </c>
       <c r="J110" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9498</v>
       </c>
       <c r="K110" s="8" t="n">
         <v>60</v>
@@ -5799,7 +5799,7 @@
         <v>145</v>
       </c>
       <c r="J111" s="11" t="n">
-        <v>0.7931</v>
+        <v>0.7924</v>
       </c>
       <c r="K111" s="8" t="n">
         <v>70</v>
@@ -5939,7 +5939,7 @@
         <v>30</v>
       </c>
       <c r="J114" s="7" t="n">
-        <v>0.6666</v>
+        <v>0.6663</v>
       </c>
       <c r="K114" s="5" t="n">
         <v>15</v>
@@ -5987,7 +5987,7 @@
         <v>30</v>
       </c>
       <c r="J115" s="11" t="n">
-        <v>0.6666</v>
+        <v>0.6663</v>
       </c>
       <c r="K115" s="8" t="n">
         <v>15</v>
@@ -6159,7 +6159,7 @@
         <v>10</v>
       </c>
       <c r="J119" s="11" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="K119" s="8" t="n">
         <v>5</v>
@@ -6207,7 +6207,7 @@
         <v>10</v>
       </c>
       <c r="J120" s="11" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="K120" s="8" t="n">
         <v>5</v>
@@ -6435,7 +6435,7 @@
         <v>81</v>
       </c>
       <c r="J125" s="7" t="n">
-        <v>0.8493000000000001</v>
+        <v>0.901</v>
       </c>
       <c r="K125" s="5" t="n">
         <v>34</v>
@@ -6483,7 +6483,7 @@
         <v>60</v>
       </c>
       <c r="J126" s="11" t="n">
-        <v>0.8666</v>
+        <v>0.9498</v>
       </c>
       <c r="K126" s="8" t="n">
         <v>29</v>
@@ -6563,7 +6563,7 @@
         <v>21</v>
       </c>
       <c r="J128" s="11" t="n">
-        <v>0.8</v>
+        <v>0.7616000000000001</v>
       </c>
       <c r="K128" s="8" t="n">
         <v>5</v>
@@ -6767,7 +6767,7 @@
         <v>8173</v>
       </c>
       <c r="J133" s="4" t="n">
-        <v>0.6345</v>
+        <v>0.8091</v>
       </c>
       <c r="K133" s="2" t="n">
         <v>2374</v>
@@ -6903,7 +6903,7 @@
         <v>323</v>
       </c>
       <c r="J136" s="7" t="n">
-        <v>0.7879</v>
+        <v>0.7894</v>
       </c>
       <c r="K136" s="5" t="n">
         <v>80</v>
@@ -7095,7 +7095,7 @@
         <v>63</v>
       </c>
       <c r="J140" s="11" t="n">
-        <v>0.8333</v>
+        <v>0.841</v>
       </c>
       <c r="K140" s="8" t="n">
         <v>15</v>
@@ -7283,7 +7283,7 @@
         <v>1238</v>
       </c>
       <c r="J144" s="7" t="n">
-        <v>0.8418</v>
+        <v>0.8502</v>
       </c>
       <c r="K144" s="5" t="n">
         <v>305</v>
@@ -7331,7 +7331,7 @@
         <v>60</v>
       </c>
       <c r="J145" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9498</v>
       </c>
       <c r="K145" s="8" t="n">
         <v>15</v>
@@ -7379,7 +7379,7 @@
         <v>208</v>
       </c>
       <c r="J146" s="11" t="n">
-        <v>0.8315</v>
+        <v>0.8314</v>
       </c>
       <c r="K146" s="8" t="n">
         <v>40</v>
@@ -7427,7 +7427,7 @@
         <v>180</v>
       </c>
       <c r="J147" s="11" t="n">
-        <v>0.9277</v>
+        <v>0.9273</v>
       </c>
       <c r="K147" s="8" t="n">
         <v>45</v>
@@ -7523,7 +7523,7 @@
         <v>60</v>
       </c>
       <c r="J149" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9497</v>
       </c>
       <c r="K149" s="8" t="n">
         <v>10</v>
@@ -7667,7 +7667,7 @@
         <v>100</v>
       </c>
       <c r="J152" s="11" t="n">
-        <v>0.8363</v>
+        <v>0.9492</v>
       </c>
       <c r="K152" s="8" t="n">
         <v>55</v>
@@ -7715,7 +7715,7 @@
         <v>190</v>
       </c>
       <c r="J153" s="11" t="n">
-        <v>0.8736</v>
+        <v>0.8733</v>
       </c>
       <c r="K153" s="8" t="n">
         <v>45</v>
@@ -7763,7 +7763,7 @@
         <v>130</v>
       </c>
       <c r="J154" s="11" t="n">
-        <v>0.6589</v>
+        <v>0.6534</v>
       </c>
       <c r="K154" s="8" t="n">
         <v>30</v>
@@ -7807,7 +7807,7 @@
         <v>747</v>
       </c>
       <c r="J155" s="7" t="n">
-        <v>0.7712</v>
+        <v>0.7749</v>
       </c>
       <c r="K155" s="5" t="n">
         <v>170</v>
@@ -7903,7 +7903,7 @@
         <v>160</v>
       </c>
       <c r="J157" s="11" t="n">
-        <v>0.775</v>
+        <v>0.7995</v>
       </c>
       <c r="K157" s="8" t="n">
         <v>40</v>
@@ -7951,7 +7951,7 @@
         <v>60</v>
       </c>
       <c r="J158" s="11" t="n">
-        <v>0.8833</v>
+        <v>0.883</v>
       </c>
       <c r="K158" s="8" t="n">
         <v>15</v>
@@ -7999,7 +7999,7 @@
         <v>30</v>
       </c>
       <c r="J159" s="11" t="n">
-        <v>0.5666</v>
+        <v>0.5664</v>
       </c>
       <c r="K159" s="8" t="n">
         <v>5</v>
@@ -8095,7 +8095,7 @@
         <v>199</v>
       </c>
       <c r="J161" s="11" t="n">
-        <v>0.6888</v>
+        <v>0.6831</v>
       </c>
       <c r="K161" s="8" t="n">
         <v>40</v>
@@ -8191,7 +8191,7 @@
         <v>38</v>
       </c>
       <c r="J163" s="11" t="n">
-        <v>0.975</v>
+        <v>0.9735</v>
       </c>
       <c r="K163" s="8" t="n">
         <v>10</v>
@@ -8235,7 +8235,7 @@
         <v>4126</v>
       </c>
       <c r="J164" s="7" t="n">
-        <v>0.5155999999999999</v>
+        <v>0.7825</v>
       </c>
       <c r="K164" s="5" t="n">
         <v>985</v>
@@ -8283,7 +8283,7 @@
         <v>175</v>
       </c>
       <c r="J165" s="11" t="n">
-        <v>0.8742</v>
+        <v>0.874</v>
       </c>
       <c r="K165" s="8" t="n">
         <v>45</v>
@@ -8379,7 +8379,7 @@
         <v>260</v>
       </c>
       <c r="J167" s="11" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.7842</v>
       </c>
       <c r="K167" s="8" t="n">
         <v>55</v>
@@ -8427,7 +8427,7 @@
         <v>81</v>
       </c>
       <c r="J168" s="11" t="n">
-        <v>0.075</v>
+        <v>0.7279</v>
       </c>
       <c r="K168" s="8" t="n">
         <v>20</v>
@@ -8475,7 +8475,7 @@
         <v>160</v>
       </c>
       <c r="J169" s="11" t="n">
-        <v>0.375</v>
+        <v>0.7936</v>
       </c>
       <c r="K169" s="8" t="n">
         <v>40</v>
@@ -8523,7 +8523,7 @@
         <v>80</v>
       </c>
       <c r="J170" s="11" t="n">
-        <v>0.4375</v>
+        <v>0.4625</v>
       </c>
       <c r="K170" s="8" t="n">
         <v>15</v>
@@ -8571,7 +8571,7 @@
         <v>59</v>
       </c>
       <c r="J171" s="11" t="n">
-        <v>0.7333</v>
+        <v>0.7285</v>
       </c>
       <c r="K171" s="8" t="n">
         <v>15</v>
@@ -8619,7 +8619,7 @@
         <v>280</v>
       </c>
       <c r="J172" s="11" t="n">
-        <v>0.7714</v>
+        <v>0.771</v>
       </c>
       <c r="K172" s="8" t="n">
         <v>65</v>
@@ -8667,7 +8667,7 @@
         <v>160</v>
       </c>
       <c r="J173" s="11" t="n">
-        <v>0.8148</v>
+        <v>0.8434</v>
       </c>
       <c r="K173" s="8" t="n">
         <v>40</v>
@@ -8811,7 +8811,7 @@
         <v>60</v>
       </c>
       <c r="J176" s="11" t="n">
-        <v>0.9</v>
+        <v>0.9163</v>
       </c>
       <c r="K176" s="8" t="n">
         <v>15</v>
@@ -8859,7 +8859,7 @@
         <v>79</v>
       </c>
       <c r="J177" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9489</v>
       </c>
       <c r="K177" s="8" t="n">
         <v>15</v>
@@ -9003,7 +9003,7 @@
         <v>60</v>
       </c>
       <c r="J180" s="11" t="n">
-        <v>0.8833</v>
+        <v>0.8829</v>
       </c>
       <c r="K180" s="8" t="n">
         <v>15</v>
@@ -9051,7 +9051,7 @@
         <v>180</v>
       </c>
       <c r="J181" s="11" t="n">
-        <v>0</v>
+        <v>0.8107</v>
       </c>
       <c r="K181" s="8" t="n">
         <v>40</v>
@@ -9147,7 +9147,7 @@
         <v>200</v>
       </c>
       <c r="J183" s="11" t="n">
-        <v>0.7909</v>
+        <v>0.795</v>
       </c>
       <c r="K183" s="8" t="n">
         <v>50</v>
@@ -9195,7 +9195,7 @@
         <v>198</v>
       </c>
       <c r="J184" s="11" t="n">
-        <v>0.76</v>
+        <v>0.7621</v>
       </c>
       <c r="K184" s="8" t="n">
         <v>50</v>
@@ -9243,7 +9243,7 @@
         <v>99</v>
       </c>
       <c r="J185" s="11" t="n">
-        <v>0.88</v>
+        <v>0.8787</v>
       </c>
       <c r="K185" s="8" t="n">
         <v>20</v>
@@ -9339,7 +9339,7 @@
         <v>41</v>
       </c>
       <c r="J187" s="11" t="n">
-        <v>0.85</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="K187" s="8" t="n">
         <v>10</v>
@@ -9387,7 +9387,7 @@
         <v>59</v>
       </c>
       <c r="J188" s="11" t="n">
-        <v>0.6833</v>
+        <v>0.6604</v>
       </c>
       <c r="K188" s="8" t="n">
         <v>15</v>
@@ -9435,7 +9435,7 @@
         <v>278</v>
       </c>
       <c r="J189" s="11" t="n">
-        <v>0.7665999999999999</v>
+        <v>0.7762</v>
       </c>
       <c r="K189" s="8" t="n">
         <v>70</v>
@@ -9483,7 +9483,7 @@
         <v>293</v>
       </c>
       <c r="J190" s="11" t="n">
-        <v>0</v>
+        <v>0.8663999999999999</v>
       </c>
       <c r="K190" s="8" t="n">
         <v>70</v>
@@ -9531,7 +9531,7 @@
         <v>416</v>
       </c>
       <c r="J191" s="11" t="n">
-        <v>0.4428</v>
+        <v>0.6343</v>
       </c>
       <c r="K191" s="8" t="n">
         <v>90</v>
@@ -9579,7 +9579,7 @@
         <v>110</v>
       </c>
       <c r="J192" s="11" t="n">
-        <v>0.1</v>
+        <v>0.5907</v>
       </c>
       <c r="K192" s="8" t="n">
         <v>20</v>
@@ -9627,7 +9627,7 @@
         <v>139</v>
       </c>
       <c r="J193" s="11" t="n">
-        <v>0</v>
+        <v>0.7479</v>
       </c>
       <c r="K193" s="8" t="n">
         <v>40</v>
@@ -9675,7 +9675,7 @@
         <v>80</v>
       </c>
       <c r="J194" s="11" t="n">
-        <v>0.73</v>
+        <v>0.875</v>
       </c>
       <c r="K194" s="8" t="n">
         <v>25</v>
@@ -9723,7 +9723,7 @@
         <v>120</v>
       </c>
       <c r="J195" s="11" t="n">
-        <v>0.675</v>
+        <v>0.858</v>
       </c>
       <c r="K195" s="8" t="n">
         <v>30</v>
@@ -9771,7 +9771,7 @@
         <v>99</v>
       </c>
       <c r="J196" s="11" t="n">
-        <v>0.7</v>
+        <v>0.8787</v>
       </c>
       <c r="K196" s="8" t="n">
         <v>25</v>
@@ -9819,7 +9819,7 @@
         <v>140</v>
       </c>
       <c r="J197" s="11" t="n">
-        <v>0.1357</v>
+        <v>0.8354</v>
       </c>
       <c r="K197" s="8" t="n">
         <v>35</v>
@@ -9863,7 +9863,7 @@
         <v>219</v>
       </c>
       <c r="J198" s="7" t="n">
-        <v>0</v>
+        <v>0.9404</v>
       </c>
       <c r="K198" s="5" t="n">
         <v>55</v>
@@ -9911,7 +9911,7 @@
         <v>139</v>
       </c>
       <c r="J199" s="11" t="n">
-        <v>0</v>
+        <v>0.9564</v>
       </c>
       <c r="K199" s="8" t="n">
         <v>35</v>
@@ -9959,7 +9959,7 @@
         <v>80</v>
       </c>
       <c r="J200" s="11" t="n">
-        <v>0</v>
+        <v>0.9125</v>
       </c>
       <c r="K200" s="8" t="n">
         <v>20</v>
@@ -10003,7 +10003,7 @@
         <v>1200</v>
       </c>
       <c r="J201" s="7" t="n">
-        <v>0.7716</v>
+        <v>0.8599</v>
       </c>
       <c r="K201" s="5" t="n">
         <v>435</v>
@@ -10051,7 +10051,7 @@
         <v>119</v>
       </c>
       <c r="J202" s="11" t="n">
-        <v>0.9583</v>
+        <v>0.9577</v>
       </c>
       <c r="K202" s="8" t="n">
         <v>30</v>
@@ -10099,7 +10099,7 @@
         <v>40</v>
       </c>
       <c r="J203" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K203" s="8" t="n">
         <v>10</v>
@@ -10147,7 +10147,7 @@
         <v>19</v>
       </c>
       <c r="J204" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9471000000000001</v>
       </c>
       <c r="K204" s="8" t="n">
         <v>5</v>
@@ -10291,7 +10291,7 @@
         <v>40</v>
       </c>
       <c r="J207" s="11" t="n">
-        <v>0.8</v>
+        <v>0.825</v>
       </c>
       <c r="K207" s="8" t="n">
         <v>10</v>
@@ -10339,7 +10339,7 @@
         <v>100</v>
       </c>
       <c r="J208" s="11" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="K208" s="8" t="n">
         <v>25</v>
@@ -10387,7 +10387,7 @@
         <v>141</v>
       </c>
       <c r="J209" s="11" t="n">
-        <v>0.8071</v>
+        <v>0.9144</v>
       </c>
       <c r="K209" s="8" t="n">
         <v>35</v>
@@ -10435,7 +10435,7 @@
         <v>100</v>
       </c>
       <c r="J210" s="11" t="n">
-        <v>0.7433999999999999</v>
+        <v>0.7431</v>
       </c>
       <c r="K210" s="8" t="n">
         <v>160</v>
@@ -10483,7 +10483,7 @@
         <v>381</v>
       </c>
       <c r="J211" s="11" t="n">
-        <v>0.7917999999999999</v>
+        <v>0.8313</v>
       </c>
       <c r="K211" s="8" t="n">
         <v>95</v>
@@ -10531,7 +10531,7 @@
         <v>40</v>
       </c>
       <c r="J212" s="11" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="K212" s="8" t="n">
         <v>10</v>
@@ -10667,7 +10667,7 @@
         <v>200</v>
       </c>
       <c r="J215" s="7" t="n">
-        <v>0.8197</v>
+        <v>0.8192</v>
       </c>
       <c r="K215" s="5" t="n">
         <v>314</v>
@@ -10715,7 +10715,7 @@
         <v>60</v>
       </c>
       <c r="J216" s="11" t="n">
-        <v>0.8</v>
+        <v>0.7998</v>
       </c>
       <c r="K216" s="8" t="n">
         <v>10</v>
@@ -10763,7 +10763,7 @@
         <v>20</v>
       </c>
       <c r="J217" s="11" t="n">
-        <v>0.925</v>
+        <v>0.85</v>
       </c>
       <c r="K217" s="8" t="n">
         <v>5</v>
@@ -10811,7 +10811,7 @@
         <v>100</v>
       </c>
       <c r="J218" s="11" t="n">
-        <v>0.8044</v>
+        <v>0.8185</v>
       </c>
       <c r="K218" s="8" t="n">
         <v>294</v>
@@ -10907,7 +10907,7 @@
         <v>3382</v>
       </c>
       <c r="J220" s="4" t="n">
-        <v>0.762</v>
+        <v>0.837</v>
       </c>
       <c r="K220" s="2" t="n">
         <v>833</v>
@@ -10951,7 +10951,7 @@
         <v>60</v>
       </c>
       <c r="J221" s="7" t="n">
-        <v>0.7166</v>
+        <v>0.7163</v>
       </c>
       <c r="K221" s="5" t="n">
         <v>15</v>
@@ -10999,7 +10999,7 @@
         <v>60</v>
       </c>
       <c r="J222" s="11" t="n">
-        <v>0.7166</v>
+        <v>0.7163</v>
       </c>
       <c r="K222" s="8" t="n">
         <v>15</v>
@@ -11043,7 +11043,7 @@
         <v>20</v>
       </c>
       <c r="J223" s="7" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="K223" s="5" t="n">
         <v>5</v>
@@ -11091,7 +11091,7 @@
         <v>20</v>
       </c>
       <c r="J224" s="11" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="K224" s="8" t="n">
         <v>5</v>
@@ -11135,7 +11135,7 @@
         <v>140</v>
       </c>
       <c r="J225" s="7" t="n">
-        <v>0.9308999999999999</v>
+        <v>0.9429</v>
       </c>
       <c r="K225" s="5" t="n">
         <v>35</v>
@@ -11183,7 +11183,7 @@
         <v>100</v>
       </c>
       <c r="J226" s="11" t="n">
-        <v>0.9333</v>
+        <v>0.95</v>
       </c>
       <c r="K226" s="8" t="n">
         <v>25</v>
@@ -11275,7 +11275,7 @@
         <v>522</v>
       </c>
       <c r="J228" s="7" t="n">
-        <v>0.9096</v>
+        <v>0.9076</v>
       </c>
       <c r="K228" s="5" t="n">
         <v>130</v>
@@ -11371,7 +11371,7 @@
         <v>241</v>
       </c>
       <c r="J230" s="11" t="n">
-        <v>0.9458</v>
+        <v>0.9411</v>
       </c>
       <c r="K230" s="8" t="n">
         <v>60</v>
@@ -11419,7 +11419,7 @@
         <v>201</v>
       </c>
       <c r="J231" s="11" t="n">
-        <v>0.86</v>
+        <v>0.8604000000000001</v>
       </c>
       <c r="K231" s="8" t="n">
         <v>50</v>
@@ -11463,7 +11463,7 @@
         <v>608</v>
       </c>
       <c r="J232" s="7" t="n">
-        <v>0.7508</v>
+        <v>0.7742</v>
       </c>
       <c r="K232" s="5" t="n">
         <v>135</v>
@@ -11511,7 +11511,7 @@
         <v>45</v>
       </c>
       <c r="J233" s="11" t="n">
-        <v>0.525</v>
+        <v>0.533</v>
       </c>
       <c r="K233" s="8" t="n">
         <v>5</v>
@@ -11655,7 +11655,7 @@
         <v>140</v>
       </c>
       <c r="J236" s="11" t="n">
-        <v>0.3571</v>
+        <v>0.4212</v>
       </c>
       <c r="K236" s="8" t="n">
         <v>25</v>
@@ -11703,7 +11703,7 @@
         <v>209</v>
       </c>
       <c r="J237" s="11" t="n">
-        <v>0.9454</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="K237" s="8" t="n">
         <v>50</v>
@@ -11751,7 +11751,7 @@
         <v>174</v>
       </c>
       <c r="J238" s="11" t="n">
-        <v>0.8351</v>
+        <v>0.8673</v>
       </c>
       <c r="K238" s="8" t="n">
         <v>45</v>
@@ -11795,7 +11795,7 @@
         <v>703</v>
       </c>
       <c r="J239" s="7" t="n">
-        <v>0.8763</v>
+        <v>0.8942</v>
       </c>
       <c r="K239" s="5" t="n">
         <v>160</v>
@@ -11843,7 +11843,7 @@
         <v>241</v>
       </c>
       <c r="J240" s="11" t="n">
-        <v>0.8272</v>
+        <v>0.8376</v>
       </c>
       <c r="K240" s="8" t="n">
         <v>55</v>
@@ -11891,7 +11891,7 @@
         <v>290</v>
       </c>
       <c r="J241" s="11" t="n">
-        <v>0.9517</v>
+        <v>0.9510999999999999</v>
       </c>
       <c r="K241" s="8" t="n">
         <v>70</v>
@@ -11981,7 +11981,7 @@
         <v>20</v>
       </c>
       <c r="J243" s="11" t="n">
-        <v>0.55</v>
+        <v>0.95</v>
       </c>
       <c r="K243" s="8" t="n">
         <v>5</v>
@@ -12029,7 +12029,7 @@
         <v>132</v>
       </c>
       <c r="J244" s="11" t="n">
-        <v>0.8384</v>
+        <v>0.8557</v>
       </c>
       <c r="K244" s="8" t="n">
         <v>30</v>
@@ -12073,7 +12073,7 @@
         <v>439</v>
       </c>
       <c r="J245" s="7" t="n">
-        <v>0.2632</v>
+        <v>0.7539</v>
       </c>
       <c r="K245" s="5" t="n">
         <v>134</v>
@@ -12121,7 +12121,7 @@
         <v>60</v>
       </c>
       <c r="J246" s="11" t="n">
-        <v>0</v>
+        <v>0.7166</v>
       </c>
       <c r="K246" s="8" t="n">
         <v>39</v>
@@ -12169,7 +12169,7 @@
         <v>79</v>
       </c>
       <c r="J247" s="11" t="n">
-        <v>0.4375</v>
+        <v>0.7593</v>
       </c>
       <c r="K247" s="8" t="n">
         <v>20</v>
@@ -12217,7 +12217,7 @@
         <v>160</v>
       </c>
       <c r="J248" s="11" t="n">
-        <v>0</v>
+        <v>0.7499</v>
       </c>
       <c r="K248" s="8" t="n">
         <v>40</v>
@@ -12265,7 +12265,7 @@
         <v>40</v>
       </c>
       <c r="J249" s="11" t="n">
-        <v>0</v>
+        <v>0.675</v>
       </c>
       <c r="K249" s="8" t="n">
         <v>10</v>
@@ -12357,7 +12357,7 @@
         <v>460</v>
       </c>
       <c r="J251" s="7" t="n">
-        <v>0.8421999999999999</v>
+        <v>0.8451</v>
       </c>
       <c r="K251" s="5" t="n">
         <v>120</v>
@@ -12405,7 +12405,7 @@
         <v>340</v>
       </c>
       <c r="J252" s="11" t="n">
-        <v>0.8411</v>
+        <v>0.8406</v>
       </c>
       <c r="K252" s="8" t="n">
         <v>90</v>
@@ -12453,7 +12453,7 @@
         <v>120</v>
       </c>
       <c r="J253" s="11" t="n">
-        <v>0.8454</v>
+        <v>0.858</v>
       </c>
       <c r="K253" s="8" t="n">
         <v>30</v>
@@ -12497,7 +12497,7 @@
         <v>430</v>
       </c>
       <c r="J254" s="7" t="n">
-        <v>0.7983</v>
+        <v>0.8065</v>
       </c>
       <c r="K254" s="5" t="n">
         <v>99</v>
@@ -12545,7 +12545,7 @@
         <v>330</v>
       </c>
       <c r="J255" s="11" t="n">
-        <v>0.7948</v>
+        <v>0.8055</v>
       </c>
       <c r="K255" s="8" t="n">
         <v>79</v>
@@ -12737,7 +12737,7 @@
         <v>7405</v>
       </c>
       <c r="J259" s="4" t="n">
-        <v>0.7672</v>
+        <v>0.9396</v>
       </c>
       <c r="K259" s="2" t="n">
         <v>3694</v>
@@ -12873,7 +12873,7 @@
         <v>1842</v>
       </c>
       <c r="J262" s="7" t="n">
-        <v>0.8434</v>
+        <v>0.9550999999999999</v>
       </c>
       <c r="K262" s="5" t="n">
         <v>914</v>
@@ -12921,7 +12921,7 @@
         <v>80</v>
       </c>
       <c r="J263" s="11" t="n">
-        <v>0.2777</v>
+        <v>0.85</v>
       </c>
       <c r="K263" s="8" t="n">
         <v>35</v>
@@ -12969,7 +12969,7 @@
         <v>40</v>
       </c>
       <c r="J264" s="11" t="n">
-        <v>0.475</v>
+        <v>0.875</v>
       </c>
       <c r="K264" s="8" t="n">
         <v>20</v>
@@ -13017,7 +13017,7 @@
         <v>52</v>
       </c>
       <c r="J265" s="11" t="n">
-        <v>0.98</v>
+        <v>0.9804</v>
       </c>
       <c r="K265" s="8" t="n">
         <v>24</v>
@@ -13065,7 +13065,7 @@
         <v>69</v>
       </c>
       <c r="J266" s="11" t="n">
-        <v>0.9714</v>
+        <v>0.9704</v>
       </c>
       <c r="K266" s="8" t="n">
         <v>35</v>
@@ -13113,7 +13113,7 @@
         <v>120</v>
       </c>
       <c r="J267" s="11" t="n">
-        <v>0.9666</v>
+        <v>0.983</v>
       </c>
       <c r="K267" s="8" t="n">
         <v>60</v>
@@ -13161,7 +13161,7 @@
         <v>70</v>
       </c>
       <c r="J268" s="11" t="n">
-        <v>0.8833</v>
+        <v>0.8851</v>
       </c>
       <c r="K268" s="8" t="n">
         <v>35</v>
@@ -13209,7 +13209,7 @@
         <v>369</v>
       </c>
       <c r="J269" s="11" t="n">
-        <v>0.9621</v>
+        <v>0.9858</v>
       </c>
       <c r="K269" s="8" t="n">
         <v>185</v>
@@ -13257,7 +13257,7 @@
         <v>10</v>
       </c>
       <c r="J270" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K270" s="8" t="n">
         <v>5</v>
@@ -13305,7 +13305,7 @@
         <v>110</v>
       </c>
       <c r="J271" s="11" t="n">
-        <v>0.7181</v>
+        <v>0.9902</v>
       </c>
       <c r="K271" s="8" t="n">
         <v>55</v>
@@ -13353,7 +13353,7 @@
         <v>110</v>
       </c>
       <c r="J272" s="11" t="n">
-        <v>0.9727</v>
+        <v>0.9719</v>
       </c>
       <c r="K272" s="8" t="n">
         <v>55</v>
@@ -13401,7 +13401,7 @@
         <v>90</v>
       </c>
       <c r="J273" s="11" t="n">
-        <v>0.9777</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="K273" s="8" t="n">
         <v>50</v>
@@ -13449,7 +13449,7 @@
         <v>60</v>
       </c>
       <c r="J274" s="11" t="n">
-        <v>0.9</v>
+        <v>0.8997000000000001</v>
       </c>
       <c r="K274" s="8" t="n">
         <v>30</v>
@@ -13497,7 +13497,7 @@
         <v>121</v>
       </c>
       <c r="J275" s="11" t="n">
-        <v>0.8914</v>
+        <v>0.8921</v>
       </c>
       <c r="K275" s="8" t="n">
         <v>60</v>
@@ -13545,7 +13545,7 @@
         <v>80</v>
       </c>
       <c r="J276" s="11" t="n">
-        <v>0.9428</v>
+        <v>0.95</v>
       </c>
       <c r="K276" s="8" t="n">
         <v>40</v>
@@ -13689,7 +13689,7 @@
         <v>50</v>
       </c>
       <c r="J279" s="11" t="n">
-        <v>0.2</v>
+        <v>0.98</v>
       </c>
       <c r="K279" s="8" t="n">
         <v>25</v>
@@ -13737,7 +13737,7 @@
         <v>10</v>
       </c>
       <c r="J280" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K280" s="8" t="n">
         <v>5</v>
@@ -13785,7 +13785,7 @@
         <v>119</v>
       </c>
       <c r="J281" s="11" t="n">
-        <v>0.9666</v>
+        <v>0.9577</v>
       </c>
       <c r="K281" s="8" t="n">
         <v>55</v>
@@ -13833,7 +13833,7 @@
         <v>70</v>
       </c>
       <c r="J282" s="11" t="n">
-        <v>0.9714</v>
+        <v>0.9709</v>
       </c>
       <c r="K282" s="8" t="n">
         <v>35</v>
@@ -13881,7 +13881,7 @@
         <v>51</v>
       </c>
       <c r="J283" s="11" t="n">
-        <v>1</v>
+        <v>0.9997</v>
       </c>
       <c r="K283" s="8" t="n">
         <v>25</v>
@@ -13929,7 +13929,7 @@
         <v>30</v>
       </c>
       <c r="J284" s="11" t="n">
-        <v>1</v>
+        <v>0.9998</v>
       </c>
       <c r="K284" s="8" t="n">
         <v>15</v>
@@ -14025,7 +14025,7 @@
         <v>61</v>
       </c>
       <c r="J286" s="11" t="n">
-        <v>0.15</v>
+        <v>0.9503</v>
       </c>
       <c r="K286" s="8" t="n">
         <v>30</v>
@@ -14069,7 +14069,7 @@
         <v>660</v>
       </c>
       <c r="J287" s="7" t="n">
-        <v>0.2906</v>
+        <v>0.8695000000000001</v>
       </c>
       <c r="K287" s="5" t="n">
         <v>343</v>
@@ -14117,7 +14117,7 @@
         <v>11</v>
       </c>
       <c r="J288" s="11" t="n">
-        <v>0</v>
+        <v>0.909</v>
       </c>
       <c r="K288" s="8" t="n">
         <v>5</v>
@@ -14165,7 +14165,7 @@
         <v>80</v>
       </c>
       <c r="J289" s="11" t="n">
-        <v>0.2625</v>
+        <v>0.65</v>
       </c>
       <c r="K289" s="8" t="n">
         <v>40</v>
@@ -14213,7 +14213,7 @@
         <v>120</v>
       </c>
       <c r="J290" s="11" t="n">
-        <v>0.4153</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="K290" s="8" t="n">
         <v>65</v>
@@ -14261,7 +14261,7 @@
         <v>70</v>
       </c>
       <c r="J291" s="11" t="n">
-        <v>0.2857</v>
+        <v>0.9566</v>
       </c>
       <c r="K291" s="8" t="n">
         <v>35</v>
@@ -14309,7 +14309,7 @@
         <v>80</v>
       </c>
       <c r="J292" s="11" t="n">
-        <v>0.125</v>
+        <v>1</v>
       </c>
       <c r="K292" s="8" t="n">
         <v>40</v>
@@ -14357,7 +14357,7 @@
         <v>199</v>
       </c>
       <c r="J293" s="11" t="n">
-        <v>0.1857</v>
+        <v>0.8137</v>
       </c>
       <c r="K293" s="8" t="n">
         <v>108</v>
@@ -14405,7 +14405,7 @@
         <v>100</v>
       </c>
       <c r="J294" s="11" t="n">
-        <v>0.54</v>
+        <v>0.91</v>
       </c>
       <c r="K294" s="8" t="n">
         <v>50</v>
@@ -14449,7 +14449,7 @@
         <v>1409</v>
       </c>
       <c r="J295" s="7" t="n">
-        <v>0.4896</v>
+        <v>0.9081</v>
       </c>
       <c r="K295" s="5" t="n">
         <v>697</v>
@@ -14497,7 +14497,7 @@
         <v>90</v>
       </c>
       <c r="J296" s="11" t="n">
-        <v>0.73</v>
+        <v>0.8774</v>
       </c>
       <c r="K296" s="8" t="n">
         <v>50</v>
@@ -14545,7 +14545,7 @@
         <v>30</v>
       </c>
       <c r="J297" s="11" t="n">
-        <v>0.2666</v>
+        <v>0.7999000000000001</v>
       </c>
       <c r="K297" s="8" t="n">
         <v>20</v>
@@ -14593,7 +14593,7 @@
         <v>20</v>
       </c>
       <c r="J298" s="11" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K298" s="8" t="n">
         <v>10</v>
@@ -14641,7 +14641,7 @@
         <v>19</v>
       </c>
       <c r="J299" s="11" t="n">
-        <v>0.65</v>
+        <v>0.6314</v>
       </c>
       <c r="K299" s="8" t="n">
         <v>5</v>
@@ -14689,7 +14689,7 @@
         <v>101</v>
       </c>
       <c r="J300" s="11" t="n">
-        <v>0.15</v>
+        <v>0.6435</v>
       </c>
       <c r="K300" s="8" t="n">
         <v>45</v>
@@ -14737,7 +14737,7 @@
         <v>100</v>
       </c>
       <c r="J301" s="11" t="n">
-        <v>0.38</v>
+        <v>0.91</v>
       </c>
       <c r="K301" s="8" t="n">
         <v>50</v>
@@ -14785,7 +14785,7 @@
         <v>130</v>
       </c>
       <c r="J302" s="11" t="n">
-        <v>0.325</v>
+        <v>0.8534</v>
       </c>
       <c r="K302" s="8" t="n">
         <v>65</v>
@@ -14833,7 +14833,7 @@
         <v>20</v>
       </c>
       <c r="J303" s="11" t="n">
-        <v>0.45</v>
+        <v>0.95</v>
       </c>
       <c r="K303" s="8" t="n">
         <v>10</v>
@@ -14881,7 +14881,7 @@
         <v>310</v>
       </c>
       <c r="J304" s="11" t="n">
-        <v>0.5096000000000001</v>
+        <v>0.9802</v>
       </c>
       <c r="K304" s="8" t="n">
         <v>150</v>
@@ -14929,7 +14929,7 @@
         <v>50</v>
       </c>
       <c r="J305" s="11" t="n">
-        <v>0</v>
+        <v>0.88</v>
       </c>
       <c r="K305" s="8" t="n">
         <v>25</v>
@@ -15025,7 +15025,7 @@
         <v>110</v>
       </c>
       <c r="J307" s="11" t="n">
-        <v>0.7454</v>
+        <v>0.9176</v>
       </c>
       <c r="K307" s="8" t="n">
         <v>60</v>
@@ -15073,7 +15073,7 @@
         <v>210</v>
       </c>
       <c r="J308" s="11" t="n">
-        <v>0.7571</v>
+        <v>0.9757</v>
       </c>
       <c r="K308" s="8" t="n">
         <v>98</v>
@@ -15121,7 +15121,7 @@
         <v>79</v>
       </c>
       <c r="J309" s="11" t="n">
-        <v>0.575</v>
+        <v>0.9488</v>
       </c>
       <c r="K309" s="8" t="n">
         <v>40</v>
@@ -15169,7 +15169,7 @@
         <v>110</v>
       </c>
       <c r="J310" s="11" t="n">
-        <v>0.3363</v>
+        <v>0.9631999999999999</v>
       </c>
       <c r="K310" s="8" t="n">
         <v>54</v>
@@ -15217,7 +15217,7 @@
         <v>10</v>
       </c>
       <c r="J311" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K311" s="8" t="n">
         <v>5</v>
@@ -15261,7 +15261,7 @@
         <v>1475</v>
       </c>
       <c r="J312" s="7" t="n">
-        <v>0.9764</v>
+        <v>0.9772</v>
       </c>
       <c r="K312" s="5" t="n">
         <v>735</v>
@@ -15549,7 +15549,7 @@
         <v>81</v>
       </c>
       <c r="J318" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9502</v>
       </c>
       <c r="K318" s="8" t="n">
         <v>40</v>
@@ -15597,7 +15597,7 @@
         <v>141</v>
       </c>
       <c r="J319" s="11" t="n">
-        <v>0.9928</v>
+        <v>0.9923999999999999</v>
       </c>
       <c r="K319" s="8" t="n">
         <v>70</v>
@@ -15645,7 +15645,7 @@
         <v>499</v>
       </c>
       <c r="J320" s="11" t="n">
-        <v>0.9714</v>
+        <v>0.9713000000000001</v>
       </c>
       <c r="K320" s="8" t="n">
         <v>250</v>
@@ -15741,7 +15741,7 @@
         <v>70</v>
       </c>
       <c r="J322" s="11" t="n">
-        <v>0.9571</v>
+        <v>0.9566</v>
       </c>
       <c r="K322" s="8" t="n">
         <v>35</v>
@@ -15837,7 +15837,7 @@
         <v>30</v>
       </c>
       <c r="J324" s="11" t="n">
-        <v>1</v>
+        <v>0.9998</v>
       </c>
       <c r="K324" s="8" t="n">
         <v>15</v>
@@ -15885,7 +15885,7 @@
         <v>18</v>
       </c>
       <c r="J325" s="11" t="n">
-        <v>1</v>
+        <v>0.9998</v>
       </c>
       <c r="K325" s="8" t="n">
         <v>10</v>
@@ -16077,7 +16077,7 @@
         <v>30</v>
       </c>
       <c r="J329" s="11" t="n">
-        <v>1</v>
+        <v>0.9997</v>
       </c>
       <c r="K329" s="8" t="n">
         <v>15</v>
@@ -16173,7 +16173,7 @@
         <v>30</v>
       </c>
       <c r="J331" s="11" t="n">
-        <v>0.9666</v>
+        <v>0.9664</v>
       </c>
       <c r="K331" s="8" t="n">
         <v>10</v>
@@ -16413,7 +16413,7 @@
         <v>60</v>
       </c>
       <c r="J336" s="11" t="n">
-        <v>0.9929</v>
+        <v>0.983</v>
       </c>
       <c r="K336" s="8" t="n">
         <v>30</v>
@@ -16461,7 +16461,7 @@
         <v>30</v>
       </c>
       <c r="J337" s="11" t="n">
-        <v>1</v>
+        <v>0.9997</v>
       </c>
       <c r="K337" s="8" t="n">
         <v>15</v>
@@ -16509,7 +16509,7 @@
         <v>30</v>
       </c>
       <c r="J338" s="11" t="n">
-        <v>0.9666</v>
+        <v>0.9664</v>
       </c>
       <c r="K338" s="8" t="n">
         <v>15</v>
@@ -16557,7 +16557,7 @@
         <v>50</v>
       </c>
       <c r="J339" s="11" t="n">
-        <v>0.92</v>
+        <v>0.96</v>
       </c>
       <c r="K339" s="8" t="n">
         <v>25</v>
@@ -16605,7 +16605,7 @@
         <v>30</v>
       </c>
       <c r="J340" s="11" t="n">
-        <v>1</v>
+        <v>0.9998</v>
       </c>
       <c r="K340" s="8" t="n">
         <v>15</v>
@@ -16649,7 +16649,7 @@
         <v>411</v>
       </c>
       <c r="J341" s="7" t="n">
-        <v>0.6226</v>
+        <v>0.8731</v>
       </c>
       <c r="K341" s="5" t="n">
         <v>205</v>
@@ -16697,7 +16697,7 @@
         <v>161</v>
       </c>
       <c r="J342" s="11" t="n">
-        <v>0.5379</v>
+        <v>0.745</v>
       </c>
       <c r="K342" s="8" t="n">
         <v>80</v>
@@ -16745,7 +16745,7 @@
         <v>10</v>
       </c>
       <c r="J343" s="11" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K343" s="8" t="n">
         <v>5</v>
@@ -16793,7 +16793,7 @@
         <v>60</v>
       </c>
       <c r="J344" s="11" t="n">
-        <v>0.5714</v>
+        <v>0.9663</v>
       </c>
       <c r="K344" s="8" t="n">
         <v>30</v>
@@ -16841,7 +16841,7 @@
         <v>150</v>
       </c>
       <c r="J345" s="11" t="n">
-        <v>0.8333</v>
+        <v>0.9661</v>
       </c>
       <c r="K345" s="8" t="n">
         <v>75</v>
@@ -16889,7 +16889,7 @@
         <v>20</v>
       </c>
       <c r="J346" s="11" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K346" s="8" t="n">
         <v>10</v>
@@ -16937,7 +16937,7 @@
         <v>10</v>
       </c>
       <c r="J347" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K347" s="8" t="n">
         <v>5</v>
@@ -16981,7 +16981,7 @@
         <v>1529</v>
       </c>
       <c r="J348" s="7" t="n">
-        <v>0.9622000000000001</v>
+        <v>0.959</v>
       </c>
       <c r="K348" s="5" t="n">
         <v>760</v>
@@ -17125,7 +17125,7 @@
         <v>182</v>
       </c>
       <c r="J351" s="11" t="n">
-        <v>0.9425</v>
+        <v>0.9167999999999999</v>
       </c>
       <c r="K351" s="8" t="n">
         <v>85</v>
@@ -17221,7 +17221,7 @@
         <v>387</v>
       </c>
       <c r="J353" s="11" t="n">
-        <v>0.9615</v>
+        <v>0.9606</v>
       </c>
       <c r="K353" s="8" t="n">
         <v>199</v>
@@ -17269,7 +17269,7 @@
         <v>70</v>
       </c>
       <c r="J354" s="11" t="n">
-        <v>1</v>
+        <v>0.9994</v>
       </c>
       <c r="K354" s="8" t="n">
         <v>35</v>
@@ -17365,7 +17365,7 @@
         <v>59</v>
       </c>
       <c r="J356" s="11" t="n">
-        <v>1</v>
+        <v>0.9992</v>
       </c>
       <c r="K356" s="8" t="n">
         <v>30</v>
@@ -17413,7 +17413,7 @@
         <v>81</v>
       </c>
       <c r="J357" s="11" t="n">
-        <v>0.9375</v>
+        <v>0.9377</v>
       </c>
       <c r="K357" s="8" t="n">
         <v>35</v>
@@ -17461,7 +17461,7 @@
         <v>60</v>
       </c>
       <c r="J358" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9497</v>
       </c>
       <c r="K358" s="8" t="n">
         <v>30</v>
@@ -17509,7 +17509,7 @@
         <v>100</v>
       </c>
       <c r="J359" s="11" t="n">
-        <v>0.9666</v>
+        <v>0.97</v>
       </c>
       <c r="K359" s="8" t="n">
         <v>51</v>
@@ -17605,7 +17605,7 @@
         <v>60</v>
       </c>
       <c r="J361" s="11" t="n">
-        <v>0.9</v>
+        <v>0.8997000000000001</v>
       </c>
       <c r="K361" s="8" t="n">
         <v>30</v>
@@ -17653,7 +17653,7 @@
         <v>30</v>
       </c>
       <c r="J362" s="11" t="n">
-        <v>0.9666</v>
+        <v>0.9665</v>
       </c>
       <c r="K362" s="8" t="n">
         <v>15</v>
@@ -17797,7 +17797,7 @@
         <v>81</v>
       </c>
       <c r="J365" s="11" t="n">
-        <v>0.9125</v>
+        <v>0.9131</v>
       </c>
       <c r="K365" s="8" t="n">
         <v>40</v>
@@ -17845,7 +17845,7 @@
         <v>59</v>
       </c>
       <c r="J366" s="11" t="n">
-        <v>1</v>
+        <v>0.9993</v>
       </c>
       <c r="K366" s="8" t="n">
         <v>30</v>
@@ -17893,7 +17893,7 @@
         <v>70</v>
       </c>
       <c r="J367" s="11" t="n">
-        <v>0.9857</v>
+        <v>0.9849</v>
       </c>
       <c r="K367" s="8" t="n">
         <v>35</v>
@@ -17937,7 +17937,7 @@
         <v>69</v>
       </c>
       <c r="J368" s="7" t="n">
-        <v>1</v>
+        <v>0.9994</v>
       </c>
       <c r="K368" s="5" t="n">
         <v>35</v>
@@ -17985,7 +17985,7 @@
         <v>69</v>
       </c>
       <c r="J369" s="11" t="n">
-        <v>1</v>
+        <v>0.9994</v>
       </c>
       <c r="K369" s="8" t="n">
         <v>35</v>
@@ -18033,7 +18033,7 @@
         <v>4559</v>
       </c>
       <c r="J370" s="4" t="n">
-        <v>0.6481</v>
+        <v>0.8364</v>
       </c>
       <c r="K370" s="2" t="n">
         <v>2268</v>
@@ -18169,7 +18169,7 @@
         <v>240</v>
       </c>
       <c r="J373" s="7" t="n">
-        <v>0.8833</v>
+        <v>0.9162</v>
       </c>
       <c r="K373" s="5" t="n">
         <v>125</v>
@@ -18265,7 +18265,7 @@
         <v>190</v>
       </c>
       <c r="J375" s="11" t="n">
-        <v>0.8894</v>
+        <v>0.931</v>
       </c>
       <c r="K375" s="8" t="n">
         <v>100</v>
@@ -18309,7 +18309,7 @@
         <v>89</v>
       </c>
       <c r="J376" s="7" t="n">
-        <v>0.9111</v>
+        <v>0.9095</v>
       </c>
       <c r="K376" s="5" t="n">
         <v>45</v>
@@ -18357,7 +18357,7 @@
         <v>89</v>
       </c>
       <c r="J377" s="11" t="n">
-        <v>0.9111</v>
+        <v>0.9095</v>
       </c>
       <c r="K377" s="8" t="n">
         <v>45</v>
@@ -18401,7 +18401,7 @@
         <v>1314</v>
       </c>
       <c r="J378" s="7" t="n">
-        <v>0.7772</v>
+        <v>0.8405</v>
       </c>
       <c r="K378" s="5" t="n">
         <v>645</v>
@@ -18449,7 +18449,7 @@
         <v>99</v>
       </c>
       <c r="J379" s="11" t="n">
-        <v>0.88</v>
+        <v>0.8686</v>
       </c>
       <c r="K379" s="8" t="n">
         <v>50</v>
@@ -18497,7 +18497,7 @@
         <v>30</v>
       </c>
       <c r="J380" s="11" t="n">
-        <v>0</v>
+        <v>0.7998</v>
       </c>
       <c r="K380" s="8" t="n">
         <v>15</v>
@@ -18545,7 +18545,7 @@
         <v>162</v>
       </c>
       <c r="J381" s="11" t="n">
-        <v>0.7937</v>
+        <v>0.839</v>
       </c>
       <c r="K381" s="8" t="n">
         <v>75</v>
@@ -18593,7 +18593,7 @@
         <v>192</v>
       </c>
       <c r="J382" s="11" t="n">
-        <v>0.8134</v>
+        <v>0.8121</v>
       </c>
       <c r="K382" s="8" t="n">
         <v>90</v>
@@ -18641,7 +18641,7 @@
         <v>270</v>
       </c>
       <c r="J383" s="11" t="n">
-        <v>0.8481</v>
+        <v>0.8478</v>
       </c>
       <c r="K383" s="8" t="n">
         <v>135</v>
@@ -18689,7 +18689,7 @@
         <v>364</v>
       </c>
       <c r="J384" s="11" t="n">
-        <v>0.8594000000000001</v>
+        <v>0.8921</v>
       </c>
       <c r="K384" s="8" t="n">
         <v>180</v>
@@ -18737,7 +18737,7 @@
         <v>119</v>
       </c>
       <c r="J385" s="11" t="n">
-        <v>0.6583</v>
+        <v>0.8568</v>
       </c>
       <c r="K385" s="8" t="n">
         <v>65</v>
@@ -18785,7 +18785,7 @@
         <v>78</v>
       </c>
       <c r="J386" s="11" t="n">
-        <v>0.375</v>
+        <v>0.6022999999999999</v>
       </c>
       <c r="K386" s="8" t="n">
         <v>35</v>
@@ -18921,7 +18921,7 @@
         <v>140</v>
       </c>
       <c r="J389" s="7" t="n">
-        <v>0.6214</v>
+        <v>0.8998</v>
       </c>
       <c r="K389" s="5" t="n">
         <v>69</v>
@@ -18969,7 +18969,7 @@
         <v>10</v>
       </c>
       <c r="J390" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K390" s="8" t="n">
         <v>5</v>
@@ -19017,7 +19017,7 @@
         <v>10</v>
       </c>
       <c r="J391" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K391" s="8" t="n">
         <v>5</v>
@@ -19065,7 +19065,7 @@
         <v>40</v>
       </c>
       <c r="J392" s="11" t="n">
-        <v>0.4</v>
+        <v>0.875</v>
       </c>
       <c r="K392" s="8" t="n">
         <v>19</v>
@@ -19161,7 +19161,7 @@
         <v>60</v>
       </c>
       <c r="J394" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9495</v>
       </c>
       <c r="K394" s="8" t="n">
         <v>30</v>
@@ -19205,7 +19205,7 @@
         <v>612</v>
       </c>
       <c r="J395" s="7" t="n">
-        <v>0.4672</v>
+        <v>0.8331</v>
       </c>
       <c r="K395" s="5" t="n">
         <v>305</v>
@@ -19253,7 +19253,7 @@
         <v>50</v>
       </c>
       <c r="J396" s="11" t="n">
-        <v>0.2857</v>
+        <v>0.72</v>
       </c>
       <c r="K396" s="8" t="n">
         <v>25</v>
@@ -19349,7 +19349,7 @@
         <v>152</v>
       </c>
       <c r="J398" s="11" t="n">
-        <v>0.8333</v>
+        <v>0.835</v>
       </c>
       <c r="K398" s="8" t="n">
         <v>80</v>
@@ -19445,7 +19445,7 @@
         <v>10</v>
       </c>
       <c r="J400" s="11" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="K400" s="8" t="n">
         <v>5</v>
@@ -19493,7 +19493,7 @@
         <v>10</v>
       </c>
       <c r="J401" s="11" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K401" s="8" t="n">
         <v>5</v>
@@ -19541,7 +19541,7 @@
         <v>180</v>
       </c>
       <c r="J402" s="11" t="n">
-        <v>0.1277</v>
+        <v>0.8607</v>
       </c>
       <c r="K402" s="8" t="n">
         <v>90</v>
@@ -19589,7 +19589,7 @@
         <v>100</v>
       </c>
       <c r="J403" s="11" t="n">
-        <v>0.34</v>
+        <v>0.89</v>
       </c>
       <c r="K403" s="8" t="n">
         <v>50</v>
@@ -19681,7 +19681,7 @@
         <v>240</v>
       </c>
       <c r="J405" s="7" t="n">
-        <v>0.4354</v>
+        <v>0.9789</v>
       </c>
       <c r="K405" s="5" t="n">
         <v>120</v>
@@ -19729,7 +19729,7 @@
         <v>11</v>
       </c>
       <c r="J406" s="11" t="n">
-        <v>0</v>
+        <v>0.9999</v>
       </c>
       <c r="K406" s="8" t="n">
         <v>5</v>
@@ -19777,7 +19777,7 @@
         <v>50</v>
       </c>
       <c r="J407" s="11" t="n">
-        <v>0.54</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K407" s="8" t="n">
         <v>25</v>
@@ -19825,7 +19825,7 @@
         <v>10</v>
       </c>
       <c r="J408" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K408" s="8" t="n">
         <v>5</v>
@@ -19873,7 +19873,7 @@
         <v>30</v>
       </c>
       <c r="J409" s="11" t="n">
-        <v>0.6333</v>
+        <v>0.9663</v>
       </c>
       <c r="K409" s="8" t="n">
         <v>15</v>
@@ -19921,7 +19921,7 @@
         <v>20</v>
       </c>
       <c r="J410" s="11" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K410" s="8" t="n">
         <v>10</v>
@@ -19969,7 +19969,7 @@
         <v>59</v>
       </c>
       <c r="J411" s="11" t="n">
-        <v>0.5</v>
+        <v>0.9993</v>
       </c>
       <c r="K411" s="8" t="n">
         <v>30</v>
@@ -20017,7 +20017,7 @@
         <v>60</v>
       </c>
       <c r="J412" s="11" t="n">
-        <v>0.3166</v>
+        <v>0.9831</v>
       </c>
       <c r="K412" s="8" t="n">
         <v>30</v>
@@ -20061,7 +20061,7 @@
         <v>1163</v>
       </c>
       <c r="J413" s="7" t="n">
-        <v>0.4641</v>
+        <v>0.7813</v>
       </c>
       <c r="K413" s="5" t="n">
         <v>598</v>
@@ -20109,7 +20109,7 @@
         <v>49</v>
       </c>
       <c r="J414" s="11" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.7548</v>
       </c>
       <c r="K414" s="8" t="n">
         <v>25</v>
@@ -20157,7 +20157,7 @@
         <v>60</v>
       </c>
       <c r="J415" s="11" t="n">
-        <v>0.15</v>
+        <v>0.6329</v>
       </c>
       <c r="K415" s="8" t="n">
         <v>25</v>
@@ -20205,7 +20205,7 @@
         <v>20</v>
       </c>
       <c r="J416" s="11" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="K416" s="8" t="n">
         <v>10</v>
@@ -20253,7 +20253,7 @@
         <v>20</v>
       </c>
       <c r="J417" s="11" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="K417" s="8" t="n">
         <v>10</v>
@@ -20301,7 +20301,7 @@
         <v>139</v>
       </c>
       <c r="J418" s="11" t="n">
-        <v>0.6928</v>
+        <v>0.6903</v>
       </c>
       <c r="K418" s="8" t="n">
         <v>65</v>
@@ -20349,7 +20349,7 @@
         <v>120</v>
       </c>
       <c r="J419" s="11" t="n">
-        <v>0.7416</v>
+        <v>0.7329</v>
       </c>
       <c r="K419" s="8" t="n">
         <v>64</v>
@@ -20397,7 +20397,7 @@
         <v>19</v>
       </c>
       <c r="J420" s="11" t="n">
-        <v>0.85</v>
+        <v>0.8945</v>
       </c>
       <c r="K420" s="8" t="n">
         <v>10</v>
@@ -20445,7 +20445,7 @@
         <v>100</v>
       </c>
       <c r="J421" s="11" t="n">
-        <v>0.38</v>
+        <v>0.65</v>
       </c>
       <c r="K421" s="8" t="n">
         <v>55</v>
@@ -20493,7 +20493,7 @@
         <v>50</v>
       </c>
       <c r="J422" s="11" t="n">
-        <v>0</v>
+        <v>0.86</v>
       </c>
       <c r="K422" s="8" t="n">
         <v>25</v>
@@ -20541,7 +20541,7 @@
         <v>120</v>
       </c>
       <c r="J423" s="11" t="n">
-        <v>0.6333</v>
+        <v>0.8915999999999999</v>
       </c>
       <c r="K423" s="8" t="n">
         <v>65</v>
@@ -20589,7 +20589,7 @@
         <v>50</v>
       </c>
       <c r="J424" s="11" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K424" s="8" t="n">
         <v>25</v>
@@ -20637,7 +20637,7 @@
         <v>59</v>
       </c>
       <c r="J425" s="11" t="n">
-        <v>0.4166</v>
+        <v>0.6606</v>
       </c>
       <c r="K425" s="8" t="n">
         <v>25</v>
@@ -20685,7 +20685,7 @@
         <v>119</v>
       </c>
       <c r="J426" s="11" t="n">
-        <v>0.6583</v>
+        <v>0.8905</v>
       </c>
       <c r="K426" s="8" t="n">
         <v>60</v>
@@ -20733,7 +20733,7 @@
         <v>30</v>
       </c>
       <c r="J427" s="11" t="n">
-        <v>0.9</v>
+        <v>0.8996</v>
       </c>
       <c r="K427" s="8" t="n">
         <v>20</v>
@@ -20781,7 +20781,7 @@
         <v>91</v>
       </c>
       <c r="J428" s="11" t="n">
-        <v>0.2333</v>
+        <v>0.8238</v>
       </c>
       <c r="K428" s="8" t="n">
         <v>45</v>
@@ -20829,7 +20829,7 @@
         <v>117</v>
       </c>
       <c r="J429" s="11" t="n">
-        <v>0.2285</v>
+        <v>0.8371</v>
       </c>
       <c r="K429" s="8" t="n">
         <v>69</v>
@@ -20873,7 +20873,7 @@
         <v>430</v>
       </c>
       <c r="J430" s="7" t="n">
-        <v>0.8242</v>
+        <v>0.8343</v>
       </c>
       <c r="K430" s="5" t="n">
         <v>201</v>
@@ -20921,7 +20921,7 @@
         <v>190</v>
       </c>
       <c r="J431" s="11" t="n">
-        <v>0.7947</v>
+        <v>0.7995</v>
       </c>
       <c r="K431" s="8" t="n">
         <v>90</v>
@@ -20969,7 +20969,7 @@
         <v>230</v>
       </c>
       <c r="J432" s="11" t="n">
-        <v>0.8583</v>
+        <v>0.8732</v>
       </c>
       <c r="K432" s="8" t="n">
         <v>106</v>
@@ -21061,7 +21061,7 @@
         <v>49</v>
       </c>
       <c r="J434" s="7" t="n">
-        <v>0.9</v>
+        <v>0.8976</v>
       </c>
       <c r="K434" s="5" t="n">
         <v>35</v>
@@ -21109,7 +21109,7 @@
         <v>49</v>
       </c>
       <c r="J435" s="11" t="n">
-        <v>0.9</v>
+        <v>0.8976</v>
       </c>
       <c r="K435" s="8" t="n">
         <v>35</v>
@@ -21153,7 +21153,7 @@
         <v>100</v>
       </c>
       <c r="J436" s="7" t="n">
-        <v>0.7199</v>
+        <v>0.7296</v>
       </c>
       <c r="K436" s="5" t="n">
         <v>50</v>
@@ -21249,7 +21249,7 @@
         <v>90</v>
       </c>
       <c r="J438" s="11" t="n">
-        <v>0.6888</v>
+        <v>0.6996</v>
       </c>
       <c r="K438" s="8" t="n">
         <v>45</v>
@@ -21293,7 +21293,7 @@
         <v>51</v>
       </c>
       <c r="J439" s="7" t="n">
-        <v>0.7598</v>
+        <v>0.7645999999999999</v>
       </c>
       <c r="K439" s="5" t="n">
         <v>20</v>
@@ -21389,7 +21389,7 @@
         <v>21</v>
       </c>
       <c r="J441" s="11" t="n">
-        <v>0.75</v>
+        <v>0.7616000000000001</v>
       </c>
       <c r="K441" s="8" t="n">
         <v>5</v>
@@ -21545,7 +21545,7 @@
         <v>30</v>
       </c>
       <c r="J445" s="7" t="n">
-        <v>0.7665999999999999</v>
+        <v>0.7664</v>
       </c>
       <c r="K445" s="5" t="n">
         <v>10</v>
@@ -21593,7 +21593,7 @@
         <v>30</v>
       </c>
       <c r="J446" s="11" t="n">
-        <v>0.7665999999999999</v>
+        <v>0.7664</v>
       </c>
       <c r="K446" s="8" t="n">
         <v>10</v>
@@ -21669,7 +21669,7 @@
         <v>41</v>
       </c>
       <c r="J448" s="7" t="n">
-        <v>1</v>
+        <v>0.9996</v>
       </c>
       <c r="K448" s="5" t="n">
         <v>15</v>
@@ -21717,7 +21717,7 @@
         <v>41</v>
       </c>
       <c r="J449" s="11" t="n">
-        <v>1</v>
+        <v>0.9996</v>
       </c>
       <c r="K449" s="8" t="n">
         <v>15</v>
@@ -21889,7 +21889,7 @@
         <v>958</v>
       </c>
       <c r="J453" s="4" t="n">
-        <v>0.7929</v>
+        <v>0.9516</v>
       </c>
       <c r="K453" s="2" t="n">
         <v>495</v>
@@ -21933,7 +21933,7 @@
         <v>20</v>
       </c>
       <c r="J454" s="7" t="n">
-        <v>0.45</v>
+        <v>0.95</v>
       </c>
       <c r="K454" s="5" t="n">
         <v>10</v>
@@ -21981,7 +21981,7 @@
         <v>10</v>
       </c>
       <c r="J455" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K455" s="8" t="n">
         <v>5</v>
@@ -22073,7 +22073,7 @@
         <v>149</v>
       </c>
       <c r="J457" s="7" t="n">
-        <v>0.8399</v>
+        <v>0.9796</v>
       </c>
       <c r="K457" s="5" t="n">
         <v>85</v>
@@ -22169,7 +22169,7 @@
         <v>10</v>
       </c>
       <c r="J459" s="11" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="K459" s="8" t="n">
         <v>5</v>
@@ -22265,7 +22265,7 @@
         <v>10</v>
       </c>
       <c r="J461" s="11" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="K461" s="8" t="n">
         <v>5</v>
@@ -22361,7 +22361,7 @@
         <v>60</v>
       </c>
       <c r="J463" s="11" t="n">
-        <v>0.9857</v>
+        <v>0.9828</v>
       </c>
       <c r="K463" s="8" t="n">
         <v>35</v>
@@ -22505,7 +22505,7 @@
         <v>10</v>
       </c>
       <c r="J466" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K466" s="8" t="n">
         <v>5</v>
@@ -22553,7 +22553,7 @@
         <v>9</v>
       </c>
       <c r="J467" s="11" t="n">
-        <v>1</v>
+        <v>0.9999</v>
       </c>
       <c r="K467" s="8" t="n">
         <v>5</v>
@@ -22597,7 +22597,7 @@
         <v>439</v>
       </c>
       <c r="J468" s="7" t="n">
-        <v>0.7232</v>
+        <v>0.9678</v>
       </c>
       <c r="K468" s="5" t="n">
         <v>225</v>
@@ -22645,7 +22645,7 @@
         <v>30</v>
       </c>
       <c r="J469" s="11" t="n">
-        <v>1</v>
+        <v>0.9997</v>
       </c>
       <c r="K469" s="8" t="n">
         <v>15</v>
@@ -22693,7 +22693,7 @@
         <v>9</v>
       </c>
       <c r="J470" s="11" t="n">
-        <v>0</v>
+        <v>0.8888</v>
       </c>
       <c r="K470" s="8" t="n">
         <v>5</v>
@@ -22741,7 +22741,7 @@
         <v>40</v>
       </c>
       <c r="J471" s="11" t="n">
-        <v>0.475</v>
+        <v>0.975</v>
       </c>
       <c r="K471" s="8" t="n">
         <v>20</v>
@@ -22789,7 +22789,7 @@
         <v>30</v>
       </c>
       <c r="J472" s="11" t="n">
-        <v>0.6</v>
+        <v>0.9332</v>
       </c>
       <c r="K472" s="8" t="n">
         <v>15</v>
@@ -22837,7 +22837,7 @@
         <v>70</v>
       </c>
       <c r="J473" s="11" t="n">
-        <v>0.9142</v>
+        <v>0.9135</v>
       </c>
       <c r="K473" s="8" t="n">
         <v>35</v>
@@ -22933,7 +22933,7 @@
         <v>10</v>
       </c>
       <c r="J475" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="K475" s="8" t="n">
         <v>5</v>
@@ -23029,7 +23029,7 @@
         <v>90</v>
       </c>
       <c r="J477" s="11" t="n">
-        <v>0.9666</v>
+        <v>0.9661</v>
       </c>
       <c r="K477" s="8" t="n">
         <v>45</v>
@@ -23077,7 +23077,7 @@
         <v>50</v>
       </c>
       <c r="J478" s="11" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="K478" s="8" t="n">
         <v>25</v>
@@ -23125,7 +23125,7 @@
         <v>30</v>
       </c>
       <c r="J479" s="11" t="n">
-        <v>0.6666</v>
+        <v>0.9997</v>
       </c>
       <c r="K479" s="8" t="n">
         <v>15</v>
@@ -23173,7 +23173,7 @@
         <v>30</v>
       </c>
       <c r="J480" s="11" t="n">
-        <v>0.3333</v>
+        <v>0.9998</v>
       </c>
       <c r="K480" s="8" t="n">
         <v>15</v>
@@ -23217,7 +23217,7 @@
         <v>160</v>
       </c>
       <c r="J481" s="7" t="n">
-        <v>0.8187</v>
+        <v>0.9059</v>
       </c>
       <c r="K481" s="5" t="n">
         <v>80</v>
@@ -23265,7 +23265,7 @@
         <v>30</v>
       </c>
       <c r="J482" s="11" t="n">
-        <v>1</v>
+        <v>0.9997</v>
       </c>
       <c r="K482" s="8" t="n">
         <v>15</v>
@@ -23313,7 +23313,7 @@
         <v>130</v>
       </c>
       <c r="J483" s="11" t="n">
-        <v>0.7769</v>
+        <v>0.8842</v>
       </c>
       <c r="K483" s="8" t="n">
         <v>65</v>
@@ -23449,7 +23449,7 @@
         <v>30</v>
       </c>
       <c r="J486" s="7" t="n">
-        <v>0.8333</v>
+        <v>0.833</v>
       </c>
       <c r="K486" s="5" t="n">
         <v>15</v>
@@ -23497,7 +23497,7 @@
         <v>30</v>
       </c>
       <c r="J487" s="11" t="n">
-        <v>0.8333</v>
+        <v>0.833</v>
       </c>
       <c r="K487" s="8" t="n">
         <v>15</v>
@@ -23541,7 +23541,7 @@
         <v>110</v>
       </c>
       <c r="J488" s="7" t="n">
-        <v>0.9545</v>
+        <v>0.9537</v>
       </c>
       <c r="K488" s="5" t="n">
         <v>55</v>
@@ -23589,7 +23589,7 @@
         <v>110</v>
       </c>
       <c r="J489" s="11" t="n">
-        <v>0.9545</v>
+        <v>0.9537</v>
       </c>
       <c r="K489" s="8" t="n">
         <v>55</v>
@@ -23637,7 +23637,7 @@
         <v>473</v>
       </c>
       <c r="J490" s="4" t="n">
-        <v>0.8908</v>
+        <v>0.9532</v>
       </c>
       <c r="K490" s="2" t="n">
         <v>245</v>
@@ -23681,7 +23681,7 @@
         <v>10</v>
       </c>
       <c r="J491" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K491" s="5" t="n">
         <v>5</v>
@@ -23729,7 +23729,7 @@
         <v>10</v>
       </c>
       <c r="J492" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K492" s="8" t="n">
         <v>5</v>
@@ -23865,7 +23865,7 @@
         <v>443</v>
       </c>
       <c r="J495" s="7" t="n">
-        <v>0.9059</v>
+        <v>0.95</v>
       </c>
       <c r="K495" s="5" t="n">
         <v>230</v>
@@ -23961,7 +23961,7 @@
         <v>59</v>
       </c>
       <c r="J497" s="11" t="n">
-        <v>0.5</v>
+        <v>0.847</v>
       </c>
       <c r="K497" s="8" t="n">
         <v>30</v>
@@ -24009,7 +24009,7 @@
         <v>50</v>
       </c>
       <c r="J498" s="11" t="n">
-        <v>0.8367</v>
+        <v>0.82</v>
       </c>
       <c r="K498" s="8" t="n">
         <v>20</v>
@@ -24105,7 +24105,7 @@
         <v>60</v>
       </c>
       <c r="J500" s="11" t="n">
-        <v>0.9833</v>
+        <v>0.983</v>
       </c>
       <c r="K500" s="8" t="n">
         <v>30</v>
@@ -24153,7 +24153,7 @@
         <v>15</v>
       </c>
       <c r="J501" s="11" t="n">
-        <v>1</v>
+        <v>0.9997</v>
       </c>
       <c r="K501" s="8" t="n">
         <v>15</v>
@@ -24249,7 +24249,7 @@
         <v>59</v>
       </c>
       <c r="J503" s="11" t="n">
-        <v>1</v>
+        <v>0.9994</v>
       </c>
       <c r="K503" s="8" t="n">
         <v>30</v>
@@ -24345,7 +24345,7 @@
         <v>70</v>
       </c>
       <c r="J505" s="11" t="n">
-        <v>1</v>
+        <v>0.9993</v>
       </c>
       <c r="K505" s="8" t="n">
         <v>35</v>
@@ -24393,7 +24393,7 @@
         <v>1851</v>
       </c>
       <c r="J506" s="4" t="n">
-        <v>0.6777</v>
+        <v>0.8333</v>
       </c>
       <c r="K506" s="2" t="n">
         <v>903</v>
@@ -24437,7 +24437,7 @@
         <v>75</v>
       </c>
       <c r="J507" s="7" t="n">
-        <v>0.7060999999999999</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="K507" s="5" t="n">
         <v>35</v>
@@ -24581,7 +24581,7 @@
         <v>15</v>
       </c>
       <c r="J510" s="11" t="n">
-        <v>0.2307</v>
+        <v>0.3999</v>
       </c>
       <c r="K510" s="8" t="n">
         <v>5</v>
@@ -24629,7 +24629,7 @@
         <v>20</v>
       </c>
       <c r="J511" s="11" t="n">
-        <v>0.525</v>
+        <v>0.95</v>
       </c>
       <c r="K511" s="8" t="n">
         <v>10</v>
@@ -24673,7 +24673,7 @@
         <v>63</v>
       </c>
       <c r="J512" s="7" t="n">
-        <v>0.9166</v>
+        <v>0.9201</v>
       </c>
       <c r="K512" s="5" t="n">
         <v>30</v>
@@ -24721,7 +24721,7 @@
         <v>63</v>
       </c>
       <c r="J513" s="11" t="n">
-        <v>0.9166</v>
+        <v>0.9201</v>
       </c>
       <c r="K513" s="8" t="n">
         <v>30</v>
@@ -24765,7 +24765,7 @@
         <v>528</v>
       </c>
       <c r="J514" s="7" t="n">
-        <v>0.8032</v>
+        <v>0.8576</v>
       </c>
       <c r="K514" s="5" t="n">
         <v>265</v>
@@ -24813,7 +24813,7 @@
         <v>189</v>
       </c>
       <c r="J515" s="11" t="n">
-        <v>0.921</v>
+        <v>0.92</v>
       </c>
       <c r="K515" s="8" t="n">
         <v>100</v>
@@ -24909,7 +24909,7 @@
         <v>49</v>
       </c>
       <c r="J517" s="11" t="n">
-        <v>0.96</v>
+        <v>0.9589</v>
       </c>
       <c r="K517" s="8" t="n">
         <v>25</v>
@@ -24957,7 +24957,7 @@
         <v>150</v>
       </c>
       <c r="J518" s="11" t="n">
-        <v>0.6666</v>
+        <v>0.7331</v>
       </c>
       <c r="K518" s="8" t="n">
         <v>75</v>
@@ -25005,7 +25005,7 @@
         <v>120</v>
       </c>
       <c r="J519" s="11" t="n">
-        <v>0.7083</v>
+        <v>0.8666</v>
       </c>
       <c r="K519" s="8" t="n">
         <v>55</v>
@@ -25081,7 +25081,7 @@
         <v>346</v>
       </c>
       <c r="J521" s="7" t="n">
-        <v>0.3595</v>
+        <v>0.8321</v>
       </c>
       <c r="K521" s="5" t="n">
         <v>170</v>
@@ -25129,7 +25129,7 @@
         <v>50</v>
       </c>
       <c r="J522" s="11" t="n">
-        <v>0.4</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K522" s="8" t="n">
         <v>25</v>
@@ -25177,7 +25177,7 @@
         <v>10</v>
       </c>
       <c r="J523" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K523" s="8" t="n">
         <v>5</v>
@@ -25225,7 +25225,7 @@
         <v>20</v>
       </c>
       <c r="J524" s="11" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="K524" s="8" t="n">
         <v>10</v>
@@ -25273,7 +25273,7 @@
         <v>261</v>
       </c>
       <c r="J525" s="11" t="n">
-        <v>0.4</v>
+        <v>0.8004</v>
       </c>
       <c r="K525" s="8" t="n">
         <v>125</v>
@@ -25321,7 +25321,7 @@
         <v>5</v>
       </c>
       <c r="J526" s="11" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K526" s="8" t="n">
         <v>5</v>
@@ -25365,7 +25365,7 @@
         <v>139</v>
       </c>
       <c r="J527" s="7" t="n">
-        <v>0.8358</v>
+        <v>0.8484</v>
       </c>
       <c r="K527" s="5" t="n">
         <v>70</v>
@@ -25413,7 +25413,7 @@
         <v>70</v>
       </c>
       <c r="J528" s="11" t="n">
-        <v>0.8571</v>
+        <v>0.8567</v>
       </c>
       <c r="K528" s="8" t="n">
         <v>35</v>
@@ -25461,7 +25461,7 @@
         <v>69</v>
       </c>
       <c r="J529" s="11" t="n">
-        <v>0.8142</v>
+        <v>0.84</v>
       </c>
       <c r="K529" s="8" t="n">
         <v>35</v>
@@ -25505,7 +25505,7 @@
         <v>20</v>
       </c>
       <c r="J530" s="7" t="n">
-        <v>0.45</v>
+        <v>0.9</v>
       </c>
       <c r="K530" s="5" t="n">
         <v>10</v>
@@ -25553,7 +25553,7 @@
         <v>20</v>
       </c>
       <c r="J531" s="11" t="n">
-        <v>0.45</v>
+        <v>0.9</v>
       </c>
       <c r="K531" s="8" t="n">
         <v>10</v>
@@ -25677,7 +25677,7 @@
         <v>80</v>
       </c>
       <c r="J534" s="7" t="n">
-        <v>0.8375</v>
+        <v>0.8373</v>
       </c>
       <c r="K534" s="5" t="n">
         <v>38</v>
@@ -25725,7 +25725,7 @@
         <v>60</v>
       </c>
       <c r="J535" s="11" t="n">
-        <v>0.8833</v>
+        <v>0.8831</v>
       </c>
       <c r="K535" s="8" t="n">
         <v>28</v>
@@ -25817,7 +25817,7 @@
         <v>410</v>
       </c>
       <c r="J537" s="7" t="n">
-        <v>0.8683</v>
+        <v>0.8754</v>
       </c>
       <c r="K537" s="5" t="n">
         <v>200</v>
@@ -25865,7 +25865,7 @@
         <v>90</v>
       </c>
       <c r="J538" s="11" t="n">
-        <v>0.8333</v>
+        <v>0.8331</v>
       </c>
       <c r="K538" s="8" t="n">
         <v>40</v>
@@ -25913,7 +25913,7 @@
         <v>51</v>
       </c>
       <c r="J539" s="11" t="n">
-        <v>0.82</v>
+        <v>0.8233</v>
       </c>
       <c r="K539" s="8" t="n">
         <v>25</v>
@@ -25961,7 +25961,7 @@
         <v>49</v>
       </c>
       <c r="J540" s="11" t="n">
-        <v>0.8</v>
+        <v>0.9996</v>
       </c>
       <c r="K540" s="8" t="n">
         <v>25</v>
@@ -26009,7 +26009,7 @@
         <v>30</v>
       </c>
       <c r="J541" s="11" t="n">
-        <v>1</v>
+        <v>0.9999</v>
       </c>
       <c r="K541" s="8" t="n">
         <v>15</v>
@@ -26105,7 +26105,7 @@
         <v>90</v>
       </c>
       <c r="J543" s="11" t="n">
-        <v>0.9444</v>
+        <v>0.9442</v>
       </c>
       <c r="K543" s="8" t="n">
         <v>45</v>
@@ -26249,7 +26249,7 @@
         <v>10</v>
       </c>
       <c r="J546" s="11" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K546" s="8" t="n">
         <v>5</v>
@@ -26293,7 +26293,7 @@
         <v>180</v>
       </c>
       <c r="J547" s="7" t="n">
-        <v>0.2222</v>
+        <v>0.6166</v>
       </c>
       <c r="K547" s="5" t="n">
         <v>85</v>
@@ -26341,7 +26341,7 @@
         <v>10</v>
       </c>
       <c r="J548" s="11" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="K548" s="8" t="n">
         <v>5</v>
@@ -26389,7 +26389,7 @@
         <v>70</v>
       </c>
       <c r="J549" s="11" t="n">
-        <v>0.2142</v>
+        <v>0.4713</v>
       </c>
       <c r="K549" s="8" t="n">
         <v>30</v>
@@ -26437,7 +26437,7 @@
         <v>100</v>
       </c>
       <c r="J550" s="11" t="n">
-        <v>0.23</v>
+        <v>0.75</v>
       </c>
       <c r="K550" s="8" t="n">
         <v>50</v>
@@ -26485,7 +26485,7 @@
         <v>3175</v>
       </c>
       <c r="J551" s="4" t="n">
-        <v>0.4828</v>
+        <v>0.9066</v>
       </c>
       <c r="K551" s="2" t="n">
         <v>929</v>
@@ -26529,7 +26529,7 @@
         <v>917</v>
       </c>
       <c r="J552" s="7" t="n">
-        <v>0.1352</v>
+        <v>0.9167999999999999</v>
       </c>
       <c r="K552" s="5" t="n">
         <v>225</v>
@@ -26577,7 +26577,7 @@
         <v>60</v>
       </c>
       <c r="J553" s="11" t="n">
-        <v>0</v>
+        <v>0.983</v>
       </c>
       <c r="K553" s="8" t="n">
         <v>15</v>
@@ -26721,7 +26721,7 @@
         <v>60</v>
       </c>
       <c r="J556" s="11" t="n">
-        <v>1</v>
+        <v>0.9664</v>
       </c>
       <c r="K556" s="8" t="n">
         <v>15</v>
@@ -26769,7 +26769,7 @@
         <v>80</v>
       </c>
       <c r="J557" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K557" s="8" t="n">
         <v>20</v>
@@ -26817,7 +26817,7 @@
         <v>260</v>
       </c>
       <c r="J558" s="11" t="n">
-        <v>0</v>
+        <v>0.9532</v>
       </c>
       <c r="K558" s="8" t="n">
         <v>65</v>
@@ -26865,7 +26865,7 @@
         <v>200</v>
       </c>
       <c r="J559" s="11" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="K559" s="8" t="n">
         <v>50</v>
@@ -26913,7 +26913,7 @@
         <v>20</v>
       </c>
       <c r="J560" s="11" t="n">
-        <v>0</v>
+        <v>0.55</v>
       </c>
       <c r="K560" s="8" t="n">
         <v>0</v>
@@ -26955,7 +26955,7 @@
         <v>59</v>
       </c>
       <c r="J561" s="11" t="n">
-        <v>0</v>
+        <v>0.9488</v>
       </c>
       <c r="K561" s="8" t="n">
         <v>15</v>
@@ -27003,7 +27003,7 @@
         <v>98</v>
       </c>
       <c r="J562" s="11" t="n">
-        <v>0</v>
+        <v>0.8671</v>
       </c>
       <c r="K562" s="8" t="n">
         <v>25</v>
@@ -27047,7 +27047,7 @@
         <v>79</v>
       </c>
       <c r="J563" s="7" t="n">
-        <v>0.9</v>
+        <v>0.9743000000000001</v>
       </c>
       <c r="K563" s="5" t="n">
         <v>20</v>
@@ -27095,7 +27095,7 @@
         <v>79</v>
       </c>
       <c r="J564" s="11" t="n">
-        <v>0.9</v>
+        <v>0.9743000000000001</v>
       </c>
       <c r="K564" s="8" t="n">
         <v>20</v>
@@ -27139,7 +27139,7 @@
         <v>2179</v>
       </c>
       <c r="J565" s="7" t="n">
-        <v>0.6139</v>
+        <v>0.8998</v>
       </c>
       <c r="K565" s="5" t="n">
         <v>684</v>
@@ -27187,7 +27187,7 @@
         <v>180</v>
       </c>
       <c r="J566" s="11" t="n">
-        <v>0</v>
+        <v>0.905</v>
       </c>
       <c r="K566" s="8" t="n">
         <v>45</v>
@@ -27235,7 +27235,7 @@
         <v>160</v>
       </c>
       <c r="J567" s="11" t="n">
-        <v>0</v>
+        <v>0.9247</v>
       </c>
       <c r="K567" s="8" t="n">
         <v>40</v>
@@ -27331,7 +27331,7 @@
         <v>179</v>
       </c>
       <c r="J569" s="11" t="n">
-        <v>0.8944</v>
+        <v>0.8931</v>
       </c>
       <c r="K569" s="8" t="n">
         <v>45</v>
@@ -27379,7 +27379,7 @@
         <v>120</v>
       </c>
       <c r="J570" s="11" t="n">
-        <v>0.9333</v>
+        <v>0.9331</v>
       </c>
       <c r="K570" s="8" t="n">
         <v>30</v>
@@ -27427,7 +27427,7 @@
         <v>120</v>
       </c>
       <c r="J571" s="11" t="n">
-        <v>0.7083</v>
+        <v>0.8164</v>
       </c>
       <c r="K571" s="8" t="n">
         <v>30</v>
@@ -27475,7 +27475,7 @@
         <v>141</v>
       </c>
       <c r="J572" s="11" t="n">
-        <v>0.9214</v>
+        <v>0.9213</v>
       </c>
       <c r="K572" s="8" t="n">
         <v>35</v>
@@ -27609,7 +27609,7 @@
         <v>40</v>
       </c>
       <c r="J575" s="11" t="n">
-        <v>0</v>
+        <v>0.775</v>
       </c>
       <c r="K575" s="8" t="n">
         <v>20</v>
@@ -27657,7 +27657,7 @@
         <v>100</v>
       </c>
       <c r="J576" s="11" t="n">
-        <v>0</v>
+        <v>0.7938</v>
       </c>
       <c r="K576" s="8" t="n">
         <v>144</v>
@@ -27705,7 +27705,7 @@
         <v>140</v>
       </c>
       <c r="J577" s="11" t="n">
-        <v>0</v>
+        <v>0.9137999999999999</v>
       </c>
       <c r="K577" s="8" t="n">
         <v>30</v>
@@ -27753,7 +27753,7 @@
         <v>99</v>
       </c>
       <c r="J578" s="11" t="n">
-        <v>0.9416</v>
+        <v>0.9393</v>
       </c>
       <c r="K578" s="8" t="n">
         <v>30</v>
@@ -27801,7 +27801,7 @@
         <v>180</v>
       </c>
       <c r="J579" s="11" t="n">
-        <v>0.8555</v>
+        <v>0.8552999999999999</v>
       </c>
       <c r="K579" s="8" t="n">
         <v>45</v>
@@ -27849,7 +27849,7 @@
         <v>120</v>
       </c>
       <c r="J580" s="11" t="n">
-        <v>0.925</v>
+        <v>0.9247</v>
       </c>
       <c r="K580" s="8" t="n">
         <v>30</v>
@@ -27897,7 +27897,7 @@
         <v>100</v>
       </c>
       <c r="J581" s="11" t="n">
-        <v>0.9555</v>
+        <v>0.96</v>
       </c>
       <c r="K581" s="8" t="n">
         <v>25</v>
@@ -27945,7 +27945,7 @@
         <v>220</v>
       </c>
       <c r="J582" s="11" t="n">
-        <v>0.9666</v>
+        <v>0.9675</v>
       </c>
       <c r="K582" s="8" t="n">
         <v>55</v>
@@ -27993,7 +27993,7 @@
         <v>20</v>
       </c>
       <c r="J583" s="11" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="K583" s="8" t="n">
         <v>5</v>
@@ -28041,7 +28041,7 @@
         <v>200</v>
       </c>
       <c r="J584" s="11" t="n">
-        <v>0.6712</v>
+        <v>0.885</v>
       </c>
       <c r="K584" s="8" t="n">
         <v>55</v>
@@ -28129,7 +28129,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>% &gt; 12 °Brix</t>
+          <t>% ≥ 12 °Brix</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -28181,7 +28181,7 @@
         <v>95</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.6947</v>
+        <v>0.6943</v>
       </c>
       <c r="J2" s="8" t="n">
         <v>45</v>
@@ -28224,7 +28224,7 @@
         <v>165</v>
       </c>
       <c r="I3" s="14" t="n">
-        <v>0.3999</v>
+        <v>0.6906</v>
       </c>
       <c r="J3" s="12" t="n">
         <v>80</v>
@@ -28267,7 +28267,7 @@
         <v>664</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.8488</v>
+        <v>0.8431</v>
       </c>
       <c r="J4" s="8" t="n">
         <v>319</v>
@@ -28310,7 +28310,7 @@
         <v>1290</v>
       </c>
       <c r="I5" s="14" t="n">
-        <v>0.5151</v>
+        <v>0.7485000000000001</v>
       </c>
       <c r="J5" s="12" t="n">
         <v>580</v>
@@ -28353,7 +28353,7 @@
         <v>401</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.9002</v>
+        <v>0.8997000000000001</v>
       </c>
       <c r="J6" s="8" t="n">
         <v>194</v>
@@ -28396,7 +28396,7 @@
         <v>543</v>
       </c>
       <c r="I7" s="14" t="n">
-        <v>0.9391</v>
+        <v>0.9371</v>
       </c>
       <c r="J7" s="12" t="n">
         <v>264</v>
@@ -28439,7 +28439,7 @@
         <v>452</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.6704</v>
+        <v>0.6788</v>
       </c>
       <c r="J8" s="8" t="n">
         <v>214</v>
@@ -28482,7 +28482,7 @@
         <v>866</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>0.8578</v>
+        <v>0.8793</v>
       </c>
       <c r="J9" s="12" t="n">
         <v>400</v>
@@ -28525,7 +28525,7 @@
         <v>1000</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.475</v>
+        <v>0.7796999999999999</v>
       </c>
       <c r="J10" s="8" t="n">
         <v>460</v>
@@ -28568,7 +28568,7 @@
         <v>1000</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>0.6364</v>
+        <v>0.9386</v>
       </c>
       <c r="J11" s="12" t="n">
         <v>509</v>
@@ -28611,7 +28611,7 @@
         <v>155</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.8129</v>
+        <v>0.8127</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>75</v>
@@ -28654,7 +28654,7 @@
         <v>281</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>0.8925</v>
+        <v>0.8929</v>
       </c>
       <c r="J13" s="12" t="n">
         <v>135</v>
@@ -28697,7 +28697,7 @@
         <v>314</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.8328</v>
+        <v>0.834</v>
       </c>
       <c r="J14" s="8" t="n">
         <v>150</v>
@@ -28740,7 +28740,7 @@
         <v>30</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>0.6666</v>
+        <v>0.6663</v>
       </c>
       <c r="J15" s="12" t="n">
         <v>15</v>
@@ -28912,7 +28912,7 @@
         <v>81</v>
       </c>
       <c r="I19" s="14" t="n">
-        <v>0.8493000000000001</v>
+        <v>0.901</v>
       </c>
       <c r="J19" s="12" t="n">
         <v>34</v>
@@ -29041,7 +29041,7 @@
         <v>323</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>0.7879</v>
+        <v>0.7894</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>80</v>
@@ -29084,7 +29084,7 @@
         <v>1238</v>
       </c>
       <c r="I23" s="14" t="n">
-        <v>0.8418</v>
+        <v>0.8502</v>
       </c>
       <c r="J23" s="12" t="n">
         <v>305</v>
@@ -29127,7 +29127,7 @@
         <v>747</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>0.7712</v>
+        <v>0.7749</v>
       </c>
       <c r="J24" s="8" t="n">
         <v>170</v>
@@ -29170,7 +29170,7 @@
         <v>4126</v>
       </c>
       <c r="I25" s="14" t="n">
-        <v>0.5155999999999999</v>
+        <v>0.7825</v>
       </c>
       <c r="J25" s="12" t="n">
         <v>985</v>
@@ -29213,7 +29213,7 @@
         <v>219</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>0</v>
+        <v>0.9404</v>
       </c>
       <c r="J26" s="8" t="n">
         <v>55</v>
@@ -29256,7 +29256,7 @@
         <v>1200</v>
       </c>
       <c r="I27" s="14" t="n">
-        <v>0.7716</v>
+        <v>0.8599</v>
       </c>
       <c r="J27" s="12" t="n">
         <v>435</v>
@@ -29342,7 +29342,7 @@
         <v>200</v>
       </c>
       <c r="I29" s="14" t="n">
-        <v>0.8197</v>
+        <v>0.8192</v>
       </c>
       <c r="J29" s="12" t="n">
         <v>314</v>
@@ -29385,7 +29385,7 @@
         <v>60</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>0.7166</v>
+        <v>0.7163</v>
       </c>
       <c r="J30" s="8" t="n">
         <v>15</v>
@@ -29428,7 +29428,7 @@
         <v>20</v>
       </c>
       <c r="I31" s="14" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="J31" s="12" t="n">
         <v>5</v>
@@ -29471,7 +29471,7 @@
         <v>140</v>
       </c>
       <c r="I32" s="11" t="n">
-        <v>0.9308999999999999</v>
+        <v>0.9429</v>
       </c>
       <c r="J32" s="8" t="n">
         <v>35</v>
@@ -29514,7 +29514,7 @@
         <v>522</v>
       </c>
       <c r="I33" s="14" t="n">
-        <v>0.9096</v>
+        <v>0.9076</v>
       </c>
       <c r="J33" s="12" t="n">
         <v>130</v>
@@ -29557,7 +29557,7 @@
         <v>608</v>
       </c>
       <c r="I34" s="11" t="n">
-        <v>0.7508</v>
+        <v>0.7742</v>
       </c>
       <c r="J34" s="8" t="n">
         <v>135</v>
@@ -29600,7 +29600,7 @@
         <v>703</v>
       </c>
       <c r="I35" s="14" t="n">
-        <v>0.8763</v>
+        <v>0.8942</v>
       </c>
       <c r="J35" s="12" t="n">
         <v>160</v>
@@ -29643,7 +29643,7 @@
         <v>439</v>
       </c>
       <c r="I36" s="11" t="n">
-        <v>0.2632</v>
+        <v>0.7539</v>
       </c>
       <c r="J36" s="8" t="n">
         <v>134</v>
@@ -29686,7 +29686,7 @@
         <v>460</v>
       </c>
       <c r="I37" s="14" t="n">
-        <v>0.8421999999999999</v>
+        <v>0.8451</v>
       </c>
       <c r="J37" s="12" t="n">
         <v>120</v>
@@ -29729,7 +29729,7 @@
         <v>430</v>
       </c>
       <c r="I38" s="11" t="n">
-        <v>0.7983</v>
+        <v>0.8065</v>
       </c>
       <c r="J38" s="8" t="n">
         <v>99</v>
@@ -29815,7 +29815,7 @@
         <v>1842</v>
       </c>
       <c r="I40" s="11" t="n">
-        <v>0.8434</v>
+        <v>0.9550999999999999</v>
       </c>
       <c r="J40" s="8" t="n">
         <v>914</v>
@@ -29858,7 +29858,7 @@
         <v>660</v>
       </c>
       <c r="I41" s="14" t="n">
-        <v>0.2906</v>
+        <v>0.8695000000000001</v>
       </c>
       <c r="J41" s="12" t="n">
         <v>343</v>
@@ -29901,7 +29901,7 @@
         <v>1409</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>0.4896</v>
+        <v>0.9081</v>
       </c>
       <c r="J42" s="8" t="n">
         <v>697</v>
@@ -29944,7 +29944,7 @@
         <v>1475</v>
       </c>
       <c r="I43" s="14" t="n">
-        <v>0.9764</v>
+        <v>0.9772</v>
       </c>
       <c r="J43" s="12" t="n">
         <v>735</v>
@@ -29987,7 +29987,7 @@
         <v>411</v>
       </c>
       <c r="I44" s="11" t="n">
-        <v>0.6226</v>
+        <v>0.8731</v>
       </c>
       <c r="J44" s="8" t="n">
         <v>205</v>
@@ -30030,7 +30030,7 @@
         <v>1529</v>
       </c>
       <c r="I45" s="14" t="n">
-        <v>0.9622000000000001</v>
+        <v>0.959</v>
       </c>
       <c r="J45" s="12" t="n">
         <v>760</v>
@@ -30073,7 +30073,7 @@
         <v>69</v>
       </c>
       <c r="I46" s="11" t="n">
-        <v>1</v>
+        <v>0.9994</v>
       </c>
       <c r="J46" s="8" t="n">
         <v>35</v>
@@ -30159,7 +30159,7 @@
         <v>240</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>0.8833</v>
+        <v>0.9162</v>
       </c>
       <c r="J48" s="8" t="n">
         <v>125</v>
@@ -30202,7 +30202,7 @@
         <v>89</v>
       </c>
       <c r="I49" s="14" t="n">
-        <v>0.9111</v>
+        <v>0.9095</v>
       </c>
       <c r="J49" s="12" t="n">
         <v>45</v>
@@ -30245,7 +30245,7 @@
         <v>1314</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>0.7772</v>
+        <v>0.8405</v>
       </c>
       <c r="J50" s="8" t="n">
         <v>645</v>
@@ -30331,7 +30331,7 @@
         <v>140</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>0.6214</v>
+        <v>0.8998</v>
       </c>
       <c r="J52" s="8" t="n">
         <v>69</v>
@@ -30374,7 +30374,7 @@
         <v>612</v>
       </c>
       <c r="I53" s="14" t="n">
-        <v>0.4672</v>
+        <v>0.8331</v>
       </c>
       <c r="J53" s="12" t="n">
         <v>305</v>
@@ -30417,7 +30417,7 @@
         <v>240</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>0.4354</v>
+        <v>0.9789</v>
       </c>
       <c r="J54" s="8" t="n">
         <v>120</v>
@@ -30460,7 +30460,7 @@
         <v>1163</v>
       </c>
       <c r="I55" s="14" t="n">
-        <v>0.4641</v>
+        <v>0.7813</v>
       </c>
       <c r="J55" s="12" t="n">
         <v>598</v>
@@ -30503,7 +30503,7 @@
         <v>430</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>0.8242</v>
+        <v>0.8343</v>
       </c>
       <c r="J56" s="8" t="n">
         <v>201</v>
@@ -30546,7 +30546,7 @@
         <v>49</v>
       </c>
       <c r="I57" s="14" t="n">
-        <v>0.9</v>
+        <v>0.8976</v>
       </c>
       <c r="J57" s="12" t="n">
         <v>35</v>
@@ -30589,7 +30589,7 @@
         <v>100</v>
       </c>
       <c r="I58" s="11" t="n">
-        <v>0.7199</v>
+        <v>0.7296</v>
       </c>
       <c r="J58" s="8" t="n">
         <v>50</v>
@@ -30632,7 +30632,7 @@
         <v>51</v>
       </c>
       <c r="I59" s="14" t="n">
-        <v>0.7598</v>
+        <v>0.7645999999999999</v>
       </c>
       <c r="J59" s="12" t="n">
         <v>20</v>
@@ -30675,7 +30675,7 @@
         <v>30</v>
       </c>
       <c r="I60" s="11" t="n">
-        <v>0.7665999999999999</v>
+        <v>0.7664</v>
       </c>
       <c r="J60" s="8" t="n">
         <v>10</v>
@@ -30718,7 +30718,7 @@
         <v>41</v>
       </c>
       <c r="I61" s="14" t="n">
-        <v>1</v>
+        <v>0.9996</v>
       </c>
       <c r="J61" s="12" t="n">
         <v>15</v>
@@ -30804,7 +30804,7 @@
         <v>20</v>
       </c>
       <c r="I63" s="14" t="n">
-        <v>0.45</v>
+        <v>0.95</v>
       </c>
       <c r="J63" s="12" t="n">
         <v>10</v>
@@ -30847,7 +30847,7 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="n">
-        <v>0.8399</v>
+        <v>0.9796</v>
       </c>
       <c r="J64" s="8" t="n">
         <v>85</v>
@@ -30890,7 +30890,7 @@
         <v>439</v>
       </c>
       <c r="I65" s="14" t="n">
-        <v>0.7232</v>
+        <v>0.9678</v>
       </c>
       <c r="J65" s="12" t="n">
         <v>225</v>
@@ -30933,7 +30933,7 @@
         <v>160</v>
       </c>
       <c r="I66" s="11" t="n">
-        <v>0.8187</v>
+        <v>0.9059</v>
       </c>
       <c r="J66" s="8" t="n">
         <v>80</v>
@@ -31019,7 +31019,7 @@
         <v>30</v>
       </c>
       <c r="I68" s="11" t="n">
-        <v>0.8333</v>
+        <v>0.833</v>
       </c>
       <c r="J68" s="8" t="n">
         <v>15</v>
@@ -31062,7 +31062,7 @@
         <v>110</v>
       </c>
       <c r="I69" s="14" t="n">
-        <v>0.9545</v>
+        <v>0.9537</v>
       </c>
       <c r="J69" s="12" t="n">
         <v>55</v>
@@ -31105,7 +31105,7 @@
         <v>10</v>
       </c>
       <c r="I70" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J70" s="8" t="n">
         <v>5</v>
@@ -31191,7 +31191,7 @@
         <v>443</v>
       </c>
       <c r="I72" s="11" t="n">
-        <v>0.9059</v>
+        <v>0.95</v>
       </c>
       <c r="J72" s="8" t="n">
         <v>230</v>
@@ -31234,7 +31234,7 @@
         <v>75</v>
       </c>
       <c r="I73" s="14" t="n">
-        <v>0.7060999999999999</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="J73" s="12" t="n">
         <v>35</v>
@@ -31277,7 +31277,7 @@
         <v>63</v>
       </c>
       <c r="I74" s="11" t="n">
-        <v>0.9166</v>
+        <v>0.9201</v>
       </c>
       <c r="J74" s="8" t="n">
         <v>30</v>
@@ -31320,7 +31320,7 @@
         <v>528</v>
       </c>
       <c r="I75" s="14" t="n">
-        <v>0.8032</v>
+        <v>0.8576</v>
       </c>
       <c r="J75" s="12" t="n">
         <v>265</v>
@@ -31363,7 +31363,7 @@
         <v>346</v>
       </c>
       <c r="I76" s="11" t="n">
-        <v>0.3595</v>
+        <v>0.8321</v>
       </c>
       <c r="J76" s="8" t="n">
         <v>170</v>
@@ -31406,7 +31406,7 @@
         <v>139</v>
       </c>
       <c r="I77" s="14" t="n">
-        <v>0.8358</v>
+        <v>0.8484</v>
       </c>
       <c r="J77" s="12" t="n">
         <v>70</v>
@@ -31449,7 +31449,7 @@
         <v>20</v>
       </c>
       <c r="I78" s="11" t="n">
-        <v>0.45</v>
+        <v>0.9</v>
       </c>
       <c r="J78" s="8" t="n">
         <v>10</v>
@@ -31529,7 +31529,7 @@
         <v>80</v>
       </c>
       <c r="I80" s="11" t="n">
-        <v>0.8375</v>
+        <v>0.8373</v>
       </c>
       <c r="J80" s="8" t="n">
         <v>38</v>
@@ -31572,7 +31572,7 @@
         <v>410</v>
       </c>
       <c r="I81" s="14" t="n">
-        <v>0.8683</v>
+        <v>0.8754</v>
       </c>
       <c r="J81" s="12" t="n">
         <v>200</v>
@@ -31615,7 +31615,7 @@
         <v>180</v>
       </c>
       <c r="I82" s="11" t="n">
-        <v>0.2222</v>
+        <v>0.6166</v>
       </c>
       <c r="J82" s="8" t="n">
         <v>85</v>
@@ -31658,7 +31658,7 @@
         <v>917</v>
       </c>
       <c r="I83" s="14" t="n">
-        <v>0.1352</v>
+        <v>0.9167999999999999</v>
       </c>
       <c r="J83" s="12" t="n">
         <v>225</v>
@@ -31701,7 +31701,7 @@
         <v>79</v>
       </c>
       <c r="I84" s="11" t="n">
-        <v>0.9</v>
+        <v>0.9743000000000001</v>
       </c>
       <c r="J84" s="8" t="n">
         <v>20</v>
@@ -31744,7 +31744,7 @@
         <v>2179</v>
       </c>
       <c r="I85" s="14" t="n">
-        <v>0.6139</v>
+        <v>0.8998</v>
       </c>
       <c r="J85" s="12" t="n">
         <v>684</v>
@@ -32538,7 +32538,7 @@
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>% &gt; 12 °Brix = sección 'VALORES DE AZUCAR' (rango MAYORES DE 12).</t>
+          <t>% ≥ 12 °Brix = % de muestras con 12 °Brix o más (equivale al rango MAYORES DE 12 del ERP).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Informe A4: columna Nº medidas firmeza renombrada, Nº muestras de azúcar deducidas y rangos con dos decimales comprobables a mano
El azúcar de cada bloque se pasa a muestras enteras (N deducido de los % del ERP)
y media, mín, máx y rangos se calculan sobre esas muestras.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016MoDN2MbHCPujrwTZ2bJdV
</commit_message>
<xml_diff>
--- a/Datos de azucar y firmeza por melon en general.xlsx
+++ b/Datos de azucar y firmeza por melon en general.xlsx
@@ -557,7 +557,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Muestras azúcar (estim.)</t>
+          <t>Muestras azúcar (deducidas)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -619,7 +619,7 @@
         <v>7407</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>0.8304</v>
+        <v>0.8308</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>3509</v>
@@ -667,7 +667,7 @@
         <v>95</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>0.6943</v>
+        <v>0.6947</v>
       </c>
       <c r="K3" s="5" t="n">
         <v>45</v>
@@ -719,7 +719,7 @@
         <v>95</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>0.6943</v>
+        <v>0.6947</v>
       </c>
       <c r="K4" s="8" t="n">
         <v>45</v>
@@ -767,7 +767,7 @@
         <v>165</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>0.6906</v>
+        <v>0.6909</v>
       </c>
       <c r="K5" s="5" t="n">
         <v>80</v>
@@ -871,7 +871,7 @@
         <v>35</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>0.3999</v>
+        <v>0.4</v>
       </c>
       <c r="K7" s="8" t="n">
         <v>15</v>
@@ -975,7 +975,7 @@
         <v>110</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>0.8087</v>
+        <v>0.8091</v>
       </c>
       <c r="K9" s="8" t="n">
         <v>55</v>
@@ -1023,7 +1023,7 @@
         <v>664</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>0.8431</v>
+        <v>0.8434</v>
       </c>
       <c r="K10" s="5" t="n">
         <v>319</v>
@@ -1075,7 +1075,7 @@
         <v>15</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>0.06660000000000001</v>
+        <v>0.0667</v>
       </c>
       <c r="K11" s="8" t="n">
         <v>5</v>
@@ -1231,7 +1231,7 @@
         <v>99</v>
       </c>
       <c r="J14" s="11" t="n">
-        <v>0.8989</v>
+        <v>0.899</v>
       </c>
       <c r="K14" s="8" t="n">
         <v>54</v>
@@ -1387,7 +1387,7 @@
         <v>142</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>0.753</v>
+        <v>0.7534999999999999</v>
       </c>
       <c r="K17" s="8" t="n">
         <v>65</v>
@@ -1491,7 +1491,7 @@
         <v>70</v>
       </c>
       <c r="J19" s="11" t="n">
-        <v>0.9425</v>
+        <v>0.9429</v>
       </c>
       <c r="K19" s="8" t="n">
         <v>35</v>
@@ -1543,7 +1543,7 @@
         <v>118</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>0.9486</v>
+        <v>0.9492</v>
       </c>
       <c r="K20" s="8" t="n">
         <v>60</v>
@@ -1595,7 +1595,7 @@
         <v>70</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>0.9567</v>
+        <v>0.9571</v>
       </c>
       <c r="K21" s="8" t="n">
         <v>35</v>
@@ -1643,7 +1643,7 @@
         <v>1290</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>0.7485000000000001</v>
+        <v>0.7488</v>
       </c>
       <c r="K22" s="5" t="n">
         <v>580</v>
@@ -1695,7 +1695,7 @@
         <v>140</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>0.7138</v>
+        <v>0.7143</v>
       </c>
       <c r="K23" s="8" t="n">
         <v>65</v>
@@ -1851,7 +1851,7 @@
         <v>90</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>0.7108</v>
+        <v>0.7111</v>
       </c>
       <c r="K26" s="8" t="n">
         <v>40</v>
@@ -1903,7 +1903,7 @@
         <v>150</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>0.9462</v>
+        <v>0.9467</v>
       </c>
       <c r="K27" s="8" t="n">
         <v>75</v>
@@ -2111,7 +2111,7 @@
         <v>140</v>
       </c>
       <c r="J31" s="11" t="n">
-        <v>0.8995</v>
+        <v>0.9</v>
       </c>
       <c r="K31" s="8" t="n">
         <v>70</v>
@@ -2215,7 +2215,7 @@
         <v>101</v>
       </c>
       <c r="J33" s="11" t="n">
-        <v>0.9207</v>
+        <v>0.9208</v>
       </c>
       <c r="K33" s="8" t="n">
         <v>50</v>
@@ -2319,7 +2319,7 @@
         <v>292</v>
       </c>
       <c r="J35" s="11" t="n">
-        <v>0.6261</v>
+        <v>0.6267</v>
       </c>
       <c r="K35" s="8" t="n">
         <v>115</v>
@@ -2423,7 +2423,7 @@
         <v>157</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>0.643</v>
+        <v>0.6433</v>
       </c>
       <c r="K37" s="8" t="n">
         <v>70</v>
@@ -2471,7 +2471,7 @@
         <v>401</v>
       </c>
       <c r="J38" s="7" t="n">
-        <v>0.8997000000000001</v>
+        <v>0.9002</v>
       </c>
       <c r="K38" s="5" t="n">
         <v>194</v>
@@ -2523,7 +2523,7 @@
         <v>180</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>0.9826</v>
+        <v>0.9833</v>
       </c>
       <c r="K39" s="8" t="n">
         <v>90</v>
@@ -2627,7 +2627,7 @@
         <v>211</v>
       </c>
       <c r="J41" s="11" t="n">
-        <v>0.8242</v>
+        <v>0.8246</v>
       </c>
       <c r="K41" s="8" t="n">
         <v>100</v>
@@ -2675,7 +2675,7 @@
         <v>543</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>0.9371</v>
+        <v>0.9374</v>
       </c>
       <c r="K42" s="5" t="n">
         <v>264</v>
@@ -2727,7 +2727,7 @@
         <v>112</v>
       </c>
       <c r="J43" s="11" t="n">
-        <v>0.9997</v>
+        <v>1</v>
       </c>
       <c r="K43" s="8" t="n">
         <v>55</v>
@@ -2779,7 +2779,7 @@
         <v>30</v>
       </c>
       <c r="J44" s="11" t="n">
-        <v>0.8999</v>
+        <v>0.9</v>
       </c>
       <c r="K44" s="8" t="n">
         <v>15</v>
@@ -2831,7 +2831,7 @@
         <v>60</v>
       </c>
       <c r="J45" s="11" t="n">
-        <v>0.8831</v>
+        <v>0.8833</v>
       </c>
       <c r="K45" s="8" t="n">
         <v>30</v>
@@ -2883,7 +2883,7 @@
         <v>141</v>
       </c>
       <c r="J46" s="11" t="n">
-        <v>0.9142</v>
+        <v>0.9149</v>
       </c>
       <c r="K46" s="8" t="n">
         <v>69</v>
@@ -2987,7 +2987,7 @@
         <v>30</v>
       </c>
       <c r="J48" s="11" t="n">
-        <v>0.9998</v>
+        <v>1</v>
       </c>
       <c r="K48" s="8" t="n">
         <v>15</v>
@@ -3039,7 +3039,7 @@
         <v>30</v>
       </c>
       <c r="J49" s="11" t="n">
-        <v>0.8331</v>
+        <v>0.8333</v>
       </c>
       <c r="K49" s="8" t="n">
         <v>10</v>
@@ -3191,7 +3191,7 @@
         <v>452</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>0.6788</v>
+        <v>0.6792</v>
       </c>
       <c r="K52" s="5" t="n">
         <v>214</v>
@@ -3295,7 +3295,7 @@
         <v>101</v>
       </c>
       <c r="J54" s="11" t="n">
-        <v>0.6039</v>
+        <v>0.604</v>
       </c>
       <c r="K54" s="8" t="n">
         <v>45</v>
@@ -3451,7 +3451,7 @@
         <v>130</v>
       </c>
       <c r="J57" s="11" t="n">
-        <v>0.6993</v>
+        <v>0.7</v>
       </c>
       <c r="K57" s="8" t="n">
         <v>59</v>
@@ -3503,7 +3503,7 @@
         <v>161</v>
       </c>
       <c r="J58" s="11" t="n">
-        <v>0.7201</v>
+        <v>0.7205</v>
       </c>
       <c r="K58" s="8" t="n">
         <v>80</v>
@@ -3551,7 +3551,7 @@
         <v>866</v>
       </c>
       <c r="J59" s="7" t="n">
-        <v>0.8793</v>
+        <v>0.8799</v>
       </c>
       <c r="K59" s="5" t="n">
         <v>400</v>
@@ -3655,7 +3655,7 @@
         <v>30</v>
       </c>
       <c r="J61" s="11" t="n">
-        <v>0.7664</v>
+        <v>0.7667</v>
       </c>
       <c r="K61" s="8" t="n">
         <v>15</v>
@@ -3863,7 +3863,7 @@
         <v>137</v>
       </c>
       <c r="J65" s="11" t="n">
-        <v>0.5976</v>
+        <v>0.5985</v>
       </c>
       <c r="K65" s="8" t="n">
         <v>35</v>
@@ -3967,7 +3967,7 @@
         <v>70</v>
       </c>
       <c r="J67" s="11" t="n">
-        <v>0.9424</v>
+        <v>0.9429</v>
       </c>
       <c r="K67" s="8" t="n">
         <v>35</v>
@@ -4019,7 +4019,7 @@
         <v>139</v>
       </c>
       <c r="J68" s="11" t="n">
-        <v>0.9272</v>
+        <v>0.9281</v>
       </c>
       <c r="K68" s="8" t="n">
         <v>65</v>
@@ -4059,7 +4059,7 @@
         <v>1</v>
       </c>
       <c r="F69" s="10" t="n">
-        <v>14.39</v>
+        <v>14.38</v>
       </c>
       <c r="G69" s="8" t="n">
         <v>9</v>
@@ -4071,7 +4071,7 @@
         <v>390</v>
       </c>
       <c r="J69" s="11" t="n">
-        <v>0.9532</v>
+        <v>0.9538</v>
       </c>
       <c r="K69" s="8" t="n">
         <v>195</v>
@@ -4119,7 +4119,7 @@
         <v>1000</v>
       </c>
       <c r="J70" s="7" t="n">
-        <v>0.7796999999999999</v>
+        <v>0.78</v>
       </c>
       <c r="K70" s="5" t="n">
         <v>460</v>
@@ -4223,7 +4223,7 @@
         <v>189</v>
       </c>
       <c r="J72" s="11" t="n">
-        <v>0.9201</v>
+        <v>0.9206</v>
       </c>
       <c r="K72" s="8" t="n">
         <v>95</v>
@@ -4275,7 +4275,7 @@
         <v>30</v>
       </c>
       <c r="J73" s="11" t="n">
-        <v>0.6331</v>
+        <v>0.6333</v>
       </c>
       <c r="K73" s="8" t="n">
         <v>15</v>
@@ -4327,7 +4327,7 @@
         <v>130</v>
       </c>
       <c r="J74" s="11" t="n">
-        <v>0.8223</v>
+        <v>0.8231000000000001</v>
       </c>
       <c r="K74" s="8" t="n">
         <v>65</v>
@@ -4639,7 +4639,7 @@
         <v>60</v>
       </c>
       <c r="J80" s="11" t="n">
-        <v>0.9829</v>
+        <v>0.9833</v>
       </c>
       <c r="K80" s="8" t="n">
         <v>25</v>
@@ -4899,7 +4899,7 @@
         <v>71</v>
       </c>
       <c r="J85" s="11" t="n">
-        <v>0.7461</v>
+        <v>0.7465000000000001</v>
       </c>
       <c r="K85" s="8" t="n">
         <v>35</v>
@@ -4951,7 +4951,7 @@
         <v>130</v>
       </c>
       <c r="J86" s="11" t="n">
-        <v>0.1842</v>
+        <v>0.1846</v>
       </c>
       <c r="K86" s="8" t="n">
         <v>30</v>
@@ -5091,7 +5091,7 @@
         <v>9</v>
       </c>
       <c r="F89" s="6" t="n">
-        <v>14.15</v>
+        <v>14.14</v>
       </c>
       <c r="G89" s="5" t="n">
         <v>8</v>
@@ -5103,7 +5103,7 @@
         <v>1000</v>
       </c>
       <c r="J89" s="7" t="n">
-        <v>0.9386</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="K89" s="5" t="n">
         <v>509</v>
@@ -5155,7 +5155,7 @@
         <v>109</v>
       </c>
       <c r="J90" s="11" t="n">
-        <v>0.8894</v>
+        <v>0.8899</v>
       </c>
       <c r="K90" s="8" t="n">
         <v>54</v>
@@ -5207,7 +5207,7 @@
         <v>150</v>
       </c>
       <c r="J91" s="11" t="n">
-        <v>0.9796</v>
+        <v>0.98</v>
       </c>
       <c r="K91" s="8" t="n">
         <v>75</v>
@@ -5311,7 +5311,7 @@
         <v>299</v>
       </c>
       <c r="J93" s="11" t="n">
-        <v>0.9425</v>
+        <v>0.9431</v>
       </c>
       <c r="K93" s="8" t="n">
         <v>155</v>
@@ -5363,7 +5363,7 @@
         <v>261</v>
       </c>
       <c r="J94" s="11" t="n">
-        <v>0.9804</v>
+        <v>0.9808</v>
       </c>
       <c r="K94" s="8" t="n">
         <v>130</v>
@@ -5519,7 +5519,7 @@
         <v>21</v>
       </c>
       <c r="J97" s="11" t="n">
-        <v>0.8092</v>
+        <v>0.8095</v>
       </c>
       <c r="K97" s="8" t="n">
         <v>10</v>
@@ -5619,7 +5619,7 @@
         <v>155</v>
       </c>
       <c r="J99" s="7" t="n">
-        <v>0.8127</v>
+        <v>0.8129</v>
       </c>
       <c r="K99" s="5" t="n">
         <v>75</v>
@@ -5659,7 +5659,7 @@
         <v>1</v>
       </c>
       <c r="F100" s="10" t="n">
-        <v>13.7</v>
+        <v>13.69</v>
       </c>
       <c r="G100" s="8" t="n">
         <v>9</v>
@@ -5671,7 +5671,7 @@
         <v>95</v>
       </c>
       <c r="J100" s="11" t="n">
-        <v>0.7049</v>
+        <v>0.7053</v>
       </c>
       <c r="K100" s="8" t="n">
         <v>45</v>
@@ -5823,7 +5823,7 @@
         <v>281</v>
       </c>
       <c r="J103" s="7" t="n">
-        <v>0.8929</v>
+        <v>0.8932</v>
       </c>
       <c r="K103" s="5" t="n">
         <v>135</v>
@@ -5875,7 +5875,7 @@
         <v>140</v>
       </c>
       <c r="J104" s="11" t="n">
-        <v>0.9353</v>
+        <v>0.9357</v>
       </c>
       <c r="K104" s="8" t="n">
         <v>65</v>
@@ -5927,7 +5927,7 @@
         <v>71</v>
       </c>
       <c r="J105" s="11" t="n">
-        <v>0.8023</v>
+        <v>0.8028</v>
       </c>
       <c r="K105" s="8" t="n">
         <v>35</v>
@@ -6031,7 +6031,7 @@
         <v>30</v>
       </c>
       <c r="J107" s="11" t="n">
-        <v>0.8997000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="K107" s="8" t="n">
         <v>15</v>
@@ -6079,7 +6079,7 @@
         <v>314</v>
       </c>
       <c r="J108" s="7" t="n">
-        <v>0.834</v>
+        <v>0.8344</v>
       </c>
       <c r="K108" s="5" t="n">
         <v>150</v>
@@ -6131,7 +6131,7 @@
         <v>29</v>
       </c>
       <c r="J109" s="11" t="n">
-        <v>0.5171</v>
+        <v>0.5172</v>
       </c>
       <c r="K109" s="8" t="n">
         <v>10</v>
@@ -6183,7 +6183,7 @@
         <v>120</v>
       </c>
       <c r="J110" s="11" t="n">
-        <v>0.9498</v>
+        <v>0.95</v>
       </c>
       <c r="K110" s="8" t="n">
         <v>60</v>
@@ -6235,7 +6235,7 @@
         <v>145</v>
       </c>
       <c r="J111" s="11" t="n">
-        <v>0.7924</v>
+        <v>0.7931</v>
       </c>
       <c r="K111" s="8" t="n">
         <v>70</v>
@@ -6387,7 +6387,7 @@
         <v>30</v>
       </c>
       <c r="J114" s="7" t="n">
-        <v>0.6663</v>
+        <v>0.6667</v>
       </c>
       <c r="K114" s="5" t="n">
         <v>15</v>
@@ -6439,7 +6439,7 @@
         <v>30</v>
       </c>
       <c r="J115" s="11" t="n">
-        <v>0.6663</v>
+        <v>0.6667</v>
       </c>
       <c r="K115" s="8" t="n">
         <v>15</v>
@@ -6927,7 +6927,7 @@
         <v>81</v>
       </c>
       <c r="J125" s="7" t="n">
-        <v>0.901</v>
+        <v>0.9012</v>
       </c>
       <c r="K125" s="5" t="n">
         <v>34</v>
@@ -6979,7 +6979,7 @@
         <v>60</v>
       </c>
       <c r="J126" s="11" t="n">
-        <v>0.9498</v>
+        <v>0.95</v>
       </c>
       <c r="K126" s="8" t="n">
         <v>29</v>
@@ -7067,7 +7067,7 @@
         <v>21</v>
       </c>
       <c r="J128" s="11" t="n">
-        <v>0.7616000000000001</v>
+        <v>0.7619</v>
       </c>
       <c r="K128" s="8" t="n">
         <v>5</v>
@@ -7275,7 +7275,7 @@
         <v>69</v>
       </c>
       <c r="F133" s="3" t="n">
-        <v>13.4</v>
+        <v>13.49</v>
       </c>
       <c r="G133" s="2" t="n">
         <v>5</v>
@@ -7284,10 +7284,10 @@
         <v>19</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>8173</v>
+        <v>10631</v>
       </c>
       <c r="J133" s="4" t="n">
-        <v>0.8091</v>
+        <v>0.8151</v>
       </c>
       <c r="K133" s="2" t="n">
         <v>2374</v>
@@ -7435,7 +7435,7 @@
         <v>323</v>
       </c>
       <c r="J136" s="7" t="n">
-        <v>0.7894</v>
+        <v>0.7895</v>
       </c>
       <c r="K136" s="5" t="n">
         <v>80</v>
@@ -7643,7 +7643,7 @@
         <v>63</v>
       </c>
       <c r="J140" s="11" t="n">
-        <v>0.841</v>
+        <v>0.8413</v>
       </c>
       <c r="K140" s="8" t="n">
         <v>15</v>
@@ -7835,7 +7835,7 @@
         <v>10</v>
       </c>
       <c r="F144" s="6" t="n">
-        <v>13.86</v>
+        <v>14.08</v>
       </c>
       <c r="G144" s="5" t="n">
         <v>5</v>
@@ -7844,10 +7844,10 @@
         <v>18</v>
       </c>
       <c r="I144" s="5" t="n">
-        <v>1238</v>
+        <v>1855</v>
       </c>
       <c r="J144" s="7" t="n">
-        <v>0.8502</v>
+        <v>0.8836000000000001</v>
       </c>
       <c r="K144" s="5" t="n">
         <v>305</v>
@@ -7887,7 +7887,7 @@
         <v>1</v>
       </c>
       <c r="F145" s="10" t="n">
-        <v>14.73</v>
+        <v>14.72</v>
       </c>
       <c r="G145" s="8" t="n">
         <v>8</v>
@@ -7899,7 +7899,7 @@
         <v>60</v>
       </c>
       <c r="J145" s="11" t="n">
-        <v>0.9498</v>
+        <v>0.95</v>
       </c>
       <c r="K145" s="8" t="n">
         <v>15</v>
@@ -7951,7 +7951,7 @@
         <v>208</v>
       </c>
       <c r="J146" s="11" t="n">
-        <v>0.8314</v>
+        <v>0.8317</v>
       </c>
       <c r="K146" s="8" t="n">
         <v>40</v>
@@ -8003,7 +8003,7 @@
         <v>180</v>
       </c>
       <c r="J147" s="11" t="n">
-        <v>0.9273</v>
+        <v>0.9278</v>
       </c>
       <c r="K147" s="8" t="n">
         <v>45</v>
@@ -8107,7 +8107,7 @@
         <v>60</v>
       </c>
       <c r="J149" s="11" t="n">
-        <v>0.9497</v>
+        <v>0.95</v>
       </c>
       <c r="K149" s="8" t="n">
         <v>10</v>
@@ -8251,7 +8251,7 @@
         <v>1</v>
       </c>
       <c r="F152" s="10" t="n">
-        <v>14.52</v>
+        <v>14.51</v>
       </c>
       <c r="G152" s="8" t="n">
         <v>5</v>
@@ -8260,10 +8260,10 @@
         <v>16</v>
       </c>
       <c r="I152" s="8" t="n">
-        <v>100</v>
+        <v>717</v>
       </c>
       <c r="J152" s="11" t="n">
-        <v>0.9492</v>
+        <v>0.9498</v>
       </c>
       <c r="K152" s="8" t="n">
         <v>55</v>
@@ -8315,7 +8315,7 @@
         <v>190</v>
       </c>
       <c r="J153" s="11" t="n">
-        <v>0.8733</v>
+        <v>0.8737</v>
       </c>
       <c r="K153" s="8" t="n">
         <v>45</v>
@@ -8367,7 +8367,7 @@
         <v>130</v>
       </c>
       <c r="J154" s="11" t="n">
-        <v>0.6534</v>
+        <v>0.6538</v>
       </c>
       <c r="K154" s="8" t="n">
         <v>30</v>
@@ -8415,7 +8415,7 @@
         <v>747</v>
       </c>
       <c r="J155" s="7" t="n">
-        <v>0.7749</v>
+        <v>0.7751</v>
       </c>
       <c r="K155" s="5" t="n">
         <v>170</v>
@@ -8519,7 +8519,7 @@
         <v>160</v>
       </c>
       <c r="J157" s="11" t="n">
-        <v>0.7995</v>
+        <v>0.8</v>
       </c>
       <c r="K157" s="8" t="n">
         <v>40</v>
@@ -8571,7 +8571,7 @@
         <v>60</v>
       </c>
       <c r="J158" s="11" t="n">
-        <v>0.883</v>
+        <v>0.8833</v>
       </c>
       <c r="K158" s="8" t="n">
         <v>15</v>
@@ -8623,7 +8623,7 @@
         <v>30</v>
       </c>
       <c r="J159" s="11" t="n">
-        <v>0.5664</v>
+        <v>0.5667</v>
       </c>
       <c r="K159" s="8" t="n">
         <v>5</v>
@@ -8727,7 +8727,7 @@
         <v>199</v>
       </c>
       <c r="J161" s="11" t="n">
-        <v>0.6831</v>
+        <v>0.6834</v>
       </c>
       <c r="K161" s="8" t="n">
         <v>40</v>
@@ -8831,7 +8831,7 @@
         <v>38</v>
       </c>
       <c r="J163" s="11" t="n">
-        <v>0.9735</v>
+        <v>0.9737</v>
       </c>
       <c r="K163" s="8" t="n">
         <v>10</v>
@@ -8867,7 +8867,7 @@
         <v>33</v>
       </c>
       <c r="F164" s="6" t="n">
-        <v>13.11</v>
+        <v>13.1</v>
       </c>
       <c r="G164" s="5" t="n">
         <v>5</v>
@@ -8879,7 +8879,7 @@
         <v>4126</v>
       </c>
       <c r="J164" s="7" t="n">
-        <v>0.7825</v>
+        <v>0.7828000000000001</v>
       </c>
       <c r="K164" s="5" t="n">
         <v>985</v>
@@ -8931,7 +8931,7 @@
         <v>175</v>
       </c>
       <c r="J165" s="11" t="n">
-        <v>0.874</v>
+        <v>0.8743</v>
       </c>
       <c r="K165" s="8" t="n">
         <v>45</v>
@@ -9035,7 +9035,7 @@
         <v>260</v>
       </c>
       <c r="J167" s="11" t="n">
-        <v>0.7842</v>
+        <v>0.7846</v>
       </c>
       <c r="K167" s="8" t="n">
         <v>55</v>
@@ -9087,7 +9087,7 @@
         <v>81</v>
       </c>
       <c r="J168" s="11" t="n">
-        <v>0.7279</v>
+        <v>0.7284</v>
       </c>
       <c r="K168" s="8" t="n">
         <v>20</v>
@@ -9139,7 +9139,7 @@
         <v>160</v>
       </c>
       <c r="J169" s="11" t="n">
-        <v>0.7936</v>
+        <v>0.7937</v>
       </c>
       <c r="K169" s="8" t="n">
         <v>40</v>
@@ -9243,7 +9243,7 @@
         <v>59</v>
       </c>
       <c r="J171" s="11" t="n">
-        <v>0.7285</v>
+        <v>0.7288</v>
       </c>
       <c r="K171" s="8" t="n">
         <v>15</v>
@@ -9295,7 +9295,7 @@
         <v>280</v>
       </c>
       <c r="J172" s="11" t="n">
-        <v>0.771</v>
+        <v>0.7714</v>
       </c>
       <c r="K172" s="8" t="n">
         <v>65</v>
@@ -9347,7 +9347,7 @@
         <v>160</v>
       </c>
       <c r="J173" s="11" t="n">
-        <v>0.8434</v>
+        <v>0.8438</v>
       </c>
       <c r="K173" s="8" t="n">
         <v>40</v>
@@ -9503,7 +9503,7 @@
         <v>60</v>
       </c>
       <c r="J176" s="11" t="n">
-        <v>0.9163</v>
+        <v>0.9167</v>
       </c>
       <c r="K176" s="8" t="n">
         <v>15</v>
@@ -9555,7 +9555,7 @@
         <v>79</v>
       </c>
       <c r="J177" s="11" t="n">
-        <v>0.9489</v>
+        <v>0.9494</v>
       </c>
       <c r="K177" s="8" t="n">
         <v>15</v>
@@ -9711,7 +9711,7 @@
         <v>60</v>
       </c>
       <c r="J180" s="11" t="n">
-        <v>0.8829</v>
+        <v>0.8833</v>
       </c>
       <c r="K180" s="8" t="n">
         <v>15</v>
@@ -9763,7 +9763,7 @@
         <v>180</v>
       </c>
       <c r="J181" s="11" t="n">
-        <v>0.8107</v>
+        <v>0.8111</v>
       </c>
       <c r="K181" s="8" t="n">
         <v>40</v>
@@ -9919,7 +9919,7 @@
         <v>198</v>
       </c>
       <c r="J184" s="11" t="n">
-        <v>0.7621</v>
+        <v>0.7625999999999999</v>
       </c>
       <c r="K184" s="8" t="n">
         <v>50</v>
@@ -9971,7 +9971,7 @@
         <v>99</v>
       </c>
       <c r="J185" s="11" t="n">
-        <v>0.8787</v>
+        <v>0.8788</v>
       </c>
       <c r="K185" s="8" t="n">
         <v>20</v>
@@ -10075,7 +10075,7 @@
         <v>41</v>
       </c>
       <c r="J187" s="11" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.8537</v>
       </c>
       <c r="K187" s="8" t="n">
         <v>10</v>
@@ -10127,7 +10127,7 @@
         <v>59</v>
       </c>
       <c r="J188" s="11" t="n">
-        <v>0.6604</v>
+        <v>0.661</v>
       </c>
       <c r="K188" s="8" t="n">
         <v>15</v>
@@ -10179,7 +10179,7 @@
         <v>278</v>
       </c>
       <c r="J189" s="11" t="n">
-        <v>0.7762</v>
+        <v>0.777</v>
       </c>
       <c r="K189" s="8" t="n">
         <v>70</v>
@@ -10231,7 +10231,7 @@
         <v>293</v>
       </c>
       <c r="J190" s="11" t="n">
-        <v>0.8663999999999999</v>
+        <v>0.8669</v>
       </c>
       <c r="K190" s="8" t="n">
         <v>70</v>
@@ -10283,7 +10283,7 @@
         <v>416</v>
       </c>
       <c r="J191" s="11" t="n">
-        <v>0.6343</v>
+        <v>0.6346000000000001</v>
       </c>
       <c r="K191" s="8" t="n">
         <v>90</v>
@@ -10335,7 +10335,7 @@
         <v>110</v>
       </c>
       <c r="J192" s="11" t="n">
-        <v>0.5907</v>
+        <v>0.5909</v>
       </c>
       <c r="K192" s="8" t="n">
         <v>20</v>
@@ -10387,7 +10387,7 @@
         <v>139</v>
       </c>
       <c r="J193" s="11" t="n">
-        <v>0.7479</v>
+        <v>0.7482</v>
       </c>
       <c r="K193" s="8" t="n">
         <v>40</v>
@@ -10491,7 +10491,7 @@
         <v>120</v>
       </c>
       <c r="J195" s="11" t="n">
-        <v>0.858</v>
+        <v>0.8583</v>
       </c>
       <c r="K195" s="8" t="n">
         <v>30</v>
@@ -10543,7 +10543,7 @@
         <v>99</v>
       </c>
       <c r="J196" s="11" t="n">
-        <v>0.8787</v>
+        <v>0.8788</v>
       </c>
       <c r="K196" s="8" t="n">
         <v>25</v>
@@ -10595,7 +10595,7 @@
         <v>140</v>
       </c>
       <c r="J197" s="11" t="n">
-        <v>0.8354</v>
+        <v>0.8357</v>
       </c>
       <c r="K197" s="8" t="n">
         <v>35</v>
@@ -10643,7 +10643,7 @@
         <v>219</v>
       </c>
       <c r="J198" s="7" t="n">
-        <v>0.9404</v>
+        <v>0.9406</v>
       </c>
       <c r="K198" s="5" t="n">
         <v>55</v>
@@ -10695,7 +10695,7 @@
         <v>139</v>
       </c>
       <c r="J199" s="11" t="n">
-        <v>0.9564</v>
+        <v>0.9568</v>
       </c>
       <c r="K199" s="8" t="n">
         <v>35</v>
@@ -10783,7 +10783,7 @@
         <v>11</v>
       </c>
       <c r="F201" s="6" t="n">
-        <v>13.9</v>
+        <v>13.65</v>
       </c>
       <c r="G201" s="5" t="n">
         <v>6</v>
@@ -10792,10 +10792,10 @@
         <v>18</v>
       </c>
       <c r="I201" s="5" t="n">
-        <v>1200</v>
+        <v>1791</v>
       </c>
       <c r="J201" s="7" t="n">
-        <v>0.8599</v>
+        <v>0.8219</v>
       </c>
       <c r="K201" s="5" t="n">
         <v>435</v>
@@ -10847,7 +10847,7 @@
         <v>119</v>
       </c>
       <c r="J202" s="11" t="n">
-        <v>0.9577</v>
+        <v>0.958</v>
       </c>
       <c r="K202" s="8" t="n">
         <v>30</v>
@@ -10951,7 +10951,7 @@
         <v>19</v>
       </c>
       <c r="J204" s="11" t="n">
-        <v>0.9471000000000001</v>
+        <v>0.9474</v>
       </c>
       <c r="K204" s="8" t="n">
         <v>5</v>
@@ -11211,7 +11211,7 @@
         <v>141</v>
       </c>
       <c r="J209" s="11" t="n">
-        <v>0.9144</v>
+        <v>0.9149</v>
       </c>
       <c r="K209" s="8" t="n">
         <v>35</v>
@@ -11260,10 +11260,10 @@
         <v>18</v>
       </c>
       <c r="I210" s="8" t="n">
-        <v>100</v>
+        <v>691</v>
       </c>
       <c r="J210" s="11" t="n">
-        <v>0.7431</v>
+        <v>0.7438</v>
       </c>
       <c r="K210" s="8" t="n">
         <v>160</v>
@@ -11315,7 +11315,7 @@
         <v>381</v>
       </c>
       <c r="J211" s="11" t="n">
-        <v>0.8313</v>
+        <v>0.832</v>
       </c>
       <c r="K211" s="8" t="n">
         <v>95</v>
@@ -11503,7 +11503,7 @@
         <v>4</v>
       </c>
       <c r="F215" s="6" t="n">
-        <v>13.85</v>
+        <v>13.76</v>
       </c>
       <c r="G215" s="5" t="n">
         <v>5</v>
@@ -11512,10 +11512,10 @@
         <v>19</v>
       </c>
       <c r="I215" s="5" t="n">
-        <v>200</v>
+        <v>1450</v>
       </c>
       <c r="J215" s="7" t="n">
-        <v>0.8192</v>
+        <v>0.8193</v>
       </c>
       <c r="K215" s="5" t="n">
         <v>314</v>
@@ -11567,7 +11567,7 @@
         <v>60</v>
       </c>
       <c r="J216" s="11" t="n">
-        <v>0.7998</v>
+        <v>0.8</v>
       </c>
       <c r="K216" s="8" t="n">
         <v>10</v>
@@ -11668,10 +11668,10 @@
         <v>19</v>
       </c>
       <c r="I218" s="8" t="n">
-        <v>100</v>
+        <v>1350</v>
       </c>
       <c r="J218" s="11" t="n">
-        <v>0.8185</v>
+        <v>0.8193</v>
       </c>
       <c r="K218" s="8" t="n">
         <v>294</v>
@@ -11771,7 +11771,7 @@
         <v>3382</v>
       </c>
       <c r="J220" s="4" t="n">
-        <v>0.837</v>
+        <v>0.8374</v>
       </c>
       <c r="K220" s="2" t="n">
         <v>833</v>
@@ -11819,7 +11819,7 @@
         <v>60</v>
       </c>
       <c r="J221" s="7" t="n">
-        <v>0.7163</v>
+        <v>0.7167</v>
       </c>
       <c r="K221" s="5" t="n">
         <v>15</v>
@@ -11871,7 +11871,7 @@
         <v>60</v>
       </c>
       <c r="J222" s="11" t="n">
-        <v>0.7163</v>
+        <v>0.7167</v>
       </c>
       <c r="K222" s="8" t="n">
         <v>15</v>
@@ -12171,7 +12171,7 @@
         <v>522</v>
       </c>
       <c r="J228" s="7" t="n">
-        <v>0.9076</v>
+        <v>0.908</v>
       </c>
       <c r="K228" s="5" t="n">
         <v>130</v>
@@ -12275,7 +12275,7 @@
         <v>241</v>
       </c>
       <c r="J230" s="11" t="n">
-        <v>0.9411</v>
+        <v>0.9419</v>
       </c>
       <c r="K230" s="8" t="n">
         <v>60</v>
@@ -12327,7 +12327,7 @@
         <v>201</v>
       </c>
       <c r="J231" s="11" t="n">
-        <v>0.8604000000000001</v>
+        <v>0.8607</v>
       </c>
       <c r="K231" s="8" t="n">
         <v>50</v>
@@ -12375,7 +12375,7 @@
         <v>608</v>
       </c>
       <c r="J232" s="7" t="n">
-        <v>0.7742</v>
+        <v>0.7747000000000001</v>
       </c>
       <c r="K232" s="5" t="n">
         <v>135</v>
@@ -12427,7 +12427,7 @@
         <v>45</v>
       </c>
       <c r="J233" s="11" t="n">
-        <v>0.533</v>
+        <v>0.5333</v>
       </c>
       <c r="K233" s="8" t="n">
         <v>5</v>
@@ -12583,7 +12583,7 @@
         <v>140</v>
       </c>
       <c r="J236" s="11" t="n">
-        <v>0.4212</v>
+        <v>0.4214</v>
       </c>
       <c r="K236" s="8" t="n">
         <v>25</v>
@@ -12635,7 +12635,7 @@
         <v>209</v>
       </c>
       <c r="J237" s="11" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9426</v>
       </c>
       <c r="K237" s="8" t="n">
         <v>50</v>
@@ -12687,7 +12687,7 @@
         <v>174</v>
       </c>
       <c r="J238" s="11" t="n">
-        <v>0.8673</v>
+        <v>0.8678</v>
       </c>
       <c r="K238" s="8" t="n">
         <v>45</v>
@@ -12735,7 +12735,7 @@
         <v>703</v>
       </c>
       <c r="J239" s="7" t="n">
-        <v>0.8942</v>
+        <v>0.8947000000000001</v>
       </c>
       <c r="K239" s="5" t="n">
         <v>160</v>
@@ -12775,7 +12775,7 @@
         <v>1</v>
       </c>
       <c r="F240" s="10" t="n">
-        <v>13.85</v>
+        <v>13.84</v>
       </c>
       <c r="G240" s="8" t="n">
         <v>5</v>
@@ -12787,7 +12787,7 @@
         <v>241</v>
       </c>
       <c r="J240" s="11" t="n">
-        <v>0.8376</v>
+        <v>0.8381999999999999</v>
       </c>
       <c r="K240" s="8" t="n">
         <v>55</v>
@@ -12839,7 +12839,7 @@
         <v>290</v>
       </c>
       <c r="J241" s="11" t="n">
-        <v>0.9510999999999999</v>
+        <v>0.9517</v>
       </c>
       <c r="K241" s="8" t="n">
         <v>70</v>
@@ -12989,7 +12989,7 @@
         <v>132</v>
       </c>
       <c r="J244" s="11" t="n">
-        <v>0.8557</v>
+        <v>0.8561</v>
       </c>
       <c r="K244" s="8" t="n">
         <v>30</v>
@@ -13037,7 +13037,7 @@
         <v>439</v>
       </c>
       <c r="J245" s="7" t="n">
-        <v>0.7539</v>
+        <v>0.754</v>
       </c>
       <c r="K245" s="5" t="n">
         <v>134</v>
@@ -13089,7 +13089,7 @@
         <v>60</v>
       </c>
       <c r="J246" s="11" t="n">
-        <v>0.7166</v>
+        <v>0.7167</v>
       </c>
       <c r="K246" s="8" t="n">
         <v>39</v>
@@ -13141,7 +13141,7 @@
         <v>79</v>
       </c>
       <c r="J247" s="11" t="n">
-        <v>0.7593</v>
+        <v>0.7595</v>
       </c>
       <c r="K247" s="8" t="n">
         <v>20</v>
@@ -13193,7 +13193,7 @@
         <v>160</v>
       </c>
       <c r="J248" s="11" t="n">
-        <v>0.7499</v>
+        <v>0.75</v>
       </c>
       <c r="K248" s="8" t="n">
         <v>40</v>
@@ -13345,7 +13345,7 @@
         <v>460</v>
       </c>
       <c r="J251" s="7" t="n">
-        <v>0.8451</v>
+        <v>0.8457</v>
       </c>
       <c r="K251" s="5" t="n">
         <v>120</v>
@@ -13397,7 +13397,7 @@
         <v>340</v>
       </c>
       <c r="J252" s="11" t="n">
-        <v>0.8406</v>
+        <v>0.8411999999999999</v>
       </c>
       <c r="K252" s="8" t="n">
         <v>90</v>
@@ -13449,7 +13449,7 @@
         <v>120</v>
       </c>
       <c r="J253" s="11" t="n">
-        <v>0.858</v>
+        <v>0.8583</v>
       </c>
       <c r="K253" s="8" t="n">
         <v>30</v>
@@ -13497,7 +13497,7 @@
         <v>430</v>
       </c>
       <c r="J254" s="7" t="n">
-        <v>0.8065</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="K254" s="5" t="n">
         <v>99</v>
@@ -13549,7 +13549,7 @@
         <v>330</v>
       </c>
       <c r="J255" s="11" t="n">
-        <v>0.8055</v>
+        <v>0.8061</v>
       </c>
       <c r="K255" s="8" t="n">
         <v>79</v>
@@ -13753,7 +13753,7 @@
         <v>7405</v>
       </c>
       <c r="J259" s="4" t="n">
-        <v>0.9396</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K259" s="2" t="n">
         <v>3694</v>
@@ -13901,7 +13901,7 @@
         <v>1842</v>
       </c>
       <c r="J262" s="7" t="n">
-        <v>0.9550999999999999</v>
+        <v>0.9555</v>
       </c>
       <c r="K262" s="5" t="n">
         <v>914</v>
@@ -14045,7 +14045,7 @@
         <v>1</v>
       </c>
       <c r="F265" s="10" t="n">
-        <v>14.63</v>
+        <v>14.62</v>
       </c>
       <c r="G265" s="8" t="n">
         <v>10</v>
@@ -14057,7 +14057,7 @@
         <v>52</v>
       </c>
       <c r="J265" s="11" t="n">
-        <v>0.9804</v>
+        <v>0.9808</v>
       </c>
       <c r="K265" s="8" t="n">
         <v>24</v>
@@ -14109,7 +14109,7 @@
         <v>69</v>
       </c>
       <c r="J266" s="11" t="n">
-        <v>0.9704</v>
+        <v>0.971</v>
       </c>
       <c r="K266" s="8" t="n">
         <v>35</v>
@@ -14161,7 +14161,7 @@
         <v>120</v>
       </c>
       <c r="J267" s="11" t="n">
-        <v>0.983</v>
+        <v>0.9833</v>
       </c>
       <c r="K267" s="8" t="n">
         <v>60</v>
@@ -14213,7 +14213,7 @@
         <v>70</v>
       </c>
       <c r="J268" s="11" t="n">
-        <v>0.8851</v>
+        <v>0.8857</v>
       </c>
       <c r="K268" s="8" t="n">
         <v>35</v>
@@ -14265,7 +14265,7 @@
         <v>369</v>
       </c>
       <c r="J269" s="11" t="n">
-        <v>0.9858</v>
+        <v>0.9864000000000001</v>
       </c>
       <c r="K269" s="8" t="n">
         <v>185</v>
@@ -14369,7 +14369,7 @@
         <v>110</v>
       </c>
       <c r="J271" s="11" t="n">
-        <v>0.9902</v>
+        <v>0.9909</v>
       </c>
       <c r="K271" s="8" t="n">
         <v>55</v>
@@ -14421,7 +14421,7 @@
         <v>110</v>
       </c>
       <c r="J272" s="11" t="n">
-        <v>0.9719</v>
+        <v>0.9727</v>
       </c>
       <c r="K272" s="8" t="n">
         <v>55</v>
@@ -14473,7 +14473,7 @@
         <v>90</v>
       </c>
       <c r="J273" s="11" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.9333</v>
       </c>
       <c r="K273" s="8" t="n">
         <v>50</v>
@@ -14525,7 +14525,7 @@
         <v>60</v>
       </c>
       <c r="J274" s="11" t="n">
-        <v>0.8997000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="K274" s="8" t="n">
         <v>30</v>
@@ -14577,7 +14577,7 @@
         <v>121</v>
       </c>
       <c r="J275" s="11" t="n">
-        <v>0.8921</v>
+        <v>0.8925999999999999</v>
       </c>
       <c r="K275" s="8" t="n">
         <v>60</v>
@@ -14889,7 +14889,7 @@
         <v>119</v>
       </c>
       <c r="J281" s="11" t="n">
-        <v>0.9577</v>
+        <v>0.958</v>
       </c>
       <c r="K281" s="8" t="n">
         <v>55</v>
@@ -14941,7 +14941,7 @@
         <v>70</v>
       </c>
       <c r="J282" s="11" t="n">
-        <v>0.9709</v>
+        <v>0.9714</v>
       </c>
       <c r="K282" s="8" t="n">
         <v>35</v>
@@ -14993,7 +14993,7 @@
         <v>51</v>
       </c>
       <c r="J283" s="11" t="n">
-        <v>0.9997</v>
+        <v>1</v>
       </c>
       <c r="K283" s="8" t="n">
         <v>25</v>
@@ -15045,7 +15045,7 @@
         <v>30</v>
       </c>
       <c r="J284" s="11" t="n">
-        <v>0.9998</v>
+        <v>1</v>
       </c>
       <c r="K284" s="8" t="n">
         <v>15</v>
@@ -15149,7 +15149,7 @@
         <v>61</v>
       </c>
       <c r="J286" s="11" t="n">
-        <v>0.9503</v>
+        <v>0.9508</v>
       </c>
       <c r="K286" s="8" t="n">
         <v>30</v>
@@ -15197,7 +15197,7 @@
         <v>660</v>
       </c>
       <c r="J287" s="7" t="n">
-        <v>0.8695000000000001</v>
+        <v>0.8697</v>
       </c>
       <c r="K287" s="5" t="n">
         <v>343</v>
@@ -15249,7 +15249,7 @@
         <v>11</v>
       </c>
       <c r="J288" s="11" t="n">
-        <v>0.909</v>
+        <v>0.9091</v>
       </c>
       <c r="K288" s="8" t="n">
         <v>5</v>
@@ -15353,7 +15353,7 @@
         <v>120</v>
       </c>
       <c r="J290" s="11" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.9333</v>
       </c>
       <c r="K290" s="8" t="n">
         <v>65</v>
@@ -15405,7 +15405,7 @@
         <v>70</v>
       </c>
       <c r="J291" s="11" t="n">
-        <v>0.9566</v>
+        <v>0.9571</v>
       </c>
       <c r="K291" s="8" t="n">
         <v>35</v>
@@ -15509,7 +15509,7 @@
         <v>199</v>
       </c>
       <c r="J293" s="11" t="n">
-        <v>0.8137</v>
+        <v>0.8141</v>
       </c>
       <c r="K293" s="8" t="n">
         <v>108</v>
@@ -15609,7 +15609,7 @@
         <v>1409</v>
       </c>
       <c r="J295" s="7" t="n">
-        <v>0.9081</v>
+        <v>0.9084</v>
       </c>
       <c r="K295" s="5" t="n">
         <v>697</v>
@@ -15661,7 +15661,7 @@
         <v>90</v>
       </c>
       <c r="J296" s="11" t="n">
-        <v>0.8774</v>
+        <v>0.8778</v>
       </c>
       <c r="K296" s="8" t="n">
         <v>50</v>
@@ -15713,7 +15713,7 @@
         <v>30</v>
       </c>
       <c r="J297" s="11" t="n">
-        <v>0.7999000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="K297" s="8" t="n">
         <v>20</v>
@@ -15817,7 +15817,7 @@
         <v>19</v>
       </c>
       <c r="J299" s="11" t="n">
-        <v>0.6314</v>
+        <v>0.6316000000000001</v>
       </c>
       <c r="K299" s="8" t="n">
         <v>5</v>
@@ -15869,7 +15869,7 @@
         <v>101</v>
       </c>
       <c r="J300" s="11" t="n">
-        <v>0.6435</v>
+        <v>0.6435999999999999</v>
       </c>
       <c r="K300" s="8" t="n">
         <v>45</v>
@@ -15973,7 +15973,7 @@
         <v>130</v>
       </c>
       <c r="J302" s="11" t="n">
-        <v>0.8534</v>
+        <v>0.8538</v>
       </c>
       <c r="K302" s="8" t="n">
         <v>65</v>
@@ -16065,7 +16065,7 @@
         <v>1</v>
       </c>
       <c r="F304" s="10" t="n">
-        <v>14.96</v>
+        <v>14.95</v>
       </c>
       <c r="G304" s="8" t="n">
         <v>10</v>
@@ -16077,7 +16077,7 @@
         <v>310</v>
       </c>
       <c r="J304" s="11" t="n">
-        <v>0.9802</v>
+        <v>0.9806</v>
       </c>
       <c r="K304" s="8" t="n">
         <v>150</v>
@@ -16233,7 +16233,7 @@
         <v>110</v>
       </c>
       <c r="J307" s="11" t="n">
-        <v>0.9176</v>
+        <v>0.9182</v>
       </c>
       <c r="K307" s="8" t="n">
         <v>60</v>
@@ -16285,7 +16285,7 @@
         <v>210</v>
       </c>
       <c r="J308" s="11" t="n">
-        <v>0.9757</v>
+        <v>0.9762</v>
       </c>
       <c r="K308" s="8" t="n">
         <v>98</v>
@@ -16337,7 +16337,7 @@
         <v>79</v>
       </c>
       <c r="J309" s="11" t="n">
-        <v>0.9488</v>
+        <v>0.9494</v>
       </c>
       <c r="K309" s="8" t="n">
         <v>40</v>
@@ -16389,7 +16389,7 @@
         <v>110</v>
       </c>
       <c r="J310" s="11" t="n">
-        <v>0.9631999999999999</v>
+        <v>0.9636</v>
       </c>
       <c r="K310" s="8" t="n">
         <v>54</v>
@@ -16489,7 +16489,7 @@
         <v>1475</v>
       </c>
       <c r="J312" s="7" t="n">
-        <v>0.9772</v>
+        <v>0.9776</v>
       </c>
       <c r="K312" s="5" t="n">
         <v>735</v>
@@ -16749,7 +16749,7 @@
         <v>81</v>
       </c>
       <c r="J317" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9506</v>
       </c>
       <c r="K317" s="8" t="n">
         <v>40</v>
@@ -16801,7 +16801,7 @@
         <v>81</v>
       </c>
       <c r="J318" s="11" t="n">
-        <v>0.9502</v>
+        <v>0.9506</v>
       </c>
       <c r="K318" s="8" t="n">
         <v>40</v>
@@ -16853,7 +16853,7 @@
         <v>141</v>
       </c>
       <c r="J319" s="11" t="n">
-        <v>0.9923999999999999</v>
+        <v>0.9929</v>
       </c>
       <c r="K319" s="8" t="n">
         <v>70</v>
@@ -16905,7 +16905,7 @@
         <v>499</v>
       </c>
       <c r="J320" s="11" t="n">
-        <v>0.9713000000000001</v>
+        <v>0.9719</v>
       </c>
       <c r="K320" s="8" t="n">
         <v>250</v>
@@ -17009,7 +17009,7 @@
         <v>70</v>
       </c>
       <c r="J322" s="11" t="n">
-        <v>0.9566</v>
+        <v>0.9571</v>
       </c>
       <c r="K322" s="8" t="n">
         <v>35</v>
@@ -17113,7 +17113,7 @@
         <v>30</v>
       </c>
       <c r="J324" s="11" t="n">
-        <v>0.9998</v>
+        <v>1</v>
       </c>
       <c r="K324" s="8" t="n">
         <v>15</v>
@@ -17165,7 +17165,7 @@
         <v>18</v>
       </c>
       <c r="J325" s="11" t="n">
-        <v>0.9998</v>
+        <v>1</v>
       </c>
       <c r="K325" s="8" t="n">
         <v>10</v>
@@ -17373,7 +17373,7 @@
         <v>30</v>
       </c>
       <c r="J329" s="11" t="n">
-        <v>0.9997</v>
+        <v>1</v>
       </c>
       <c r="K329" s="8" t="n">
         <v>15</v>
@@ -17477,7 +17477,7 @@
         <v>30</v>
       </c>
       <c r="J331" s="11" t="n">
-        <v>0.9664</v>
+        <v>0.9667</v>
       </c>
       <c r="K331" s="8" t="n">
         <v>10</v>
@@ -17737,7 +17737,7 @@
         <v>60</v>
       </c>
       <c r="J336" s="11" t="n">
-        <v>0.983</v>
+        <v>0.9833</v>
       </c>
       <c r="K336" s="8" t="n">
         <v>30</v>
@@ -17789,7 +17789,7 @@
         <v>30</v>
       </c>
       <c r="J337" s="11" t="n">
-        <v>0.9997</v>
+        <v>1</v>
       </c>
       <c r="K337" s="8" t="n">
         <v>15</v>
@@ -17841,7 +17841,7 @@
         <v>30</v>
       </c>
       <c r="J338" s="11" t="n">
-        <v>0.9664</v>
+        <v>0.9667</v>
       </c>
       <c r="K338" s="8" t="n">
         <v>15</v>
@@ -17945,7 +17945,7 @@
         <v>30</v>
       </c>
       <c r="J340" s="11" t="n">
-        <v>0.9998</v>
+        <v>1</v>
       </c>
       <c r="K340" s="8" t="n">
         <v>15</v>
@@ -17993,7 +17993,7 @@
         <v>411</v>
       </c>
       <c r="J341" s="7" t="n">
-        <v>0.8731</v>
+        <v>0.8735000000000001</v>
       </c>
       <c r="K341" s="5" t="n">
         <v>205</v>
@@ -18045,7 +18045,7 @@
         <v>161</v>
       </c>
       <c r="J342" s="11" t="n">
-        <v>0.745</v>
+        <v>0.7453</v>
       </c>
       <c r="K342" s="8" t="n">
         <v>80</v>
@@ -18149,7 +18149,7 @@
         <v>60</v>
       </c>
       <c r="J344" s="11" t="n">
-        <v>0.9663</v>
+        <v>0.9667</v>
       </c>
       <c r="K344" s="8" t="n">
         <v>30</v>
@@ -18201,7 +18201,7 @@
         <v>150</v>
       </c>
       <c r="J345" s="11" t="n">
-        <v>0.9661</v>
+        <v>0.9667</v>
       </c>
       <c r="K345" s="8" t="n">
         <v>75</v>
@@ -18353,7 +18353,7 @@
         <v>1529</v>
       </c>
       <c r="J348" s="7" t="n">
-        <v>0.959</v>
+        <v>0.9595</v>
       </c>
       <c r="K348" s="5" t="n">
         <v>760</v>
@@ -18497,7 +18497,7 @@
         <v>1</v>
       </c>
       <c r="F351" s="10" t="n">
-        <v>14.55</v>
+        <v>14.54</v>
       </c>
       <c r="G351" s="8" t="n">
         <v>7</v>
@@ -18509,7 +18509,7 @@
         <v>182</v>
       </c>
       <c r="J351" s="11" t="n">
-        <v>0.9167999999999999</v>
+        <v>0.9176</v>
       </c>
       <c r="K351" s="8" t="n">
         <v>85</v>
@@ -18613,7 +18613,7 @@
         <v>387</v>
       </c>
       <c r="J353" s="11" t="n">
-        <v>0.9606</v>
+        <v>0.9612000000000001</v>
       </c>
       <c r="K353" s="8" t="n">
         <v>199</v>
@@ -18665,7 +18665,7 @@
         <v>70</v>
       </c>
       <c r="J354" s="11" t="n">
-        <v>0.9994</v>
+        <v>1</v>
       </c>
       <c r="K354" s="8" t="n">
         <v>35</v>
@@ -18769,7 +18769,7 @@
         <v>59</v>
       </c>
       <c r="J356" s="11" t="n">
-        <v>0.9992</v>
+        <v>1</v>
       </c>
       <c r="K356" s="8" t="n">
         <v>30</v>
@@ -18821,7 +18821,7 @@
         <v>81</v>
       </c>
       <c r="J357" s="11" t="n">
-        <v>0.9377</v>
+        <v>0.9383</v>
       </c>
       <c r="K357" s="8" t="n">
         <v>35</v>
@@ -18873,7 +18873,7 @@
         <v>60</v>
       </c>
       <c r="J358" s="11" t="n">
-        <v>0.9497</v>
+        <v>0.95</v>
       </c>
       <c r="K358" s="8" t="n">
         <v>30</v>
@@ -19029,7 +19029,7 @@
         <v>60</v>
       </c>
       <c r="J361" s="11" t="n">
-        <v>0.8997000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="K361" s="8" t="n">
         <v>30</v>
@@ -19081,7 +19081,7 @@
         <v>30</v>
       </c>
       <c r="J362" s="11" t="n">
-        <v>0.9665</v>
+        <v>0.9667</v>
       </c>
       <c r="K362" s="8" t="n">
         <v>15</v>
@@ -19237,7 +19237,7 @@
         <v>81</v>
       </c>
       <c r="J365" s="11" t="n">
-        <v>0.9131</v>
+        <v>0.9136</v>
       </c>
       <c r="K365" s="8" t="n">
         <v>40</v>
@@ -19289,7 +19289,7 @@
         <v>59</v>
       </c>
       <c r="J366" s="11" t="n">
-        <v>0.9993</v>
+        <v>1</v>
       </c>
       <c r="K366" s="8" t="n">
         <v>30</v>
@@ -19341,7 +19341,7 @@
         <v>70</v>
       </c>
       <c r="J367" s="11" t="n">
-        <v>0.9849</v>
+        <v>0.9857</v>
       </c>
       <c r="K367" s="8" t="n">
         <v>35</v>
@@ -19389,7 +19389,7 @@
         <v>69</v>
       </c>
       <c r="J368" s="7" t="n">
-        <v>0.9994</v>
+        <v>1</v>
       </c>
       <c r="K368" s="5" t="n">
         <v>35</v>
@@ -19441,7 +19441,7 @@
         <v>69</v>
       </c>
       <c r="J369" s="11" t="n">
-        <v>0.9994</v>
+        <v>1</v>
       </c>
       <c r="K369" s="8" t="n">
         <v>35</v>
@@ -19489,7 +19489,7 @@
         <v>4559</v>
       </c>
       <c r="J370" s="4" t="n">
-        <v>0.8364</v>
+        <v>0.8368</v>
       </c>
       <c r="K370" s="2" t="n">
         <v>2268</v>
@@ -19637,7 +19637,7 @@
         <v>240</v>
       </c>
       <c r="J373" s="7" t="n">
-        <v>0.9162</v>
+        <v>0.9167</v>
       </c>
       <c r="K373" s="5" t="n">
         <v>125</v>
@@ -19729,7 +19729,7 @@
         <v>1</v>
       </c>
       <c r="F375" s="10" t="n">
-        <v>14.85</v>
+        <v>14.84</v>
       </c>
       <c r="G375" s="8" t="n">
         <v>9</v>
@@ -19741,7 +19741,7 @@
         <v>190</v>
       </c>
       <c r="J375" s="11" t="n">
-        <v>0.931</v>
+        <v>0.9316</v>
       </c>
       <c r="K375" s="8" t="n">
         <v>100</v>
@@ -19789,7 +19789,7 @@
         <v>89</v>
       </c>
       <c r="J376" s="7" t="n">
-        <v>0.9095</v>
+        <v>0.9101</v>
       </c>
       <c r="K376" s="5" t="n">
         <v>45</v>
@@ -19841,7 +19841,7 @@
         <v>89</v>
       </c>
       <c r="J377" s="11" t="n">
-        <v>0.9095</v>
+        <v>0.9101</v>
       </c>
       <c r="K377" s="8" t="n">
         <v>45</v>
@@ -19889,7 +19889,7 @@
         <v>1314</v>
       </c>
       <c r="J378" s="7" t="n">
-        <v>0.8405</v>
+        <v>0.8409</v>
       </c>
       <c r="K378" s="5" t="n">
         <v>645</v>
@@ -19941,7 +19941,7 @@
         <v>99</v>
       </c>
       <c r="J379" s="11" t="n">
-        <v>0.8686</v>
+        <v>0.8687</v>
       </c>
       <c r="K379" s="8" t="n">
         <v>50</v>
@@ -19993,7 +19993,7 @@
         <v>30</v>
       </c>
       <c r="J380" s="11" t="n">
-        <v>0.7998</v>
+        <v>0.8</v>
       </c>
       <c r="K380" s="8" t="n">
         <v>15</v>
@@ -20045,7 +20045,7 @@
         <v>162</v>
       </c>
       <c r="J381" s="11" t="n">
-        <v>0.839</v>
+        <v>0.8395</v>
       </c>
       <c r="K381" s="8" t="n">
         <v>75</v>
@@ -20097,7 +20097,7 @@
         <v>192</v>
       </c>
       <c r="J382" s="11" t="n">
-        <v>0.8121</v>
+        <v>0.8125</v>
       </c>
       <c r="K382" s="8" t="n">
         <v>90</v>
@@ -20149,7 +20149,7 @@
         <v>270</v>
       </c>
       <c r="J383" s="11" t="n">
-        <v>0.8478</v>
+        <v>0.8481</v>
       </c>
       <c r="K383" s="8" t="n">
         <v>135</v>
@@ -20201,7 +20201,7 @@
         <v>364</v>
       </c>
       <c r="J384" s="11" t="n">
-        <v>0.8921</v>
+        <v>0.8929</v>
       </c>
       <c r="K384" s="8" t="n">
         <v>180</v>
@@ -20253,7 +20253,7 @@
         <v>119</v>
       </c>
       <c r="J385" s="11" t="n">
-        <v>0.8568</v>
+        <v>0.8571</v>
       </c>
       <c r="K385" s="8" t="n">
         <v>65</v>
@@ -20305,7 +20305,7 @@
         <v>78</v>
       </c>
       <c r="J386" s="11" t="n">
-        <v>0.6022999999999999</v>
+        <v>0.6026</v>
       </c>
       <c r="K386" s="8" t="n">
         <v>35</v>
@@ -20453,7 +20453,7 @@
         <v>140</v>
       </c>
       <c r="J389" s="7" t="n">
-        <v>0.8998</v>
+        <v>0.9</v>
       </c>
       <c r="K389" s="5" t="n">
         <v>69</v>
@@ -20713,7 +20713,7 @@
         <v>60</v>
       </c>
       <c r="J394" s="11" t="n">
-        <v>0.9495</v>
+        <v>0.95</v>
       </c>
       <c r="K394" s="8" t="n">
         <v>30</v>
@@ -20761,7 +20761,7 @@
         <v>612</v>
       </c>
       <c r="J395" s="7" t="n">
-        <v>0.8331</v>
+        <v>0.8333</v>
       </c>
       <c r="K395" s="5" t="n">
         <v>305</v>
@@ -20917,7 +20917,7 @@
         <v>152</v>
       </c>
       <c r="J398" s="11" t="n">
-        <v>0.835</v>
+        <v>0.8355</v>
       </c>
       <c r="K398" s="8" t="n">
         <v>80</v>
@@ -21113,7 +21113,7 @@
         <v>1</v>
       </c>
       <c r="F402" s="10" t="n">
-        <v>13.63</v>
+        <v>13.62</v>
       </c>
       <c r="G402" s="8" t="n">
         <v>8</v>
@@ -21125,7 +21125,7 @@
         <v>180</v>
       </c>
       <c r="J402" s="11" t="n">
-        <v>0.8607</v>
+        <v>0.8611</v>
       </c>
       <c r="K402" s="8" t="n">
         <v>90</v>
@@ -21277,7 +21277,7 @@
         <v>240</v>
       </c>
       <c r="J405" s="7" t="n">
-        <v>0.9789</v>
+        <v>0.9792</v>
       </c>
       <c r="K405" s="5" t="n">
         <v>120</v>
@@ -21329,7 +21329,7 @@
         <v>11</v>
       </c>
       <c r="J406" s="11" t="n">
-        <v>0.9999</v>
+        <v>1</v>
       </c>
       <c r="K406" s="8" t="n">
         <v>5</v>
@@ -21485,7 +21485,7 @@
         <v>30</v>
       </c>
       <c r="J409" s="11" t="n">
-        <v>0.9663</v>
+        <v>0.9667</v>
       </c>
       <c r="K409" s="8" t="n">
         <v>15</v>
@@ -21589,7 +21589,7 @@
         <v>59</v>
       </c>
       <c r="J411" s="11" t="n">
-        <v>0.9993</v>
+        <v>1</v>
       </c>
       <c r="K411" s="8" t="n">
         <v>30</v>
@@ -21641,7 +21641,7 @@
         <v>60</v>
       </c>
       <c r="J412" s="11" t="n">
-        <v>0.9831</v>
+        <v>0.9833</v>
       </c>
       <c r="K412" s="8" t="n">
         <v>30</v>
@@ -21689,7 +21689,7 @@
         <v>1163</v>
       </c>
       <c r="J413" s="7" t="n">
-        <v>0.7813</v>
+        <v>0.7816</v>
       </c>
       <c r="K413" s="5" t="n">
         <v>598</v>
@@ -21741,7 +21741,7 @@
         <v>49</v>
       </c>
       <c r="J414" s="11" t="n">
-        <v>0.7548</v>
+        <v>0.7551</v>
       </c>
       <c r="K414" s="8" t="n">
         <v>25</v>
@@ -21793,7 +21793,7 @@
         <v>60</v>
       </c>
       <c r="J415" s="11" t="n">
-        <v>0.6329</v>
+        <v>0.6333</v>
       </c>
       <c r="K415" s="8" t="n">
         <v>25</v>
@@ -21949,7 +21949,7 @@
         <v>139</v>
       </c>
       <c r="J418" s="11" t="n">
-        <v>0.6903</v>
+        <v>0.6906</v>
       </c>
       <c r="K418" s="8" t="n">
         <v>65</v>
@@ -22001,7 +22001,7 @@
         <v>120</v>
       </c>
       <c r="J419" s="11" t="n">
-        <v>0.7329</v>
+        <v>0.7333</v>
       </c>
       <c r="K419" s="8" t="n">
         <v>64</v>
@@ -22053,7 +22053,7 @@
         <v>19</v>
       </c>
       <c r="J420" s="11" t="n">
-        <v>0.8945</v>
+        <v>0.8947000000000001</v>
       </c>
       <c r="K420" s="8" t="n">
         <v>10</v>
@@ -22209,7 +22209,7 @@
         <v>120</v>
       </c>
       <c r="J423" s="11" t="n">
-        <v>0.8915999999999999</v>
+        <v>0.8917</v>
       </c>
       <c r="K423" s="8" t="n">
         <v>65</v>
@@ -22313,7 +22313,7 @@
         <v>59</v>
       </c>
       <c r="J425" s="11" t="n">
-        <v>0.6606</v>
+        <v>0.661</v>
       </c>
       <c r="K425" s="8" t="n">
         <v>25</v>
@@ -22365,7 +22365,7 @@
         <v>119</v>
       </c>
       <c r="J426" s="11" t="n">
-        <v>0.8905</v>
+        <v>0.8908</v>
       </c>
       <c r="K426" s="8" t="n">
         <v>60</v>
@@ -22417,7 +22417,7 @@
         <v>30</v>
       </c>
       <c r="J427" s="11" t="n">
-        <v>0.8996</v>
+        <v>0.9</v>
       </c>
       <c r="K427" s="8" t="n">
         <v>20</v>
@@ -22469,7 +22469,7 @@
         <v>91</v>
       </c>
       <c r="J428" s="11" t="n">
-        <v>0.8238</v>
+        <v>0.8242</v>
       </c>
       <c r="K428" s="8" t="n">
         <v>45</v>
@@ -22521,7 +22521,7 @@
         <v>117</v>
       </c>
       <c r="J429" s="11" t="n">
-        <v>0.8371</v>
+        <v>0.8376</v>
       </c>
       <c r="K429" s="8" t="n">
         <v>69</v>
@@ -22569,7 +22569,7 @@
         <v>430</v>
       </c>
       <c r="J430" s="7" t="n">
-        <v>0.8343</v>
+        <v>0.8349</v>
       </c>
       <c r="K430" s="5" t="n">
         <v>201</v>
@@ -22621,7 +22621,7 @@
         <v>190</v>
       </c>
       <c r="J431" s="11" t="n">
-        <v>0.7995</v>
+        <v>0.8</v>
       </c>
       <c r="K431" s="8" t="n">
         <v>90</v>
@@ -22673,7 +22673,7 @@
         <v>230</v>
       </c>
       <c r="J432" s="11" t="n">
-        <v>0.8732</v>
+        <v>0.8739</v>
       </c>
       <c r="K432" s="8" t="n">
         <v>106</v>
@@ -22773,7 +22773,7 @@
         <v>49</v>
       </c>
       <c r="J434" s="7" t="n">
-        <v>0.8976</v>
+        <v>0.898</v>
       </c>
       <c r="K434" s="5" t="n">
         <v>35</v>
@@ -22825,7 +22825,7 @@
         <v>49</v>
       </c>
       <c r="J435" s="11" t="n">
-        <v>0.8976</v>
+        <v>0.898</v>
       </c>
       <c r="K435" s="8" t="n">
         <v>35</v>
@@ -22861,7 +22861,7 @@
         <v>2</v>
       </c>
       <c r="F436" s="6" t="n">
-        <v>12.81</v>
+        <v>12.8</v>
       </c>
       <c r="G436" s="5" t="n">
         <v>8</v>
@@ -22873,7 +22873,7 @@
         <v>100</v>
       </c>
       <c r="J436" s="7" t="n">
-        <v>0.7296</v>
+        <v>0.73</v>
       </c>
       <c r="K436" s="5" t="n">
         <v>50</v>
@@ -22977,7 +22977,7 @@
         <v>90</v>
       </c>
       <c r="J438" s="11" t="n">
-        <v>0.6996</v>
+        <v>0.7</v>
       </c>
       <c r="K438" s="8" t="n">
         <v>45</v>
@@ -23025,7 +23025,7 @@
         <v>51</v>
       </c>
       <c r="J439" s="7" t="n">
-        <v>0.7645999999999999</v>
+        <v>0.7647</v>
       </c>
       <c r="K439" s="5" t="n">
         <v>20</v>
@@ -23129,7 +23129,7 @@
         <v>21</v>
       </c>
       <c r="J441" s="11" t="n">
-        <v>0.7616000000000001</v>
+        <v>0.7619</v>
       </c>
       <c r="K441" s="8" t="n">
         <v>5</v>
@@ -23301,7 +23301,7 @@
         <v>30</v>
       </c>
       <c r="J445" s="7" t="n">
-        <v>0.7664</v>
+        <v>0.7667</v>
       </c>
       <c r="K445" s="5" t="n">
         <v>10</v>
@@ -23353,7 +23353,7 @@
         <v>30</v>
       </c>
       <c r="J446" s="11" t="n">
-        <v>0.7664</v>
+        <v>0.7667</v>
       </c>
       <c r="K446" s="8" t="n">
         <v>10</v>
@@ -23437,7 +23437,7 @@
         <v>41</v>
       </c>
       <c r="J448" s="7" t="n">
-        <v>0.9996</v>
+        <v>1</v>
       </c>
       <c r="K448" s="5" t="n">
         <v>15</v>
@@ -23489,7 +23489,7 @@
         <v>41</v>
       </c>
       <c r="J449" s="11" t="n">
-        <v>0.9996</v>
+        <v>1</v>
       </c>
       <c r="K449" s="8" t="n">
         <v>15</v>
@@ -23673,7 +23673,7 @@
         <v>958</v>
       </c>
       <c r="J453" s="4" t="n">
-        <v>0.9516</v>
+        <v>0.952</v>
       </c>
       <c r="K453" s="2" t="n">
         <v>495</v>
@@ -23873,7 +23873,7 @@
         <v>149</v>
       </c>
       <c r="J457" s="7" t="n">
-        <v>0.9796</v>
+        <v>0.9799</v>
       </c>
       <c r="K457" s="5" t="n">
         <v>85</v>
@@ -24185,7 +24185,7 @@
         <v>60</v>
       </c>
       <c r="J463" s="11" t="n">
-        <v>0.9828</v>
+        <v>0.9833</v>
       </c>
       <c r="K463" s="8" t="n">
         <v>35</v>
@@ -24393,7 +24393,7 @@
         <v>9</v>
       </c>
       <c r="J467" s="11" t="n">
-        <v>0.9999</v>
+        <v>1</v>
       </c>
       <c r="K467" s="8" t="n">
         <v>5</v>
@@ -24441,7 +24441,7 @@
         <v>439</v>
       </c>
       <c r="J468" s="7" t="n">
-        <v>0.9678</v>
+        <v>0.9681</v>
       </c>
       <c r="K468" s="5" t="n">
         <v>225</v>
@@ -24493,7 +24493,7 @@
         <v>30</v>
       </c>
       <c r="J469" s="11" t="n">
-        <v>0.9997</v>
+        <v>1</v>
       </c>
       <c r="K469" s="8" t="n">
         <v>15</v>
@@ -24545,7 +24545,7 @@
         <v>9</v>
       </c>
       <c r="J470" s="11" t="n">
-        <v>0.8888</v>
+        <v>0.8889</v>
       </c>
       <c r="K470" s="8" t="n">
         <v>5</v>
@@ -24649,7 +24649,7 @@
         <v>30</v>
       </c>
       <c r="J472" s="11" t="n">
-        <v>0.9332</v>
+        <v>0.9333</v>
       </c>
       <c r="K472" s="8" t="n">
         <v>15</v>
@@ -24701,7 +24701,7 @@
         <v>70</v>
       </c>
       <c r="J473" s="11" t="n">
-        <v>0.9135</v>
+        <v>0.9143</v>
       </c>
       <c r="K473" s="8" t="n">
         <v>35</v>
@@ -24909,7 +24909,7 @@
         <v>90</v>
       </c>
       <c r="J477" s="11" t="n">
-        <v>0.9661</v>
+        <v>0.9667</v>
       </c>
       <c r="K477" s="8" t="n">
         <v>45</v>
@@ -25013,7 +25013,7 @@
         <v>30</v>
       </c>
       <c r="J479" s="11" t="n">
-        <v>0.9997</v>
+        <v>1</v>
       </c>
       <c r="K479" s="8" t="n">
         <v>15</v>
@@ -25065,7 +25065,7 @@
         <v>30</v>
       </c>
       <c r="J480" s="11" t="n">
-        <v>0.9998</v>
+        <v>1</v>
       </c>
       <c r="K480" s="8" t="n">
         <v>15</v>
@@ -25113,7 +25113,7 @@
         <v>160</v>
       </c>
       <c r="J481" s="7" t="n">
-        <v>0.9059</v>
+        <v>0.9062</v>
       </c>
       <c r="K481" s="5" t="n">
         <v>80</v>
@@ -25165,7 +25165,7 @@
         <v>30</v>
       </c>
       <c r="J482" s="11" t="n">
-        <v>0.9997</v>
+        <v>1</v>
       </c>
       <c r="K482" s="8" t="n">
         <v>15</v>
@@ -25217,7 +25217,7 @@
         <v>130</v>
       </c>
       <c r="J483" s="11" t="n">
-        <v>0.8842</v>
+        <v>0.8846000000000001</v>
       </c>
       <c r="K483" s="8" t="n">
         <v>65</v>
@@ -25365,7 +25365,7 @@
         <v>30</v>
       </c>
       <c r="J486" s="7" t="n">
-        <v>0.833</v>
+        <v>0.8333</v>
       </c>
       <c r="K486" s="5" t="n">
         <v>15</v>
@@ -25417,7 +25417,7 @@
         <v>30</v>
       </c>
       <c r="J487" s="11" t="n">
-        <v>0.833</v>
+        <v>0.8333</v>
       </c>
       <c r="K487" s="8" t="n">
         <v>15</v>
@@ -25465,7 +25465,7 @@
         <v>110</v>
       </c>
       <c r="J488" s="7" t="n">
-        <v>0.9537</v>
+        <v>0.9545</v>
       </c>
       <c r="K488" s="5" t="n">
         <v>55</v>
@@ -25517,7 +25517,7 @@
         <v>110</v>
       </c>
       <c r="J489" s="11" t="n">
-        <v>0.9537</v>
+        <v>0.9545</v>
       </c>
       <c r="K489" s="8" t="n">
         <v>55</v>
@@ -25565,7 +25565,7 @@
         <v>473</v>
       </c>
       <c r="J490" s="4" t="n">
-        <v>0.9532</v>
+        <v>0.9535</v>
       </c>
       <c r="K490" s="2" t="n">
         <v>245</v>
@@ -25813,7 +25813,7 @@
         <v>443</v>
       </c>
       <c r="J495" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9503</v>
       </c>
       <c r="K495" s="5" t="n">
         <v>230</v>
@@ -25917,7 +25917,7 @@
         <v>59</v>
       </c>
       <c r="J497" s="11" t="n">
-        <v>0.847</v>
+        <v>0.8475</v>
       </c>
       <c r="K497" s="8" t="n">
         <v>30</v>
@@ -26073,7 +26073,7 @@
         <v>60</v>
       </c>
       <c r="J500" s="11" t="n">
-        <v>0.983</v>
+        <v>0.9833</v>
       </c>
       <c r="K500" s="8" t="n">
         <v>30</v>
@@ -26125,7 +26125,7 @@
         <v>15</v>
       </c>
       <c r="J501" s="11" t="n">
-        <v>0.9997</v>
+        <v>1</v>
       </c>
       <c r="K501" s="8" t="n">
         <v>15</v>
@@ -26229,7 +26229,7 @@
         <v>59</v>
       </c>
       <c r="J503" s="11" t="n">
-        <v>0.9994</v>
+        <v>1</v>
       </c>
       <c r="K503" s="8" t="n">
         <v>30</v>
@@ -26333,7 +26333,7 @@
         <v>70</v>
       </c>
       <c r="J505" s="11" t="n">
-        <v>0.9993</v>
+        <v>1</v>
       </c>
       <c r="K505" s="8" t="n">
         <v>35</v>
@@ -26381,7 +26381,7 @@
         <v>1851</v>
       </c>
       <c r="J506" s="4" t="n">
-        <v>0.8333</v>
+        <v>0.8336</v>
       </c>
       <c r="K506" s="2" t="n">
         <v>903</v>
@@ -26585,7 +26585,7 @@
         <v>15</v>
       </c>
       <c r="J510" s="11" t="n">
-        <v>0.3999</v>
+        <v>0.4</v>
       </c>
       <c r="K510" s="8" t="n">
         <v>5</v>
@@ -26685,7 +26685,7 @@
         <v>63</v>
       </c>
       <c r="J512" s="7" t="n">
-        <v>0.9201</v>
+        <v>0.9206</v>
       </c>
       <c r="K512" s="5" t="n">
         <v>30</v>
@@ -26737,7 +26737,7 @@
         <v>63</v>
       </c>
       <c r="J513" s="11" t="n">
-        <v>0.9201</v>
+        <v>0.9206</v>
       </c>
       <c r="K513" s="8" t="n">
         <v>30</v>
@@ -26785,7 +26785,7 @@
         <v>528</v>
       </c>
       <c r="J514" s="7" t="n">
-        <v>0.8576</v>
+        <v>0.858</v>
       </c>
       <c r="K514" s="5" t="n">
         <v>265</v>
@@ -26837,7 +26837,7 @@
         <v>189</v>
       </c>
       <c r="J515" s="11" t="n">
-        <v>0.92</v>
+        <v>0.9206</v>
       </c>
       <c r="K515" s="8" t="n">
         <v>100</v>
@@ -26941,7 +26941,7 @@
         <v>49</v>
       </c>
       <c r="J517" s="11" t="n">
-        <v>0.9589</v>
+        <v>0.9592000000000001</v>
       </c>
       <c r="K517" s="8" t="n">
         <v>25</v>
@@ -26993,7 +26993,7 @@
         <v>150</v>
       </c>
       <c r="J518" s="11" t="n">
-        <v>0.7331</v>
+        <v>0.7333</v>
       </c>
       <c r="K518" s="8" t="n">
         <v>75</v>
@@ -27033,7 +27033,7 @@
         <v>1</v>
       </c>
       <c r="F519" s="10" t="n">
-        <v>13.63</v>
+        <v>13.62</v>
       </c>
       <c r="G519" s="8" t="n">
         <v>7</v>
@@ -27045,7 +27045,7 @@
         <v>120</v>
       </c>
       <c r="J519" s="11" t="n">
-        <v>0.8666</v>
+        <v>0.8667</v>
       </c>
       <c r="K519" s="8" t="n">
         <v>55</v>
@@ -27129,7 +27129,7 @@
         <v>346</v>
       </c>
       <c r="J521" s="7" t="n">
-        <v>0.8321</v>
+        <v>0.8324</v>
       </c>
       <c r="K521" s="5" t="n">
         <v>170</v>
@@ -27337,7 +27337,7 @@
         <v>261</v>
       </c>
       <c r="J525" s="11" t="n">
-        <v>0.8004</v>
+        <v>0.8008</v>
       </c>
       <c r="K525" s="8" t="n">
         <v>125</v>
@@ -27437,7 +27437,7 @@
         <v>139</v>
       </c>
       <c r="J527" s="7" t="n">
-        <v>0.8484</v>
+        <v>0.8489</v>
       </c>
       <c r="K527" s="5" t="n">
         <v>70</v>
@@ -27489,7 +27489,7 @@
         <v>70</v>
       </c>
       <c r="J528" s="11" t="n">
-        <v>0.8567</v>
+        <v>0.8571</v>
       </c>
       <c r="K528" s="8" t="n">
         <v>35</v>
@@ -27541,7 +27541,7 @@
         <v>69</v>
       </c>
       <c r="J529" s="11" t="n">
-        <v>0.84</v>
+        <v>0.8406</v>
       </c>
       <c r="K529" s="8" t="n">
         <v>35</v>
@@ -27777,7 +27777,7 @@
         <v>80</v>
       </c>
       <c r="J534" s="7" t="n">
-        <v>0.8373</v>
+        <v>0.8375</v>
       </c>
       <c r="K534" s="5" t="n">
         <v>38</v>
@@ -27829,7 +27829,7 @@
         <v>60</v>
       </c>
       <c r="J535" s="11" t="n">
-        <v>0.8831</v>
+        <v>0.8833</v>
       </c>
       <c r="K535" s="8" t="n">
         <v>28</v>
@@ -27929,7 +27929,7 @@
         <v>410</v>
       </c>
       <c r="J537" s="7" t="n">
-        <v>0.8754</v>
+        <v>0.8756</v>
       </c>
       <c r="K537" s="5" t="n">
         <v>200</v>
@@ -27981,7 +27981,7 @@
         <v>90</v>
       </c>
       <c r="J538" s="11" t="n">
-        <v>0.8331</v>
+        <v>0.8333</v>
       </c>
       <c r="K538" s="8" t="n">
         <v>40</v>
@@ -28033,7 +28033,7 @@
         <v>51</v>
       </c>
       <c r="J539" s="11" t="n">
-        <v>0.8233</v>
+        <v>0.8235</v>
       </c>
       <c r="K539" s="8" t="n">
         <v>25</v>
@@ -28085,7 +28085,7 @@
         <v>49</v>
       </c>
       <c r="J540" s="11" t="n">
-        <v>0.9996</v>
+        <v>1</v>
       </c>
       <c r="K540" s="8" t="n">
         <v>25</v>
@@ -28137,7 +28137,7 @@
         <v>30</v>
       </c>
       <c r="J541" s="11" t="n">
-        <v>0.9999</v>
+        <v>1</v>
       </c>
       <c r="K541" s="8" t="n">
         <v>15</v>
@@ -28241,7 +28241,7 @@
         <v>90</v>
       </c>
       <c r="J543" s="11" t="n">
-        <v>0.9442</v>
+        <v>0.9444</v>
       </c>
       <c r="K543" s="8" t="n">
         <v>45</v>
@@ -28445,7 +28445,7 @@
         <v>180</v>
       </c>
       <c r="J547" s="7" t="n">
-        <v>0.6166</v>
+        <v>0.6167</v>
       </c>
       <c r="K547" s="5" t="n">
         <v>85</v>
@@ -28549,7 +28549,7 @@
         <v>70</v>
       </c>
       <c r="J549" s="11" t="n">
-        <v>0.4713</v>
+        <v>0.4714</v>
       </c>
       <c r="K549" s="8" t="n">
         <v>30</v>
@@ -28637,7 +28637,7 @@
         <v>29</v>
       </c>
       <c r="F551" s="3" t="n">
-        <v>14.1</v>
+        <v>13.94</v>
       </c>
       <c r="G551" s="2" t="n">
         <v>7</v>
@@ -28646,10 +28646,10 @@
         <v>19</v>
       </c>
       <c r="I551" s="2" t="n">
-        <v>3175</v>
+        <v>3683</v>
       </c>
       <c r="J551" s="4" t="n">
-        <v>0.9066</v>
+        <v>0.8914</v>
       </c>
       <c r="K551" s="2" t="n">
         <v>929</v>
@@ -28697,7 +28697,7 @@
         <v>917</v>
       </c>
       <c r="J552" s="7" t="n">
-        <v>0.9167999999999999</v>
+        <v>0.9171</v>
       </c>
       <c r="K552" s="5" t="n">
         <v>225</v>
@@ -28749,7 +28749,7 @@
         <v>60</v>
       </c>
       <c r="J553" s="11" t="n">
-        <v>0.983</v>
+        <v>0.9833</v>
       </c>
       <c r="K553" s="8" t="n">
         <v>15</v>
@@ -28905,7 +28905,7 @@
         <v>60</v>
       </c>
       <c r="J556" s="11" t="n">
-        <v>0.9664</v>
+        <v>0.9667</v>
       </c>
       <c r="K556" s="8" t="n">
         <v>15</v>
@@ -29009,7 +29009,7 @@
         <v>260</v>
       </c>
       <c r="J558" s="11" t="n">
-        <v>0.9532</v>
+        <v>0.9538</v>
       </c>
       <c r="K558" s="8" t="n">
         <v>65</v>
@@ -29159,7 +29159,7 @@
         <v>59</v>
       </c>
       <c r="J561" s="11" t="n">
-        <v>0.9488</v>
+        <v>0.9492</v>
       </c>
       <c r="K561" s="8" t="n">
         <v>15</v>
@@ -29211,7 +29211,7 @@
         <v>98</v>
       </c>
       <c r="J562" s="11" t="n">
-        <v>0.8671</v>
+        <v>0.8673</v>
       </c>
       <c r="K562" s="8" t="n">
         <v>25</v>
@@ -29259,7 +29259,7 @@
         <v>79</v>
       </c>
       <c r="J563" s="7" t="n">
-        <v>0.9743000000000001</v>
+        <v>0.9747</v>
       </c>
       <c r="K563" s="5" t="n">
         <v>20</v>
@@ -29311,7 +29311,7 @@
         <v>79</v>
       </c>
       <c r="J564" s="11" t="n">
-        <v>0.9743000000000001</v>
+        <v>0.9747</v>
       </c>
       <c r="K564" s="8" t="n">
         <v>20</v>
@@ -29347,7 +29347,7 @@
         <v>19</v>
       </c>
       <c r="F565" s="6" t="n">
-        <v>13.91</v>
+        <v>13.73</v>
       </c>
       <c r="G565" s="5" t="n">
         <v>7</v>
@@ -29356,10 +29356,10 @@
         <v>18</v>
       </c>
       <c r="I565" s="5" t="n">
-        <v>2179</v>
+        <v>2687</v>
       </c>
       <c r="J565" s="7" t="n">
-        <v>0.8998</v>
+        <v>0.8802</v>
       </c>
       <c r="K565" s="5" t="n">
         <v>684</v>
@@ -29411,7 +29411,7 @@
         <v>180</v>
       </c>
       <c r="J566" s="11" t="n">
-        <v>0.905</v>
+        <v>0.9056</v>
       </c>
       <c r="K566" s="8" t="n">
         <v>45</v>
@@ -29463,7 +29463,7 @@
         <v>160</v>
       </c>
       <c r="J567" s="11" t="n">
-        <v>0.9247</v>
+        <v>0.925</v>
       </c>
       <c r="K567" s="8" t="n">
         <v>40</v>
@@ -29555,7 +29555,7 @@
         <v>1</v>
       </c>
       <c r="F569" s="10" t="n">
-        <v>13.76</v>
+        <v>13.75</v>
       </c>
       <c r="G569" s="8" t="n">
         <v>8</v>
@@ -29567,7 +29567,7 @@
         <v>179</v>
       </c>
       <c r="J569" s="11" t="n">
-        <v>0.8931</v>
+        <v>0.8939</v>
       </c>
       <c r="K569" s="8" t="n">
         <v>45</v>
@@ -29619,7 +29619,7 @@
         <v>120</v>
       </c>
       <c r="J570" s="11" t="n">
-        <v>0.9331</v>
+        <v>0.9333</v>
       </c>
       <c r="K570" s="8" t="n">
         <v>30</v>
@@ -29671,7 +29671,7 @@
         <v>120</v>
       </c>
       <c r="J571" s="11" t="n">
-        <v>0.8164</v>
+        <v>0.8167</v>
       </c>
       <c r="K571" s="8" t="n">
         <v>30</v>
@@ -29723,7 +29723,7 @@
         <v>141</v>
       </c>
       <c r="J572" s="11" t="n">
-        <v>0.9213</v>
+        <v>0.922</v>
       </c>
       <c r="K572" s="8" t="n">
         <v>35</v>
@@ -29918,10 +29918,10 @@
         <v>18</v>
       </c>
       <c r="I576" s="8" t="n">
-        <v>100</v>
+        <v>608</v>
       </c>
       <c r="J576" s="11" t="n">
-        <v>0.7938</v>
+        <v>0.7944</v>
       </c>
       <c r="K576" s="8" t="n">
         <v>144</v>
@@ -29973,7 +29973,7 @@
         <v>140</v>
       </c>
       <c r="J577" s="11" t="n">
-        <v>0.9137999999999999</v>
+        <v>0.9143</v>
       </c>
       <c r="K577" s="8" t="n">
         <v>30</v>
@@ -30025,7 +30025,7 @@
         <v>99</v>
       </c>
       <c r="J578" s="11" t="n">
-        <v>0.9393</v>
+        <v>0.9394</v>
       </c>
       <c r="K578" s="8" t="n">
         <v>30</v>
@@ -30077,7 +30077,7 @@
         <v>180</v>
       </c>
       <c r="J579" s="11" t="n">
-        <v>0.8552999999999999</v>
+        <v>0.8556</v>
       </c>
       <c r="K579" s="8" t="n">
         <v>45</v>
@@ -30129,7 +30129,7 @@
         <v>120</v>
       </c>
       <c r="J580" s="11" t="n">
-        <v>0.9247</v>
+        <v>0.925</v>
       </c>
       <c r="K580" s="8" t="n">
         <v>30</v>
@@ -30233,7 +30233,7 @@
         <v>220</v>
       </c>
       <c r="J582" s="11" t="n">
-        <v>0.9675</v>
+        <v>0.9681999999999999</v>
       </c>
       <c r="K582" s="8" t="n">
         <v>55</v>
@@ -30420,7 +30420,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Muestras azúcar (estim.)</t>
+          <t>Muestras azúcar (deducidas)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -30481,7 +30481,7 @@
         <v>95</v>
       </c>
       <c r="I2" s="11" t="n">
-        <v>0.6943</v>
+        <v>0.6947</v>
       </c>
       <c r="J2" s="8" t="n">
         <v>45</v>
@@ -30528,7 +30528,7 @@
         <v>165</v>
       </c>
       <c r="I3" s="14" t="n">
-        <v>0.6906</v>
+        <v>0.6909</v>
       </c>
       <c r="J3" s="12" t="n">
         <v>80</v>
@@ -30575,7 +30575,7 @@
         <v>664</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>0.8431</v>
+        <v>0.8434</v>
       </c>
       <c r="J4" s="8" t="n">
         <v>319</v>
@@ -30622,7 +30622,7 @@
         <v>1290</v>
       </c>
       <c r="I5" s="14" t="n">
-        <v>0.7485000000000001</v>
+        <v>0.7488</v>
       </c>
       <c r="J5" s="12" t="n">
         <v>580</v>
@@ -30669,7 +30669,7 @@
         <v>401</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0.8997000000000001</v>
+        <v>0.9002</v>
       </c>
       <c r="J6" s="8" t="n">
         <v>194</v>
@@ -30716,7 +30716,7 @@
         <v>543</v>
       </c>
       <c r="I7" s="14" t="n">
-        <v>0.9371</v>
+        <v>0.9374</v>
       </c>
       <c r="J7" s="12" t="n">
         <v>264</v>
@@ -30763,7 +30763,7 @@
         <v>452</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0.6788</v>
+        <v>0.6792</v>
       </c>
       <c r="J8" s="8" t="n">
         <v>214</v>
@@ -30810,7 +30810,7 @@
         <v>866</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>0.8793</v>
+        <v>0.8799</v>
       </c>
       <c r="J9" s="12" t="n">
         <v>400</v>
@@ -30857,7 +30857,7 @@
         <v>1000</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>0.7796999999999999</v>
+        <v>0.78</v>
       </c>
       <c r="J10" s="8" t="n">
         <v>460</v>
@@ -30892,7 +30892,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>14.15</v>
+        <v>14.14</v>
       </c>
       <c r="F11" s="12" t="n">
         <v>8</v>
@@ -30904,7 +30904,7 @@
         <v>1000</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>0.9386</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="J11" s="12" t="n">
         <v>509</v>
@@ -30951,7 +30951,7 @@
         <v>155</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>0.8127</v>
+        <v>0.8129</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>75</v>
@@ -30998,7 +30998,7 @@
         <v>281</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>0.8929</v>
+        <v>0.8932</v>
       </c>
       <c r="J13" s="12" t="n">
         <v>135</v>
@@ -31045,7 +31045,7 @@
         <v>314</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>0.834</v>
+        <v>0.8344</v>
       </c>
       <c r="J14" s="8" t="n">
         <v>150</v>
@@ -31092,7 +31092,7 @@
         <v>30</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>0.6663</v>
+        <v>0.6667</v>
       </c>
       <c r="J15" s="12" t="n">
         <v>15</v>
@@ -31280,7 +31280,7 @@
         <v>81</v>
       </c>
       <c r="I19" s="14" t="n">
-        <v>0.901</v>
+        <v>0.9012</v>
       </c>
       <c r="J19" s="12" t="n">
         <v>34</v>
@@ -31421,7 +31421,7 @@
         <v>323</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>0.7894</v>
+        <v>0.7895</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>80</v>
@@ -31456,7 +31456,7 @@
         <v>10</v>
       </c>
       <c r="E23" s="13" t="n">
-        <v>13.86</v>
+        <v>14.08</v>
       </c>
       <c r="F23" s="12" t="n">
         <v>5</v>
@@ -31465,10 +31465,10 @@
         <v>18</v>
       </c>
       <c r="H23" s="12" t="n">
-        <v>1238</v>
+        <v>1855</v>
       </c>
       <c r="I23" s="14" t="n">
-        <v>0.8502</v>
+        <v>0.8836000000000001</v>
       </c>
       <c r="J23" s="12" t="n">
         <v>305</v>
@@ -31515,7 +31515,7 @@
         <v>747</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>0.7749</v>
+        <v>0.7751</v>
       </c>
       <c r="J24" s="8" t="n">
         <v>170</v>
@@ -31550,7 +31550,7 @@
         <v>33</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>13.11</v>
+        <v>13.1</v>
       </c>
       <c r="F25" s="12" t="n">
         <v>5</v>
@@ -31562,7 +31562,7 @@
         <v>4126</v>
       </c>
       <c r="I25" s="14" t="n">
-        <v>0.7825</v>
+        <v>0.7828000000000001</v>
       </c>
       <c r="J25" s="12" t="n">
         <v>985</v>
@@ -31609,7 +31609,7 @@
         <v>219</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>0.9404</v>
+        <v>0.9406</v>
       </c>
       <c r="J26" s="8" t="n">
         <v>55</v>
@@ -31644,7 +31644,7 @@
         <v>11</v>
       </c>
       <c r="E27" s="13" t="n">
-        <v>13.9</v>
+        <v>13.65</v>
       </c>
       <c r="F27" s="12" t="n">
         <v>6</v>
@@ -31653,10 +31653,10 @@
         <v>18</v>
       </c>
       <c r="H27" s="12" t="n">
-        <v>1200</v>
+        <v>1791</v>
       </c>
       <c r="I27" s="14" t="n">
-        <v>0.8599</v>
+        <v>0.8219</v>
       </c>
       <c r="J27" s="12" t="n">
         <v>435</v>
@@ -31738,7 +31738,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="13" t="n">
-        <v>13.85</v>
+        <v>13.76</v>
       </c>
       <c r="F29" s="12" t="n">
         <v>5</v>
@@ -31747,10 +31747,10 @@
         <v>19</v>
       </c>
       <c r="H29" s="12" t="n">
-        <v>200</v>
+        <v>1450</v>
       </c>
       <c r="I29" s="14" t="n">
-        <v>0.8192</v>
+        <v>0.8193</v>
       </c>
       <c r="J29" s="12" t="n">
         <v>314</v>
@@ -31797,7 +31797,7 @@
         <v>60</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>0.7163</v>
+        <v>0.7167</v>
       </c>
       <c r="J30" s="8" t="n">
         <v>15</v>
@@ -31938,7 +31938,7 @@
         <v>522</v>
       </c>
       <c r="I33" s="14" t="n">
-        <v>0.9076</v>
+        <v>0.908</v>
       </c>
       <c r="J33" s="12" t="n">
         <v>130</v>
@@ -31985,7 +31985,7 @@
         <v>608</v>
       </c>
       <c r="I34" s="11" t="n">
-        <v>0.7742</v>
+        <v>0.7747000000000001</v>
       </c>
       <c r="J34" s="8" t="n">
         <v>135</v>
@@ -32032,7 +32032,7 @@
         <v>703</v>
       </c>
       <c r="I35" s="14" t="n">
-        <v>0.8942</v>
+        <v>0.8947000000000001</v>
       </c>
       <c r="J35" s="12" t="n">
         <v>160</v>
@@ -32079,7 +32079,7 @@
         <v>439</v>
       </c>
       <c r="I36" s="11" t="n">
-        <v>0.7539</v>
+        <v>0.754</v>
       </c>
       <c r="J36" s="8" t="n">
         <v>134</v>
@@ -32126,7 +32126,7 @@
         <v>460</v>
       </c>
       <c r="I37" s="14" t="n">
-        <v>0.8451</v>
+        <v>0.8457</v>
       </c>
       <c r="J37" s="12" t="n">
         <v>120</v>
@@ -32173,7 +32173,7 @@
         <v>430</v>
       </c>
       <c r="I38" s="11" t="n">
-        <v>0.8065</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="J38" s="8" t="n">
         <v>99</v>
@@ -32267,7 +32267,7 @@
         <v>1842</v>
       </c>
       <c r="I40" s="11" t="n">
-        <v>0.9550999999999999</v>
+        <v>0.9555</v>
       </c>
       <c r="J40" s="8" t="n">
         <v>914</v>
@@ -32314,7 +32314,7 @@
         <v>660</v>
       </c>
       <c r="I41" s="14" t="n">
-        <v>0.8695000000000001</v>
+        <v>0.8697</v>
       </c>
       <c r="J41" s="12" t="n">
         <v>343</v>
@@ -32361,7 +32361,7 @@
         <v>1409</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>0.9081</v>
+        <v>0.9084</v>
       </c>
       <c r="J42" s="8" t="n">
         <v>697</v>
@@ -32408,7 +32408,7 @@
         <v>1475</v>
       </c>
       <c r="I43" s="14" t="n">
-        <v>0.9772</v>
+        <v>0.9776</v>
       </c>
       <c r="J43" s="12" t="n">
         <v>735</v>
@@ -32455,7 +32455,7 @@
         <v>411</v>
       </c>
       <c r="I44" s="11" t="n">
-        <v>0.8731</v>
+        <v>0.8735000000000001</v>
       </c>
       <c r="J44" s="8" t="n">
         <v>205</v>
@@ -32502,7 +32502,7 @@
         <v>1529</v>
       </c>
       <c r="I45" s="14" t="n">
-        <v>0.959</v>
+        <v>0.9595</v>
       </c>
       <c r="J45" s="12" t="n">
         <v>760</v>
@@ -32549,7 +32549,7 @@
         <v>69</v>
       </c>
       <c r="I46" s="11" t="n">
-        <v>0.9994</v>
+        <v>1</v>
       </c>
       <c r="J46" s="8" t="n">
         <v>35</v>
@@ -32643,7 +32643,7 @@
         <v>240</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>0.9162</v>
+        <v>0.9167</v>
       </c>
       <c r="J48" s="8" t="n">
         <v>125</v>
@@ -32690,7 +32690,7 @@
         <v>89</v>
       </c>
       <c r="I49" s="14" t="n">
-        <v>0.9095</v>
+        <v>0.9101</v>
       </c>
       <c r="J49" s="12" t="n">
         <v>45</v>
@@ -32737,7 +32737,7 @@
         <v>1314</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>0.8405</v>
+        <v>0.8409</v>
       </c>
       <c r="J50" s="8" t="n">
         <v>645</v>
@@ -32831,7 +32831,7 @@
         <v>140</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>0.8998</v>
+        <v>0.9</v>
       </c>
       <c r="J52" s="8" t="n">
         <v>69</v>
@@ -32878,7 +32878,7 @@
         <v>612</v>
       </c>
       <c r="I53" s="14" t="n">
-        <v>0.8331</v>
+        <v>0.8333</v>
       </c>
       <c r="J53" s="12" t="n">
         <v>305</v>
@@ -32925,7 +32925,7 @@
         <v>240</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>0.9789</v>
+        <v>0.9792</v>
       </c>
       <c r="J54" s="8" t="n">
         <v>120</v>
@@ -32972,7 +32972,7 @@
         <v>1163</v>
       </c>
       <c r="I55" s="14" t="n">
-        <v>0.7813</v>
+        <v>0.7816</v>
       </c>
       <c r="J55" s="12" t="n">
         <v>598</v>
@@ -33019,7 +33019,7 @@
         <v>430</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>0.8343</v>
+        <v>0.8349</v>
       </c>
       <c r="J56" s="8" t="n">
         <v>201</v>
@@ -33066,7 +33066,7 @@
         <v>49</v>
       </c>
       <c r="I57" s="14" t="n">
-        <v>0.8976</v>
+        <v>0.898</v>
       </c>
       <c r="J57" s="12" t="n">
         <v>35</v>
@@ -33101,7 +33101,7 @@
         <v>2</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>12.81</v>
+        <v>12.8</v>
       </c>
       <c r="F58" s="8" t="n">
         <v>8</v>
@@ -33113,7 +33113,7 @@
         <v>100</v>
       </c>
       <c r="I58" s="11" t="n">
-        <v>0.7296</v>
+        <v>0.73</v>
       </c>
       <c r="J58" s="8" t="n">
         <v>50</v>
@@ -33160,7 +33160,7 @@
         <v>51</v>
       </c>
       <c r="I59" s="14" t="n">
-        <v>0.7645999999999999</v>
+        <v>0.7647</v>
       </c>
       <c r="J59" s="12" t="n">
         <v>20</v>
@@ -33207,7 +33207,7 @@
         <v>30</v>
       </c>
       <c r="I60" s="11" t="n">
-        <v>0.7664</v>
+        <v>0.7667</v>
       </c>
       <c r="J60" s="8" t="n">
         <v>10</v>
@@ -33254,7 +33254,7 @@
         <v>41</v>
       </c>
       <c r="I61" s="14" t="n">
-        <v>0.9996</v>
+        <v>1</v>
       </c>
       <c r="J61" s="12" t="n">
         <v>15</v>
@@ -33395,7 +33395,7 @@
         <v>149</v>
       </c>
       <c r="I64" s="11" t="n">
-        <v>0.9796</v>
+        <v>0.9799</v>
       </c>
       <c r="J64" s="8" t="n">
         <v>85</v>
@@ -33442,7 +33442,7 @@
         <v>439</v>
       </c>
       <c r="I65" s="14" t="n">
-        <v>0.9678</v>
+        <v>0.9681</v>
       </c>
       <c r="J65" s="12" t="n">
         <v>225</v>
@@ -33489,7 +33489,7 @@
         <v>160</v>
       </c>
       <c r="I66" s="11" t="n">
-        <v>0.9059</v>
+        <v>0.9062</v>
       </c>
       <c r="J66" s="8" t="n">
         <v>80</v>
@@ -33583,7 +33583,7 @@
         <v>30</v>
       </c>
       <c r="I68" s="11" t="n">
-        <v>0.833</v>
+        <v>0.8333</v>
       </c>
       <c r="J68" s="8" t="n">
         <v>15</v>
@@ -33630,7 +33630,7 @@
         <v>110</v>
       </c>
       <c r="I69" s="14" t="n">
-        <v>0.9537</v>
+        <v>0.9545</v>
       </c>
       <c r="J69" s="12" t="n">
         <v>55</v>
@@ -33771,7 +33771,7 @@
         <v>443</v>
       </c>
       <c r="I72" s="11" t="n">
-        <v>0.95</v>
+        <v>0.9503</v>
       </c>
       <c r="J72" s="8" t="n">
         <v>230</v>
@@ -33865,7 +33865,7 @@
         <v>63</v>
       </c>
       <c r="I74" s="11" t="n">
-        <v>0.9201</v>
+        <v>0.9206</v>
       </c>
       <c r="J74" s="8" t="n">
         <v>30</v>
@@ -33912,7 +33912,7 @@
         <v>528</v>
       </c>
       <c r="I75" s="14" t="n">
-        <v>0.8576</v>
+        <v>0.858</v>
       </c>
       <c r="J75" s="12" t="n">
         <v>265</v>
@@ -33959,7 +33959,7 @@
         <v>346</v>
       </c>
       <c r="I76" s="11" t="n">
-        <v>0.8321</v>
+        <v>0.8324</v>
       </c>
       <c r="J76" s="8" t="n">
         <v>170</v>
@@ -34006,7 +34006,7 @@
         <v>139</v>
       </c>
       <c r="I77" s="14" t="n">
-        <v>0.8484</v>
+        <v>0.8489</v>
       </c>
       <c r="J77" s="12" t="n">
         <v>70</v>
@@ -34141,7 +34141,7 @@
         <v>80</v>
       </c>
       <c r="I80" s="11" t="n">
-        <v>0.8373</v>
+        <v>0.8375</v>
       </c>
       <c r="J80" s="8" t="n">
         <v>38</v>
@@ -34188,7 +34188,7 @@
         <v>410</v>
       </c>
       <c r="I81" s="14" t="n">
-        <v>0.8754</v>
+        <v>0.8756</v>
       </c>
       <c r="J81" s="12" t="n">
         <v>200</v>
@@ -34235,7 +34235,7 @@
         <v>180</v>
       </c>
       <c r="I82" s="11" t="n">
-        <v>0.6166</v>
+        <v>0.6167</v>
       </c>
       <c r="J82" s="8" t="n">
         <v>85</v>
@@ -34282,7 +34282,7 @@
         <v>917</v>
       </c>
       <c r="I83" s="14" t="n">
-        <v>0.9167999999999999</v>
+        <v>0.9171</v>
       </c>
       <c r="J83" s="12" t="n">
         <v>225</v>
@@ -34329,7 +34329,7 @@
         <v>79</v>
       </c>
       <c r="I84" s="11" t="n">
-        <v>0.9743000000000001</v>
+        <v>0.9747</v>
       </c>
       <c r="J84" s="8" t="n">
         <v>20</v>
@@ -34364,7 +34364,7 @@
         <v>19</v>
       </c>
       <c r="E85" s="13" t="n">
-        <v>13.91</v>
+        <v>13.73</v>
       </c>
       <c r="F85" s="12" t="n">
         <v>7</v>
@@ -34373,10 +34373,10 @@
         <v>18</v>
       </c>
       <c r="H85" s="12" t="n">
-        <v>2179</v>
+        <v>2687</v>
       </c>
       <c r="I85" s="14" t="n">
-        <v>0.8998</v>
+        <v>0.8802</v>
       </c>
       <c r="J85" s="12" t="n">
         <v>684</v>

</xml_diff>